<commit_message>
Fix merit bill rate precision
</commit_message>
<xml_diff>
--- a/downloads/Merit_2026_Employee_Bulk_Calculator_350.xlsx
+++ b/downloads/Merit_2026_Employee_Bulk_Calculator_350.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employee Merit 2026" sheetId="1" r:id="R8f572a1d733f4b36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="2" r:id="Rc82762bea448476b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employee Merit 2026" sheetId="1" r:id="R305b4bf8d5c94fdc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="2" r:id="R88e72b2704da4800"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1026,10 +1026,10 @@
         <x:f>IF($L5="","",$C5*$L5)</x:f>
       </x:c>
       <x:c r="N5" s="85" t="str">
-        <x:f>IF($M5="","",$C5+$M5)</x:f>
+        <x:f>IF($M5="","",ROUNDDOWN($C5+$M5,2))</x:f>
       </x:c>
       <x:c r="O5" s="73" t="str">
-        <x:f>IF($N5="","",ROUNDDOWN($N5*$E5,3))</x:f>
+        <x:f>IF($N5="","",ROUNDDOWN(ROUNDDOWN($N5,2)*$E5,3))</x:f>
       </x:c>
       <x:c r="P5" s="76" t="str">
         <x:f>IF($L5="","",$I5*$L5)</x:f>
@@ -1079,10 +1079,10 @@
         <x:f>IF($L6="","",$C6*$L6)</x:f>
       </x:c>
       <x:c r="N6" s="86" t="str">
-        <x:f>IF($M6="","",$C6+$M6)</x:f>
+        <x:f>IF($M6="","",ROUNDDOWN($C6+$M6,2))</x:f>
       </x:c>
       <x:c r="O6" s="74" t="str">
-        <x:f>IF($N6="","",ROUNDDOWN($N6*$E6,3))</x:f>
+        <x:f>IF($N6="","",ROUNDDOWN(ROUNDDOWN($N6,2)*$E6,3))</x:f>
       </x:c>
       <x:c r="P6" s="77" t="str">
         <x:f>IF($L6="","",$I6*$L6)</x:f>
@@ -1132,10 +1132,10 @@
         <x:f>IF($L7="","",$C7*$L7)</x:f>
       </x:c>
       <x:c r="N7" s="86" t="str">
-        <x:f>IF($M7="","",$C7+$M7)</x:f>
+        <x:f>IF($M7="","",ROUNDDOWN($C7+$M7,2))</x:f>
       </x:c>
       <x:c r="O7" s="74" t="str">
-        <x:f>IF($N7="","",ROUNDDOWN($N7*$E7,3))</x:f>
+        <x:f>IF($N7="","",ROUNDDOWN(ROUNDDOWN($N7,2)*$E7,3))</x:f>
       </x:c>
       <x:c r="P7" s="77" t="str">
         <x:f>IF($L7="","",$I7*$L7)</x:f>
@@ -1185,10 +1185,10 @@
         <x:f>IF($L8="","",$C8*$L8)</x:f>
       </x:c>
       <x:c r="N8" s="86" t="str">
-        <x:f>IF($M8="","",$C8+$M8)</x:f>
+        <x:f>IF($M8="","",ROUNDDOWN($C8+$M8,2))</x:f>
       </x:c>
       <x:c r="O8" s="74" t="str">
-        <x:f>IF($N8="","",ROUNDDOWN($N8*$E8,3))</x:f>
+        <x:f>IF($N8="","",ROUNDDOWN(ROUNDDOWN($N8,2)*$E8,3))</x:f>
       </x:c>
       <x:c r="P8" s="77" t="str">
         <x:f>IF($L8="","",$I8*$L8)</x:f>
@@ -1238,10 +1238,10 @@
         <x:f>IF($L9="","",$C9*$L9)</x:f>
       </x:c>
       <x:c r="N9" s="86" t="str">
-        <x:f>IF($M9="","",$C9+$M9)</x:f>
+        <x:f>IF($M9="","",ROUNDDOWN($C9+$M9,2))</x:f>
       </x:c>
       <x:c r="O9" s="74" t="str">
-        <x:f>IF($N9="","",ROUNDDOWN($N9*$E9,3))</x:f>
+        <x:f>IF($N9="","",ROUNDDOWN(ROUNDDOWN($N9,2)*$E9,3))</x:f>
       </x:c>
       <x:c r="P9" s="77" t="str">
         <x:f>IF($L9="","",$I9*$L9)</x:f>
@@ -1291,10 +1291,10 @@
         <x:f>IF($L10="","",$C10*$L10)</x:f>
       </x:c>
       <x:c r="N10" s="86" t="str">
-        <x:f>IF($M10="","",$C10+$M10)</x:f>
+        <x:f>IF($M10="","",ROUNDDOWN($C10+$M10,2))</x:f>
       </x:c>
       <x:c r="O10" s="74" t="str">
-        <x:f>IF($N10="","",ROUNDDOWN($N10*$E10,3))</x:f>
+        <x:f>IF($N10="","",ROUNDDOWN(ROUNDDOWN($N10,2)*$E10,3))</x:f>
       </x:c>
       <x:c r="P10" s="77" t="str">
         <x:f>IF($L10="","",$I10*$L10)</x:f>
@@ -1344,10 +1344,10 @@
         <x:f>IF($L11="","",$C11*$L11)</x:f>
       </x:c>
       <x:c r="N11" s="86" t="str">
-        <x:f>IF($M11="","",$C11+$M11)</x:f>
+        <x:f>IF($M11="","",ROUNDDOWN($C11+$M11,2))</x:f>
       </x:c>
       <x:c r="O11" s="74" t="str">
-        <x:f>IF($N11="","",ROUNDDOWN($N11*$E11,3))</x:f>
+        <x:f>IF($N11="","",ROUNDDOWN(ROUNDDOWN($N11,2)*$E11,3))</x:f>
       </x:c>
       <x:c r="P11" s="77" t="str">
         <x:f>IF($L11="","",$I11*$L11)</x:f>
@@ -1397,10 +1397,10 @@
         <x:f>IF($L12="","",$C12*$L12)</x:f>
       </x:c>
       <x:c r="N12" s="86" t="str">
-        <x:f>IF($M12="","",$C12+$M12)</x:f>
+        <x:f>IF($M12="","",ROUNDDOWN($C12+$M12,2))</x:f>
       </x:c>
       <x:c r="O12" s="74" t="str">
-        <x:f>IF($N12="","",ROUNDDOWN($N12*$E12,3))</x:f>
+        <x:f>IF($N12="","",ROUNDDOWN(ROUNDDOWN($N12,2)*$E12,3))</x:f>
       </x:c>
       <x:c r="P12" s="77" t="str">
         <x:f>IF($L12="","",$I12*$L12)</x:f>
@@ -1450,10 +1450,10 @@
         <x:f>IF($L13="","",$C13*$L13)</x:f>
       </x:c>
       <x:c r="N13" s="86" t="str">
-        <x:f>IF($M13="","",$C13+$M13)</x:f>
+        <x:f>IF($M13="","",ROUNDDOWN($C13+$M13,2))</x:f>
       </x:c>
       <x:c r="O13" s="74" t="str">
-        <x:f>IF($N13="","",ROUNDDOWN($N13*$E13,3))</x:f>
+        <x:f>IF($N13="","",ROUNDDOWN(ROUNDDOWN($N13,2)*$E13,3))</x:f>
       </x:c>
       <x:c r="P13" s="77" t="str">
         <x:f>IF($L13="","",$I13*$L13)</x:f>
@@ -1503,10 +1503,10 @@
         <x:f>IF($L14="","",$C14*$L14)</x:f>
       </x:c>
       <x:c r="N14" s="86" t="str">
-        <x:f>IF($M14="","",$C14+$M14)</x:f>
+        <x:f>IF($M14="","",ROUNDDOWN($C14+$M14,2))</x:f>
       </x:c>
       <x:c r="O14" s="74" t="str">
-        <x:f>IF($N14="","",ROUNDDOWN($N14*$E14,3))</x:f>
+        <x:f>IF($N14="","",ROUNDDOWN(ROUNDDOWN($N14,2)*$E14,3))</x:f>
       </x:c>
       <x:c r="P14" s="77" t="str">
         <x:f>IF($L14="","",$I14*$L14)</x:f>
@@ -1556,10 +1556,10 @@
         <x:f>IF($L15="","",$C15*$L15)</x:f>
       </x:c>
       <x:c r="N15" s="86" t="str">
-        <x:f>IF($M15="","",$C15+$M15)</x:f>
+        <x:f>IF($M15="","",ROUNDDOWN($C15+$M15,2))</x:f>
       </x:c>
       <x:c r="O15" s="74" t="str">
-        <x:f>IF($N15="","",ROUNDDOWN($N15*$E15,3))</x:f>
+        <x:f>IF($N15="","",ROUNDDOWN(ROUNDDOWN($N15,2)*$E15,3))</x:f>
       </x:c>
       <x:c r="P15" s="77" t="str">
         <x:f>IF($L15="","",$I15*$L15)</x:f>
@@ -1609,10 +1609,10 @@
         <x:f>IF($L16="","",$C16*$L16)</x:f>
       </x:c>
       <x:c r="N16" s="86" t="str">
-        <x:f>IF($M16="","",$C16+$M16)</x:f>
+        <x:f>IF($M16="","",ROUNDDOWN($C16+$M16,2))</x:f>
       </x:c>
       <x:c r="O16" s="74" t="str">
-        <x:f>IF($N16="","",ROUNDDOWN($N16*$E16,3))</x:f>
+        <x:f>IF($N16="","",ROUNDDOWN(ROUNDDOWN($N16,2)*$E16,3))</x:f>
       </x:c>
       <x:c r="P16" s="77" t="str">
         <x:f>IF($L16="","",$I16*$L16)</x:f>
@@ -1662,10 +1662,10 @@
         <x:f>IF($L17="","",$C17*$L17)</x:f>
       </x:c>
       <x:c r="N17" s="86" t="str">
-        <x:f>IF($M17="","",$C17+$M17)</x:f>
+        <x:f>IF($M17="","",ROUNDDOWN($C17+$M17,2))</x:f>
       </x:c>
       <x:c r="O17" s="74" t="str">
-        <x:f>IF($N17="","",ROUNDDOWN($N17*$E17,3))</x:f>
+        <x:f>IF($N17="","",ROUNDDOWN(ROUNDDOWN($N17,2)*$E17,3))</x:f>
       </x:c>
       <x:c r="P17" s="77" t="str">
         <x:f>IF($L17="","",$I17*$L17)</x:f>
@@ -1715,10 +1715,10 @@
         <x:f>IF($L18="","",$C18*$L18)</x:f>
       </x:c>
       <x:c r="N18" s="86" t="str">
-        <x:f>IF($M18="","",$C18+$M18)</x:f>
+        <x:f>IF($M18="","",ROUNDDOWN($C18+$M18,2))</x:f>
       </x:c>
       <x:c r="O18" s="74" t="str">
-        <x:f>IF($N18="","",ROUNDDOWN($N18*$E18,3))</x:f>
+        <x:f>IF($N18="","",ROUNDDOWN(ROUNDDOWN($N18,2)*$E18,3))</x:f>
       </x:c>
       <x:c r="P18" s="77" t="str">
         <x:f>IF($L18="","",$I18*$L18)</x:f>
@@ -1768,10 +1768,10 @@
         <x:f>IF($L19="","",$C19*$L19)</x:f>
       </x:c>
       <x:c r="N19" s="86" t="str">
-        <x:f>IF($M19="","",$C19+$M19)</x:f>
+        <x:f>IF($M19="","",ROUNDDOWN($C19+$M19,2))</x:f>
       </x:c>
       <x:c r="O19" s="74" t="str">
-        <x:f>IF($N19="","",ROUNDDOWN($N19*$E19,3))</x:f>
+        <x:f>IF($N19="","",ROUNDDOWN(ROUNDDOWN($N19,2)*$E19,3))</x:f>
       </x:c>
       <x:c r="P19" s="77" t="str">
         <x:f>IF($L19="","",$I19*$L19)</x:f>
@@ -1821,10 +1821,10 @@
         <x:f>IF($L20="","",$C20*$L20)</x:f>
       </x:c>
       <x:c r="N20" s="86" t="str">
-        <x:f>IF($M20="","",$C20+$M20)</x:f>
+        <x:f>IF($M20="","",ROUNDDOWN($C20+$M20,2))</x:f>
       </x:c>
       <x:c r="O20" s="74" t="str">
-        <x:f>IF($N20="","",ROUNDDOWN($N20*$E20,3))</x:f>
+        <x:f>IF($N20="","",ROUNDDOWN(ROUNDDOWN($N20,2)*$E20,3))</x:f>
       </x:c>
       <x:c r="P20" s="77" t="str">
         <x:f>IF($L20="","",$I20*$L20)</x:f>
@@ -1874,10 +1874,10 @@
         <x:f>IF($L21="","",$C21*$L21)</x:f>
       </x:c>
       <x:c r="N21" s="86" t="str">
-        <x:f>IF($M21="","",$C21+$M21)</x:f>
+        <x:f>IF($M21="","",ROUNDDOWN($C21+$M21,2))</x:f>
       </x:c>
       <x:c r="O21" s="74" t="str">
-        <x:f>IF($N21="","",ROUNDDOWN($N21*$E21,3))</x:f>
+        <x:f>IF($N21="","",ROUNDDOWN(ROUNDDOWN($N21,2)*$E21,3))</x:f>
       </x:c>
       <x:c r="P21" s="77" t="str">
         <x:f>IF($L21="","",$I21*$L21)</x:f>
@@ -1927,10 +1927,10 @@
         <x:f>IF($L22="","",$C22*$L22)</x:f>
       </x:c>
       <x:c r="N22" s="86" t="str">
-        <x:f>IF($M22="","",$C22+$M22)</x:f>
+        <x:f>IF($M22="","",ROUNDDOWN($C22+$M22,2))</x:f>
       </x:c>
       <x:c r="O22" s="74" t="str">
-        <x:f>IF($N22="","",ROUNDDOWN($N22*$E22,3))</x:f>
+        <x:f>IF($N22="","",ROUNDDOWN(ROUNDDOWN($N22,2)*$E22,3))</x:f>
       </x:c>
       <x:c r="P22" s="77" t="str">
         <x:f>IF($L22="","",$I22*$L22)</x:f>
@@ -1980,10 +1980,10 @@
         <x:f>IF($L23="","",$C23*$L23)</x:f>
       </x:c>
       <x:c r="N23" s="86" t="str">
-        <x:f>IF($M23="","",$C23+$M23)</x:f>
+        <x:f>IF($M23="","",ROUNDDOWN($C23+$M23,2))</x:f>
       </x:c>
       <x:c r="O23" s="74" t="str">
-        <x:f>IF($N23="","",ROUNDDOWN($N23*$E23,3))</x:f>
+        <x:f>IF($N23="","",ROUNDDOWN(ROUNDDOWN($N23,2)*$E23,3))</x:f>
       </x:c>
       <x:c r="P23" s="77" t="str">
         <x:f>IF($L23="","",$I23*$L23)</x:f>
@@ -2033,10 +2033,10 @@
         <x:f>IF($L24="","",$C24*$L24)</x:f>
       </x:c>
       <x:c r="N24" s="86" t="str">
-        <x:f>IF($M24="","",$C24+$M24)</x:f>
+        <x:f>IF($M24="","",ROUNDDOWN($C24+$M24,2))</x:f>
       </x:c>
       <x:c r="O24" s="74" t="str">
-        <x:f>IF($N24="","",ROUNDDOWN($N24*$E24,3))</x:f>
+        <x:f>IF($N24="","",ROUNDDOWN(ROUNDDOWN($N24,2)*$E24,3))</x:f>
       </x:c>
       <x:c r="P24" s="77" t="str">
         <x:f>IF($L24="","",$I24*$L24)</x:f>
@@ -2086,10 +2086,10 @@
         <x:f>IF($L25="","",$C25*$L25)</x:f>
       </x:c>
       <x:c r="N25" s="86" t="str">
-        <x:f>IF($M25="","",$C25+$M25)</x:f>
+        <x:f>IF($M25="","",ROUNDDOWN($C25+$M25,2))</x:f>
       </x:c>
       <x:c r="O25" s="74" t="str">
-        <x:f>IF($N25="","",ROUNDDOWN($N25*$E25,3))</x:f>
+        <x:f>IF($N25="","",ROUNDDOWN(ROUNDDOWN($N25,2)*$E25,3))</x:f>
       </x:c>
       <x:c r="P25" s="77" t="str">
         <x:f>IF($L25="","",$I25*$L25)</x:f>
@@ -2139,10 +2139,10 @@
         <x:f>IF($L26="","",$C26*$L26)</x:f>
       </x:c>
       <x:c r="N26" s="86" t="str">
-        <x:f>IF($M26="","",$C26+$M26)</x:f>
+        <x:f>IF($M26="","",ROUNDDOWN($C26+$M26,2))</x:f>
       </x:c>
       <x:c r="O26" s="74" t="str">
-        <x:f>IF($N26="","",ROUNDDOWN($N26*$E26,3))</x:f>
+        <x:f>IF($N26="","",ROUNDDOWN(ROUNDDOWN($N26,2)*$E26,3))</x:f>
       </x:c>
       <x:c r="P26" s="77" t="str">
         <x:f>IF($L26="","",$I26*$L26)</x:f>
@@ -2192,10 +2192,10 @@
         <x:f>IF($L27="","",$C27*$L27)</x:f>
       </x:c>
       <x:c r="N27" s="86" t="str">
-        <x:f>IF($M27="","",$C27+$M27)</x:f>
+        <x:f>IF($M27="","",ROUNDDOWN($C27+$M27,2))</x:f>
       </x:c>
       <x:c r="O27" s="74" t="str">
-        <x:f>IF($N27="","",ROUNDDOWN($N27*$E27,3))</x:f>
+        <x:f>IF($N27="","",ROUNDDOWN(ROUNDDOWN($N27,2)*$E27,3))</x:f>
       </x:c>
       <x:c r="P27" s="77" t="str">
         <x:f>IF($L27="","",$I27*$L27)</x:f>
@@ -2245,10 +2245,10 @@
         <x:f>IF($L28="","",$C28*$L28)</x:f>
       </x:c>
       <x:c r="N28" s="86" t="str">
-        <x:f>IF($M28="","",$C28+$M28)</x:f>
+        <x:f>IF($M28="","",ROUNDDOWN($C28+$M28,2))</x:f>
       </x:c>
       <x:c r="O28" s="74" t="str">
-        <x:f>IF($N28="","",ROUNDDOWN($N28*$E28,3))</x:f>
+        <x:f>IF($N28="","",ROUNDDOWN(ROUNDDOWN($N28,2)*$E28,3))</x:f>
       </x:c>
       <x:c r="P28" s="77" t="str">
         <x:f>IF($L28="","",$I28*$L28)</x:f>
@@ -2298,10 +2298,10 @@
         <x:f>IF($L29="","",$C29*$L29)</x:f>
       </x:c>
       <x:c r="N29" s="86" t="str">
-        <x:f>IF($M29="","",$C29+$M29)</x:f>
+        <x:f>IF($M29="","",ROUNDDOWN($C29+$M29,2))</x:f>
       </x:c>
       <x:c r="O29" s="74" t="str">
-        <x:f>IF($N29="","",ROUNDDOWN($N29*$E29,3))</x:f>
+        <x:f>IF($N29="","",ROUNDDOWN(ROUNDDOWN($N29,2)*$E29,3))</x:f>
       </x:c>
       <x:c r="P29" s="77" t="str">
         <x:f>IF($L29="","",$I29*$L29)</x:f>
@@ -2351,10 +2351,10 @@
         <x:f>IF($L30="","",$C30*$L30)</x:f>
       </x:c>
       <x:c r="N30" s="86" t="str">
-        <x:f>IF($M30="","",$C30+$M30)</x:f>
+        <x:f>IF($M30="","",ROUNDDOWN($C30+$M30,2))</x:f>
       </x:c>
       <x:c r="O30" s="74" t="str">
-        <x:f>IF($N30="","",ROUNDDOWN($N30*$E30,3))</x:f>
+        <x:f>IF($N30="","",ROUNDDOWN(ROUNDDOWN($N30,2)*$E30,3))</x:f>
       </x:c>
       <x:c r="P30" s="77" t="str">
         <x:f>IF($L30="","",$I30*$L30)</x:f>
@@ -2404,10 +2404,10 @@
         <x:f>IF($L31="","",$C31*$L31)</x:f>
       </x:c>
       <x:c r="N31" s="86" t="str">
-        <x:f>IF($M31="","",$C31+$M31)</x:f>
+        <x:f>IF($M31="","",ROUNDDOWN($C31+$M31,2))</x:f>
       </x:c>
       <x:c r="O31" s="74" t="str">
-        <x:f>IF($N31="","",ROUNDDOWN($N31*$E31,3))</x:f>
+        <x:f>IF($N31="","",ROUNDDOWN(ROUNDDOWN($N31,2)*$E31,3))</x:f>
       </x:c>
       <x:c r="P31" s="77" t="str">
         <x:f>IF($L31="","",$I31*$L31)</x:f>
@@ -2457,10 +2457,10 @@
         <x:f>IF($L32="","",$C32*$L32)</x:f>
       </x:c>
       <x:c r="N32" s="86" t="str">
-        <x:f>IF($M32="","",$C32+$M32)</x:f>
+        <x:f>IF($M32="","",ROUNDDOWN($C32+$M32,2))</x:f>
       </x:c>
       <x:c r="O32" s="74" t="str">
-        <x:f>IF($N32="","",ROUNDDOWN($N32*$E32,3))</x:f>
+        <x:f>IF($N32="","",ROUNDDOWN(ROUNDDOWN($N32,2)*$E32,3))</x:f>
       </x:c>
       <x:c r="P32" s="77" t="str">
         <x:f>IF($L32="","",$I32*$L32)</x:f>
@@ -2510,10 +2510,10 @@
         <x:f>IF($L33="","",$C33*$L33)</x:f>
       </x:c>
       <x:c r="N33" s="86" t="str">
-        <x:f>IF($M33="","",$C33+$M33)</x:f>
+        <x:f>IF($M33="","",ROUNDDOWN($C33+$M33,2))</x:f>
       </x:c>
       <x:c r="O33" s="74" t="str">
-        <x:f>IF($N33="","",ROUNDDOWN($N33*$E33,3))</x:f>
+        <x:f>IF($N33="","",ROUNDDOWN(ROUNDDOWN($N33,2)*$E33,3))</x:f>
       </x:c>
       <x:c r="P33" s="77" t="str">
         <x:f>IF($L33="","",$I33*$L33)</x:f>
@@ -2563,10 +2563,10 @@
         <x:f>IF($L34="","",$C34*$L34)</x:f>
       </x:c>
       <x:c r="N34" s="86" t="str">
-        <x:f>IF($M34="","",$C34+$M34)</x:f>
+        <x:f>IF($M34="","",ROUNDDOWN($C34+$M34,2))</x:f>
       </x:c>
       <x:c r="O34" s="74" t="str">
-        <x:f>IF($N34="","",ROUNDDOWN($N34*$E34,3))</x:f>
+        <x:f>IF($N34="","",ROUNDDOWN(ROUNDDOWN($N34,2)*$E34,3))</x:f>
       </x:c>
       <x:c r="P34" s="77" t="str">
         <x:f>IF($L34="","",$I34*$L34)</x:f>
@@ -2616,10 +2616,10 @@
         <x:f>IF($L35="","",$C35*$L35)</x:f>
       </x:c>
       <x:c r="N35" s="86" t="str">
-        <x:f>IF($M35="","",$C35+$M35)</x:f>
+        <x:f>IF($M35="","",ROUNDDOWN($C35+$M35,2))</x:f>
       </x:c>
       <x:c r="O35" s="74" t="str">
-        <x:f>IF($N35="","",ROUNDDOWN($N35*$E35,3))</x:f>
+        <x:f>IF($N35="","",ROUNDDOWN(ROUNDDOWN($N35,2)*$E35,3))</x:f>
       </x:c>
       <x:c r="P35" s="77" t="str">
         <x:f>IF($L35="","",$I35*$L35)</x:f>
@@ -2669,10 +2669,10 @@
         <x:f>IF($L36="","",$C36*$L36)</x:f>
       </x:c>
       <x:c r="N36" s="86" t="str">
-        <x:f>IF($M36="","",$C36+$M36)</x:f>
+        <x:f>IF($M36="","",ROUNDDOWN($C36+$M36,2))</x:f>
       </x:c>
       <x:c r="O36" s="74" t="str">
-        <x:f>IF($N36="","",ROUNDDOWN($N36*$E36,3))</x:f>
+        <x:f>IF($N36="","",ROUNDDOWN(ROUNDDOWN($N36,2)*$E36,3))</x:f>
       </x:c>
       <x:c r="P36" s="77" t="str">
         <x:f>IF($L36="","",$I36*$L36)</x:f>
@@ -2722,10 +2722,10 @@
         <x:f>IF($L37="","",$C37*$L37)</x:f>
       </x:c>
       <x:c r="N37" s="86" t="str">
-        <x:f>IF($M37="","",$C37+$M37)</x:f>
+        <x:f>IF($M37="","",ROUNDDOWN($C37+$M37,2))</x:f>
       </x:c>
       <x:c r="O37" s="74" t="str">
-        <x:f>IF($N37="","",ROUNDDOWN($N37*$E37,3))</x:f>
+        <x:f>IF($N37="","",ROUNDDOWN(ROUNDDOWN($N37,2)*$E37,3))</x:f>
       </x:c>
       <x:c r="P37" s="77" t="str">
         <x:f>IF($L37="","",$I37*$L37)</x:f>
@@ -2775,10 +2775,10 @@
         <x:f>IF($L38="","",$C38*$L38)</x:f>
       </x:c>
       <x:c r="N38" s="86" t="str">
-        <x:f>IF($M38="","",$C38+$M38)</x:f>
+        <x:f>IF($M38="","",ROUNDDOWN($C38+$M38,2))</x:f>
       </x:c>
       <x:c r="O38" s="74" t="str">
-        <x:f>IF($N38="","",ROUNDDOWN($N38*$E38,3))</x:f>
+        <x:f>IF($N38="","",ROUNDDOWN(ROUNDDOWN($N38,2)*$E38,3))</x:f>
       </x:c>
       <x:c r="P38" s="77" t="str">
         <x:f>IF($L38="","",$I38*$L38)</x:f>
@@ -2828,10 +2828,10 @@
         <x:f>IF($L39="","",$C39*$L39)</x:f>
       </x:c>
       <x:c r="N39" s="86" t="str">
-        <x:f>IF($M39="","",$C39+$M39)</x:f>
+        <x:f>IF($M39="","",ROUNDDOWN($C39+$M39,2))</x:f>
       </x:c>
       <x:c r="O39" s="74" t="str">
-        <x:f>IF($N39="","",ROUNDDOWN($N39*$E39,3))</x:f>
+        <x:f>IF($N39="","",ROUNDDOWN(ROUNDDOWN($N39,2)*$E39,3))</x:f>
       </x:c>
       <x:c r="P39" s="77" t="str">
         <x:f>IF($L39="","",$I39*$L39)</x:f>
@@ -2881,10 +2881,10 @@
         <x:f>IF($L40="","",$C40*$L40)</x:f>
       </x:c>
       <x:c r="N40" s="86" t="str">
-        <x:f>IF($M40="","",$C40+$M40)</x:f>
+        <x:f>IF($M40="","",ROUNDDOWN($C40+$M40,2))</x:f>
       </x:c>
       <x:c r="O40" s="74" t="str">
-        <x:f>IF($N40="","",ROUNDDOWN($N40*$E40,3))</x:f>
+        <x:f>IF($N40="","",ROUNDDOWN(ROUNDDOWN($N40,2)*$E40,3))</x:f>
       </x:c>
       <x:c r="P40" s="77" t="str">
         <x:f>IF($L40="","",$I40*$L40)</x:f>
@@ -2934,10 +2934,10 @@
         <x:f>IF($L41="","",$C41*$L41)</x:f>
       </x:c>
       <x:c r="N41" s="86" t="str">
-        <x:f>IF($M41="","",$C41+$M41)</x:f>
+        <x:f>IF($M41="","",ROUNDDOWN($C41+$M41,2))</x:f>
       </x:c>
       <x:c r="O41" s="74" t="str">
-        <x:f>IF($N41="","",ROUNDDOWN($N41*$E41,3))</x:f>
+        <x:f>IF($N41="","",ROUNDDOWN(ROUNDDOWN($N41,2)*$E41,3))</x:f>
       </x:c>
       <x:c r="P41" s="77" t="str">
         <x:f>IF($L41="","",$I41*$L41)</x:f>
@@ -2987,10 +2987,10 @@
         <x:f>IF($L42="","",$C42*$L42)</x:f>
       </x:c>
       <x:c r="N42" s="86" t="str">
-        <x:f>IF($M42="","",$C42+$M42)</x:f>
+        <x:f>IF($M42="","",ROUNDDOWN($C42+$M42,2))</x:f>
       </x:c>
       <x:c r="O42" s="74" t="str">
-        <x:f>IF($N42="","",ROUNDDOWN($N42*$E42,3))</x:f>
+        <x:f>IF($N42="","",ROUNDDOWN(ROUNDDOWN($N42,2)*$E42,3))</x:f>
       </x:c>
       <x:c r="P42" s="77" t="str">
         <x:f>IF($L42="","",$I42*$L42)</x:f>
@@ -3040,10 +3040,10 @@
         <x:f>IF($L43="","",$C43*$L43)</x:f>
       </x:c>
       <x:c r="N43" s="86" t="str">
-        <x:f>IF($M43="","",$C43+$M43)</x:f>
+        <x:f>IF($M43="","",ROUNDDOWN($C43+$M43,2))</x:f>
       </x:c>
       <x:c r="O43" s="74" t="str">
-        <x:f>IF($N43="","",ROUNDDOWN($N43*$E43,3))</x:f>
+        <x:f>IF($N43="","",ROUNDDOWN(ROUNDDOWN($N43,2)*$E43,3))</x:f>
       </x:c>
       <x:c r="P43" s="77" t="str">
         <x:f>IF($L43="","",$I43*$L43)</x:f>
@@ -3093,10 +3093,10 @@
         <x:f>IF($L44="","",$C44*$L44)</x:f>
       </x:c>
       <x:c r="N44" s="86" t="str">
-        <x:f>IF($M44="","",$C44+$M44)</x:f>
+        <x:f>IF($M44="","",ROUNDDOWN($C44+$M44,2))</x:f>
       </x:c>
       <x:c r="O44" s="74" t="str">
-        <x:f>IF($N44="","",ROUNDDOWN($N44*$E44,3))</x:f>
+        <x:f>IF($N44="","",ROUNDDOWN(ROUNDDOWN($N44,2)*$E44,3))</x:f>
       </x:c>
       <x:c r="P44" s="77" t="str">
         <x:f>IF($L44="","",$I44*$L44)</x:f>
@@ -3146,10 +3146,10 @@
         <x:f>IF($L45="","",$C45*$L45)</x:f>
       </x:c>
       <x:c r="N45" s="86" t="str">
-        <x:f>IF($M45="","",$C45+$M45)</x:f>
+        <x:f>IF($M45="","",ROUNDDOWN($C45+$M45,2))</x:f>
       </x:c>
       <x:c r="O45" s="74" t="str">
-        <x:f>IF($N45="","",ROUNDDOWN($N45*$E45,3))</x:f>
+        <x:f>IF($N45="","",ROUNDDOWN(ROUNDDOWN($N45,2)*$E45,3))</x:f>
       </x:c>
       <x:c r="P45" s="77" t="str">
         <x:f>IF($L45="","",$I45*$L45)</x:f>
@@ -3199,10 +3199,10 @@
         <x:f>IF($L46="","",$C46*$L46)</x:f>
       </x:c>
       <x:c r="N46" s="86" t="str">
-        <x:f>IF($M46="","",$C46+$M46)</x:f>
+        <x:f>IF($M46="","",ROUNDDOWN($C46+$M46,2))</x:f>
       </x:c>
       <x:c r="O46" s="74" t="str">
-        <x:f>IF($N46="","",ROUNDDOWN($N46*$E46,3))</x:f>
+        <x:f>IF($N46="","",ROUNDDOWN(ROUNDDOWN($N46,2)*$E46,3))</x:f>
       </x:c>
       <x:c r="P46" s="77" t="str">
         <x:f>IF($L46="","",$I46*$L46)</x:f>
@@ -3252,10 +3252,10 @@
         <x:f>IF($L47="","",$C47*$L47)</x:f>
       </x:c>
       <x:c r="N47" s="86" t="str">
-        <x:f>IF($M47="","",$C47+$M47)</x:f>
+        <x:f>IF($M47="","",ROUNDDOWN($C47+$M47,2))</x:f>
       </x:c>
       <x:c r="O47" s="74" t="str">
-        <x:f>IF($N47="","",ROUNDDOWN($N47*$E47,3))</x:f>
+        <x:f>IF($N47="","",ROUNDDOWN(ROUNDDOWN($N47,2)*$E47,3))</x:f>
       </x:c>
       <x:c r="P47" s="77" t="str">
         <x:f>IF($L47="","",$I47*$L47)</x:f>
@@ -3305,10 +3305,10 @@
         <x:f>IF($L48="","",$C48*$L48)</x:f>
       </x:c>
       <x:c r="N48" s="86" t="str">
-        <x:f>IF($M48="","",$C48+$M48)</x:f>
+        <x:f>IF($M48="","",ROUNDDOWN($C48+$M48,2))</x:f>
       </x:c>
       <x:c r="O48" s="74" t="str">
-        <x:f>IF($N48="","",ROUNDDOWN($N48*$E48,3))</x:f>
+        <x:f>IF($N48="","",ROUNDDOWN(ROUNDDOWN($N48,2)*$E48,3))</x:f>
       </x:c>
       <x:c r="P48" s="77" t="str">
         <x:f>IF($L48="","",$I48*$L48)</x:f>
@@ -3358,10 +3358,10 @@
         <x:f>IF($L49="","",$C49*$L49)</x:f>
       </x:c>
       <x:c r="N49" s="86" t="str">
-        <x:f>IF($M49="","",$C49+$M49)</x:f>
+        <x:f>IF($M49="","",ROUNDDOWN($C49+$M49,2))</x:f>
       </x:c>
       <x:c r="O49" s="74" t="str">
-        <x:f>IF($N49="","",ROUNDDOWN($N49*$E49,3))</x:f>
+        <x:f>IF($N49="","",ROUNDDOWN(ROUNDDOWN($N49,2)*$E49,3))</x:f>
       </x:c>
       <x:c r="P49" s="77" t="str">
         <x:f>IF($L49="","",$I49*$L49)</x:f>
@@ -3411,10 +3411,10 @@
         <x:f>IF($L50="","",$C50*$L50)</x:f>
       </x:c>
       <x:c r="N50" s="86" t="str">
-        <x:f>IF($M50="","",$C50+$M50)</x:f>
+        <x:f>IF($M50="","",ROUNDDOWN($C50+$M50,2))</x:f>
       </x:c>
       <x:c r="O50" s="74" t="str">
-        <x:f>IF($N50="","",ROUNDDOWN($N50*$E50,3))</x:f>
+        <x:f>IF($N50="","",ROUNDDOWN(ROUNDDOWN($N50,2)*$E50,3))</x:f>
       </x:c>
       <x:c r="P50" s="77" t="str">
         <x:f>IF($L50="","",$I50*$L50)</x:f>
@@ -3464,10 +3464,10 @@
         <x:f>IF($L51="","",$C51*$L51)</x:f>
       </x:c>
       <x:c r="N51" s="86" t="str">
-        <x:f>IF($M51="","",$C51+$M51)</x:f>
+        <x:f>IF($M51="","",ROUNDDOWN($C51+$M51,2))</x:f>
       </x:c>
       <x:c r="O51" s="74" t="str">
-        <x:f>IF($N51="","",ROUNDDOWN($N51*$E51,3))</x:f>
+        <x:f>IF($N51="","",ROUNDDOWN(ROUNDDOWN($N51,2)*$E51,3))</x:f>
       </x:c>
       <x:c r="P51" s="77" t="str">
         <x:f>IF($L51="","",$I51*$L51)</x:f>
@@ -3517,10 +3517,10 @@
         <x:f>IF($L52="","",$C52*$L52)</x:f>
       </x:c>
       <x:c r="N52" s="86" t="str">
-        <x:f>IF($M52="","",$C52+$M52)</x:f>
+        <x:f>IF($M52="","",ROUNDDOWN($C52+$M52,2))</x:f>
       </x:c>
       <x:c r="O52" s="74" t="str">
-        <x:f>IF($N52="","",ROUNDDOWN($N52*$E52,3))</x:f>
+        <x:f>IF($N52="","",ROUNDDOWN(ROUNDDOWN($N52,2)*$E52,3))</x:f>
       </x:c>
       <x:c r="P52" s="77" t="str">
         <x:f>IF($L52="","",$I52*$L52)</x:f>
@@ -3570,10 +3570,10 @@
         <x:f>IF($L53="","",$C53*$L53)</x:f>
       </x:c>
       <x:c r="N53" s="86" t="str">
-        <x:f>IF($M53="","",$C53+$M53)</x:f>
+        <x:f>IF($M53="","",ROUNDDOWN($C53+$M53,2))</x:f>
       </x:c>
       <x:c r="O53" s="74" t="str">
-        <x:f>IF($N53="","",ROUNDDOWN($N53*$E53,3))</x:f>
+        <x:f>IF($N53="","",ROUNDDOWN(ROUNDDOWN($N53,2)*$E53,3))</x:f>
       </x:c>
       <x:c r="P53" s="77" t="str">
         <x:f>IF($L53="","",$I53*$L53)</x:f>
@@ -3623,10 +3623,10 @@
         <x:f>IF($L54="","",$C54*$L54)</x:f>
       </x:c>
       <x:c r="N54" s="86" t="str">
-        <x:f>IF($M54="","",$C54+$M54)</x:f>
+        <x:f>IF($M54="","",ROUNDDOWN($C54+$M54,2))</x:f>
       </x:c>
       <x:c r="O54" s="74" t="str">
-        <x:f>IF($N54="","",ROUNDDOWN($N54*$E54,3))</x:f>
+        <x:f>IF($N54="","",ROUNDDOWN(ROUNDDOWN($N54,2)*$E54,3))</x:f>
       </x:c>
       <x:c r="P54" s="77" t="str">
         <x:f>IF($L54="","",$I54*$L54)</x:f>
@@ -3676,10 +3676,10 @@
         <x:f>IF($L55="","",$C55*$L55)</x:f>
       </x:c>
       <x:c r="N55" s="86" t="str">
-        <x:f>IF($M55="","",$C55+$M55)</x:f>
+        <x:f>IF($M55="","",ROUNDDOWN($C55+$M55,2))</x:f>
       </x:c>
       <x:c r="O55" s="74" t="str">
-        <x:f>IF($N55="","",ROUNDDOWN($N55*$E55,3))</x:f>
+        <x:f>IF($N55="","",ROUNDDOWN(ROUNDDOWN($N55,2)*$E55,3))</x:f>
       </x:c>
       <x:c r="P55" s="77" t="str">
         <x:f>IF($L55="","",$I55*$L55)</x:f>
@@ -3729,10 +3729,10 @@
         <x:f>IF($L56="","",$C56*$L56)</x:f>
       </x:c>
       <x:c r="N56" s="86" t="str">
-        <x:f>IF($M56="","",$C56+$M56)</x:f>
+        <x:f>IF($M56="","",ROUNDDOWN($C56+$M56,2))</x:f>
       </x:c>
       <x:c r="O56" s="74" t="str">
-        <x:f>IF($N56="","",ROUNDDOWN($N56*$E56,3))</x:f>
+        <x:f>IF($N56="","",ROUNDDOWN(ROUNDDOWN($N56,2)*$E56,3))</x:f>
       </x:c>
       <x:c r="P56" s="77" t="str">
         <x:f>IF($L56="","",$I56*$L56)</x:f>
@@ -3782,10 +3782,10 @@
         <x:f>IF($L57="","",$C57*$L57)</x:f>
       </x:c>
       <x:c r="N57" s="86" t="str">
-        <x:f>IF($M57="","",$C57+$M57)</x:f>
+        <x:f>IF($M57="","",ROUNDDOWN($C57+$M57,2))</x:f>
       </x:c>
       <x:c r="O57" s="74" t="str">
-        <x:f>IF($N57="","",ROUNDDOWN($N57*$E57,3))</x:f>
+        <x:f>IF($N57="","",ROUNDDOWN(ROUNDDOWN($N57,2)*$E57,3))</x:f>
       </x:c>
       <x:c r="P57" s="77" t="str">
         <x:f>IF($L57="","",$I57*$L57)</x:f>
@@ -3835,10 +3835,10 @@
         <x:f>IF($L58="","",$C58*$L58)</x:f>
       </x:c>
       <x:c r="N58" s="86" t="str">
-        <x:f>IF($M58="","",$C58+$M58)</x:f>
+        <x:f>IF($M58="","",ROUNDDOWN($C58+$M58,2))</x:f>
       </x:c>
       <x:c r="O58" s="74" t="str">
-        <x:f>IF($N58="","",ROUNDDOWN($N58*$E58,3))</x:f>
+        <x:f>IF($N58="","",ROUNDDOWN(ROUNDDOWN($N58,2)*$E58,3))</x:f>
       </x:c>
       <x:c r="P58" s="77" t="str">
         <x:f>IF($L58="","",$I58*$L58)</x:f>
@@ -3888,10 +3888,10 @@
         <x:f>IF($L59="","",$C59*$L59)</x:f>
       </x:c>
       <x:c r="N59" s="86" t="str">
-        <x:f>IF($M59="","",$C59+$M59)</x:f>
+        <x:f>IF($M59="","",ROUNDDOWN($C59+$M59,2))</x:f>
       </x:c>
       <x:c r="O59" s="74" t="str">
-        <x:f>IF($N59="","",ROUNDDOWN($N59*$E59,3))</x:f>
+        <x:f>IF($N59="","",ROUNDDOWN(ROUNDDOWN($N59,2)*$E59,3))</x:f>
       </x:c>
       <x:c r="P59" s="77" t="str">
         <x:f>IF($L59="","",$I59*$L59)</x:f>
@@ -3941,10 +3941,10 @@
         <x:f>IF($L60="","",$C60*$L60)</x:f>
       </x:c>
       <x:c r="N60" s="86" t="str">
-        <x:f>IF($M60="","",$C60+$M60)</x:f>
+        <x:f>IF($M60="","",ROUNDDOWN($C60+$M60,2))</x:f>
       </x:c>
       <x:c r="O60" s="74" t="str">
-        <x:f>IF($N60="","",ROUNDDOWN($N60*$E60,3))</x:f>
+        <x:f>IF($N60="","",ROUNDDOWN(ROUNDDOWN($N60,2)*$E60,3))</x:f>
       </x:c>
       <x:c r="P60" s="77" t="str">
         <x:f>IF($L60="","",$I60*$L60)</x:f>
@@ -3994,10 +3994,10 @@
         <x:f>IF($L61="","",$C61*$L61)</x:f>
       </x:c>
       <x:c r="N61" s="86" t="str">
-        <x:f>IF($M61="","",$C61+$M61)</x:f>
+        <x:f>IF($M61="","",ROUNDDOWN($C61+$M61,2))</x:f>
       </x:c>
       <x:c r="O61" s="74" t="str">
-        <x:f>IF($N61="","",ROUNDDOWN($N61*$E61,3))</x:f>
+        <x:f>IF($N61="","",ROUNDDOWN(ROUNDDOWN($N61,2)*$E61,3))</x:f>
       </x:c>
       <x:c r="P61" s="77" t="str">
         <x:f>IF($L61="","",$I61*$L61)</x:f>
@@ -4047,10 +4047,10 @@
         <x:f>IF($L62="","",$C62*$L62)</x:f>
       </x:c>
       <x:c r="N62" s="86" t="str">
-        <x:f>IF($M62="","",$C62+$M62)</x:f>
+        <x:f>IF($M62="","",ROUNDDOWN($C62+$M62,2))</x:f>
       </x:c>
       <x:c r="O62" s="74" t="str">
-        <x:f>IF($N62="","",ROUNDDOWN($N62*$E62,3))</x:f>
+        <x:f>IF($N62="","",ROUNDDOWN(ROUNDDOWN($N62,2)*$E62,3))</x:f>
       </x:c>
       <x:c r="P62" s="77" t="str">
         <x:f>IF($L62="","",$I62*$L62)</x:f>
@@ -4100,10 +4100,10 @@
         <x:f>IF($L63="","",$C63*$L63)</x:f>
       </x:c>
       <x:c r="N63" s="86" t="str">
-        <x:f>IF($M63="","",$C63+$M63)</x:f>
+        <x:f>IF($M63="","",ROUNDDOWN($C63+$M63,2))</x:f>
       </x:c>
       <x:c r="O63" s="74" t="str">
-        <x:f>IF($N63="","",ROUNDDOWN($N63*$E63,3))</x:f>
+        <x:f>IF($N63="","",ROUNDDOWN(ROUNDDOWN($N63,2)*$E63,3))</x:f>
       </x:c>
       <x:c r="P63" s="77" t="str">
         <x:f>IF($L63="","",$I63*$L63)</x:f>
@@ -4153,10 +4153,10 @@
         <x:f>IF($L64="","",$C64*$L64)</x:f>
       </x:c>
       <x:c r="N64" s="86" t="str">
-        <x:f>IF($M64="","",$C64+$M64)</x:f>
+        <x:f>IF($M64="","",ROUNDDOWN($C64+$M64,2))</x:f>
       </x:c>
       <x:c r="O64" s="74" t="str">
-        <x:f>IF($N64="","",ROUNDDOWN($N64*$E64,3))</x:f>
+        <x:f>IF($N64="","",ROUNDDOWN(ROUNDDOWN($N64,2)*$E64,3))</x:f>
       </x:c>
       <x:c r="P64" s="77" t="str">
         <x:f>IF($L64="","",$I64*$L64)</x:f>
@@ -4206,10 +4206,10 @@
         <x:f>IF($L65="","",$C65*$L65)</x:f>
       </x:c>
       <x:c r="N65" s="86" t="str">
-        <x:f>IF($M65="","",$C65+$M65)</x:f>
+        <x:f>IF($M65="","",ROUNDDOWN($C65+$M65,2))</x:f>
       </x:c>
       <x:c r="O65" s="74" t="str">
-        <x:f>IF($N65="","",ROUNDDOWN($N65*$E65,3))</x:f>
+        <x:f>IF($N65="","",ROUNDDOWN(ROUNDDOWN($N65,2)*$E65,3))</x:f>
       </x:c>
       <x:c r="P65" s="77" t="str">
         <x:f>IF($L65="","",$I65*$L65)</x:f>
@@ -4259,10 +4259,10 @@
         <x:f>IF($L66="","",$C66*$L66)</x:f>
       </x:c>
       <x:c r="N66" s="86" t="str">
-        <x:f>IF($M66="","",$C66+$M66)</x:f>
+        <x:f>IF($M66="","",ROUNDDOWN($C66+$M66,2))</x:f>
       </x:c>
       <x:c r="O66" s="74" t="str">
-        <x:f>IF($N66="","",ROUNDDOWN($N66*$E66,3))</x:f>
+        <x:f>IF($N66="","",ROUNDDOWN(ROUNDDOWN($N66,2)*$E66,3))</x:f>
       </x:c>
       <x:c r="P66" s="77" t="str">
         <x:f>IF($L66="","",$I66*$L66)</x:f>
@@ -4312,10 +4312,10 @@
         <x:f>IF($L67="","",$C67*$L67)</x:f>
       </x:c>
       <x:c r="N67" s="86" t="str">
-        <x:f>IF($M67="","",$C67+$M67)</x:f>
+        <x:f>IF($M67="","",ROUNDDOWN($C67+$M67,2))</x:f>
       </x:c>
       <x:c r="O67" s="74" t="str">
-        <x:f>IF($N67="","",ROUNDDOWN($N67*$E67,3))</x:f>
+        <x:f>IF($N67="","",ROUNDDOWN(ROUNDDOWN($N67,2)*$E67,3))</x:f>
       </x:c>
       <x:c r="P67" s="77" t="str">
         <x:f>IF($L67="","",$I67*$L67)</x:f>
@@ -4365,10 +4365,10 @@
         <x:f>IF($L68="","",$C68*$L68)</x:f>
       </x:c>
       <x:c r="N68" s="86" t="str">
-        <x:f>IF($M68="","",$C68+$M68)</x:f>
+        <x:f>IF($M68="","",ROUNDDOWN($C68+$M68,2))</x:f>
       </x:c>
       <x:c r="O68" s="74" t="str">
-        <x:f>IF($N68="","",ROUNDDOWN($N68*$E68,3))</x:f>
+        <x:f>IF($N68="","",ROUNDDOWN(ROUNDDOWN($N68,2)*$E68,3))</x:f>
       </x:c>
       <x:c r="P68" s="77" t="str">
         <x:f>IF($L68="","",$I68*$L68)</x:f>
@@ -4418,10 +4418,10 @@
         <x:f>IF($L69="","",$C69*$L69)</x:f>
       </x:c>
       <x:c r="N69" s="86" t="str">
-        <x:f>IF($M69="","",$C69+$M69)</x:f>
+        <x:f>IF($M69="","",ROUNDDOWN($C69+$M69,2))</x:f>
       </x:c>
       <x:c r="O69" s="74" t="str">
-        <x:f>IF($N69="","",ROUNDDOWN($N69*$E69,3))</x:f>
+        <x:f>IF($N69="","",ROUNDDOWN(ROUNDDOWN($N69,2)*$E69,3))</x:f>
       </x:c>
       <x:c r="P69" s="77" t="str">
         <x:f>IF($L69="","",$I69*$L69)</x:f>
@@ -4471,10 +4471,10 @@
         <x:f>IF($L70="","",$C70*$L70)</x:f>
       </x:c>
       <x:c r="N70" s="86" t="str">
-        <x:f>IF($M70="","",$C70+$M70)</x:f>
+        <x:f>IF($M70="","",ROUNDDOWN($C70+$M70,2))</x:f>
       </x:c>
       <x:c r="O70" s="74" t="str">
-        <x:f>IF($N70="","",ROUNDDOWN($N70*$E70,3))</x:f>
+        <x:f>IF($N70="","",ROUNDDOWN(ROUNDDOWN($N70,2)*$E70,3))</x:f>
       </x:c>
       <x:c r="P70" s="77" t="str">
         <x:f>IF($L70="","",$I70*$L70)</x:f>
@@ -4524,10 +4524,10 @@
         <x:f>IF($L71="","",$C71*$L71)</x:f>
       </x:c>
       <x:c r="N71" s="86" t="str">
-        <x:f>IF($M71="","",$C71+$M71)</x:f>
+        <x:f>IF($M71="","",ROUNDDOWN($C71+$M71,2))</x:f>
       </x:c>
       <x:c r="O71" s="74" t="str">
-        <x:f>IF($N71="","",ROUNDDOWN($N71*$E71,3))</x:f>
+        <x:f>IF($N71="","",ROUNDDOWN(ROUNDDOWN($N71,2)*$E71,3))</x:f>
       </x:c>
       <x:c r="P71" s="77" t="str">
         <x:f>IF($L71="","",$I71*$L71)</x:f>
@@ -4577,10 +4577,10 @@
         <x:f>IF($L72="","",$C72*$L72)</x:f>
       </x:c>
       <x:c r="N72" s="86" t="str">
-        <x:f>IF($M72="","",$C72+$M72)</x:f>
+        <x:f>IF($M72="","",ROUNDDOWN($C72+$M72,2))</x:f>
       </x:c>
       <x:c r="O72" s="74" t="str">
-        <x:f>IF($N72="","",ROUNDDOWN($N72*$E72,3))</x:f>
+        <x:f>IF($N72="","",ROUNDDOWN(ROUNDDOWN($N72,2)*$E72,3))</x:f>
       </x:c>
       <x:c r="P72" s="77" t="str">
         <x:f>IF($L72="","",$I72*$L72)</x:f>
@@ -4630,10 +4630,10 @@
         <x:f>IF($L73="","",$C73*$L73)</x:f>
       </x:c>
       <x:c r="N73" s="86" t="str">
-        <x:f>IF($M73="","",$C73+$M73)</x:f>
+        <x:f>IF($M73="","",ROUNDDOWN($C73+$M73,2))</x:f>
       </x:c>
       <x:c r="O73" s="74" t="str">
-        <x:f>IF($N73="","",ROUNDDOWN($N73*$E73,3))</x:f>
+        <x:f>IF($N73="","",ROUNDDOWN(ROUNDDOWN($N73,2)*$E73,3))</x:f>
       </x:c>
       <x:c r="P73" s="77" t="str">
         <x:f>IF($L73="","",$I73*$L73)</x:f>
@@ -4683,10 +4683,10 @@
         <x:f>IF($L74="","",$C74*$L74)</x:f>
       </x:c>
       <x:c r="N74" s="86" t="str">
-        <x:f>IF($M74="","",$C74+$M74)</x:f>
+        <x:f>IF($M74="","",ROUNDDOWN($C74+$M74,2))</x:f>
       </x:c>
       <x:c r="O74" s="74" t="str">
-        <x:f>IF($N74="","",ROUNDDOWN($N74*$E74,3))</x:f>
+        <x:f>IF($N74="","",ROUNDDOWN(ROUNDDOWN($N74,2)*$E74,3))</x:f>
       </x:c>
       <x:c r="P74" s="77" t="str">
         <x:f>IF($L74="","",$I74*$L74)</x:f>
@@ -4736,10 +4736,10 @@
         <x:f>IF($L75="","",$C75*$L75)</x:f>
       </x:c>
       <x:c r="N75" s="86" t="str">
-        <x:f>IF($M75="","",$C75+$M75)</x:f>
+        <x:f>IF($M75="","",ROUNDDOWN($C75+$M75,2))</x:f>
       </x:c>
       <x:c r="O75" s="74" t="str">
-        <x:f>IF($N75="","",ROUNDDOWN($N75*$E75,3))</x:f>
+        <x:f>IF($N75="","",ROUNDDOWN(ROUNDDOWN($N75,2)*$E75,3))</x:f>
       </x:c>
       <x:c r="P75" s="77" t="str">
         <x:f>IF($L75="","",$I75*$L75)</x:f>
@@ -4789,10 +4789,10 @@
         <x:f>IF($L76="","",$C76*$L76)</x:f>
       </x:c>
       <x:c r="N76" s="86" t="str">
-        <x:f>IF($M76="","",$C76+$M76)</x:f>
+        <x:f>IF($M76="","",ROUNDDOWN($C76+$M76,2))</x:f>
       </x:c>
       <x:c r="O76" s="74" t="str">
-        <x:f>IF($N76="","",ROUNDDOWN($N76*$E76,3))</x:f>
+        <x:f>IF($N76="","",ROUNDDOWN(ROUNDDOWN($N76,2)*$E76,3))</x:f>
       </x:c>
       <x:c r="P76" s="77" t="str">
         <x:f>IF($L76="","",$I76*$L76)</x:f>
@@ -4842,10 +4842,10 @@
         <x:f>IF($L77="","",$C77*$L77)</x:f>
       </x:c>
       <x:c r="N77" s="86" t="str">
-        <x:f>IF($M77="","",$C77+$M77)</x:f>
+        <x:f>IF($M77="","",ROUNDDOWN($C77+$M77,2))</x:f>
       </x:c>
       <x:c r="O77" s="74" t="str">
-        <x:f>IF($N77="","",ROUNDDOWN($N77*$E77,3))</x:f>
+        <x:f>IF($N77="","",ROUNDDOWN(ROUNDDOWN($N77,2)*$E77,3))</x:f>
       </x:c>
       <x:c r="P77" s="77" t="str">
         <x:f>IF($L77="","",$I77*$L77)</x:f>
@@ -4895,10 +4895,10 @@
         <x:f>IF($L78="","",$C78*$L78)</x:f>
       </x:c>
       <x:c r="N78" s="86" t="str">
-        <x:f>IF($M78="","",$C78+$M78)</x:f>
+        <x:f>IF($M78="","",ROUNDDOWN($C78+$M78,2))</x:f>
       </x:c>
       <x:c r="O78" s="74" t="str">
-        <x:f>IF($N78="","",ROUNDDOWN($N78*$E78,3))</x:f>
+        <x:f>IF($N78="","",ROUNDDOWN(ROUNDDOWN($N78,2)*$E78,3))</x:f>
       </x:c>
       <x:c r="P78" s="77" t="str">
         <x:f>IF($L78="","",$I78*$L78)</x:f>
@@ -4948,10 +4948,10 @@
         <x:f>IF($L79="","",$C79*$L79)</x:f>
       </x:c>
       <x:c r="N79" s="86" t="str">
-        <x:f>IF($M79="","",$C79+$M79)</x:f>
+        <x:f>IF($M79="","",ROUNDDOWN($C79+$M79,2))</x:f>
       </x:c>
       <x:c r="O79" s="74" t="str">
-        <x:f>IF($N79="","",ROUNDDOWN($N79*$E79,3))</x:f>
+        <x:f>IF($N79="","",ROUNDDOWN(ROUNDDOWN($N79,2)*$E79,3))</x:f>
       </x:c>
       <x:c r="P79" s="77" t="str">
         <x:f>IF($L79="","",$I79*$L79)</x:f>
@@ -5001,10 +5001,10 @@
         <x:f>IF($L80="","",$C80*$L80)</x:f>
       </x:c>
       <x:c r="N80" s="86" t="str">
-        <x:f>IF($M80="","",$C80+$M80)</x:f>
+        <x:f>IF($M80="","",ROUNDDOWN($C80+$M80,2))</x:f>
       </x:c>
       <x:c r="O80" s="74" t="str">
-        <x:f>IF($N80="","",ROUNDDOWN($N80*$E80,3))</x:f>
+        <x:f>IF($N80="","",ROUNDDOWN(ROUNDDOWN($N80,2)*$E80,3))</x:f>
       </x:c>
       <x:c r="P80" s="77" t="str">
         <x:f>IF($L80="","",$I80*$L80)</x:f>
@@ -5054,10 +5054,10 @@
         <x:f>IF($L81="","",$C81*$L81)</x:f>
       </x:c>
       <x:c r="N81" s="86" t="str">
-        <x:f>IF($M81="","",$C81+$M81)</x:f>
+        <x:f>IF($M81="","",ROUNDDOWN($C81+$M81,2))</x:f>
       </x:c>
       <x:c r="O81" s="74" t="str">
-        <x:f>IF($N81="","",ROUNDDOWN($N81*$E81,3))</x:f>
+        <x:f>IF($N81="","",ROUNDDOWN(ROUNDDOWN($N81,2)*$E81,3))</x:f>
       </x:c>
       <x:c r="P81" s="77" t="str">
         <x:f>IF($L81="","",$I81*$L81)</x:f>
@@ -5107,10 +5107,10 @@
         <x:f>IF($L82="","",$C82*$L82)</x:f>
       </x:c>
       <x:c r="N82" s="86" t="str">
-        <x:f>IF($M82="","",$C82+$M82)</x:f>
+        <x:f>IF($M82="","",ROUNDDOWN($C82+$M82,2))</x:f>
       </x:c>
       <x:c r="O82" s="74" t="str">
-        <x:f>IF($N82="","",ROUNDDOWN($N82*$E82,3))</x:f>
+        <x:f>IF($N82="","",ROUNDDOWN(ROUNDDOWN($N82,2)*$E82,3))</x:f>
       </x:c>
       <x:c r="P82" s="77" t="str">
         <x:f>IF($L82="","",$I82*$L82)</x:f>
@@ -5160,10 +5160,10 @@
         <x:f>IF($L83="","",$C83*$L83)</x:f>
       </x:c>
       <x:c r="N83" s="86" t="str">
-        <x:f>IF($M83="","",$C83+$M83)</x:f>
+        <x:f>IF($M83="","",ROUNDDOWN($C83+$M83,2))</x:f>
       </x:c>
       <x:c r="O83" s="74" t="str">
-        <x:f>IF($N83="","",ROUNDDOWN($N83*$E83,3))</x:f>
+        <x:f>IF($N83="","",ROUNDDOWN(ROUNDDOWN($N83,2)*$E83,3))</x:f>
       </x:c>
       <x:c r="P83" s="77" t="str">
         <x:f>IF($L83="","",$I83*$L83)</x:f>
@@ -5213,10 +5213,10 @@
         <x:f>IF($L84="","",$C84*$L84)</x:f>
       </x:c>
       <x:c r="N84" s="86" t="str">
-        <x:f>IF($M84="","",$C84+$M84)</x:f>
+        <x:f>IF($M84="","",ROUNDDOWN($C84+$M84,2))</x:f>
       </x:c>
       <x:c r="O84" s="74" t="str">
-        <x:f>IF($N84="","",ROUNDDOWN($N84*$E84,3))</x:f>
+        <x:f>IF($N84="","",ROUNDDOWN(ROUNDDOWN($N84,2)*$E84,3))</x:f>
       </x:c>
       <x:c r="P84" s="77" t="str">
         <x:f>IF($L84="","",$I84*$L84)</x:f>
@@ -5266,10 +5266,10 @@
         <x:f>IF($L85="","",$C85*$L85)</x:f>
       </x:c>
       <x:c r="N85" s="86" t="str">
-        <x:f>IF($M85="","",$C85+$M85)</x:f>
+        <x:f>IF($M85="","",ROUNDDOWN($C85+$M85,2))</x:f>
       </x:c>
       <x:c r="O85" s="74" t="str">
-        <x:f>IF($N85="","",ROUNDDOWN($N85*$E85,3))</x:f>
+        <x:f>IF($N85="","",ROUNDDOWN(ROUNDDOWN($N85,2)*$E85,3))</x:f>
       </x:c>
       <x:c r="P85" s="77" t="str">
         <x:f>IF($L85="","",$I85*$L85)</x:f>
@@ -5319,10 +5319,10 @@
         <x:f>IF($L86="","",$C86*$L86)</x:f>
       </x:c>
       <x:c r="N86" s="86" t="str">
-        <x:f>IF($M86="","",$C86+$M86)</x:f>
+        <x:f>IF($M86="","",ROUNDDOWN($C86+$M86,2))</x:f>
       </x:c>
       <x:c r="O86" s="74" t="str">
-        <x:f>IF($N86="","",ROUNDDOWN($N86*$E86,3))</x:f>
+        <x:f>IF($N86="","",ROUNDDOWN(ROUNDDOWN($N86,2)*$E86,3))</x:f>
       </x:c>
       <x:c r="P86" s="77" t="str">
         <x:f>IF($L86="","",$I86*$L86)</x:f>
@@ -5372,10 +5372,10 @@
         <x:f>IF($L87="","",$C87*$L87)</x:f>
       </x:c>
       <x:c r="N87" s="86" t="str">
-        <x:f>IF($M87="","",$C87+$M87)</x:f>
+        <x:f>IF($M87="","",ROUNDDOWN($C87+$M87,2))</x:f>
       </x:c>
       <x:c r="O87" s="74" t="str">
-        <x:f>IF($N87="","",ROUNDDOWN($N87*$E87,3))</x:f>
+        <x:f>IF($N87="","",ROUNDDOWN(ROUNDDOWN($N87,2)*$E87,3))</x:f>
       </x:c>
       <x:c r="P87" s="77" t="str">
         <x:f>IF($L87="","",$I87*$L87)</x:f>
@@ -5425,10 +5425,10 @@
         <x:f>IF($L88="","",$C88*$L88)</x:f>
       </x:c>
       <x:c r="N88" s="86" t="str">
-        <x:f>IF($M88="","",$C88+$M88)</x:f>
+        <x:f>IF($M88="","",ROUNDDOWN($C88+$M88,2))</x:f>
       </x:c>
       <x:c r="O88" s="74" t="str">
-        <x:f>IF($N88="","",ROUNDDOWN($N88*$E88,3))</x:f>
+        <x:f>IF($N88="","",ROUNDDOWN(ROUNDDOWN($N88,2)*$E88,3))</x:f>
       </x:c>
       <x:c r="P88" s="77" t="str">
         <x:f>IF($L88="","",$I88*$L88)</x:f>
@@ -5478,10 +5478,10 @@
         <x:f>IF($L89="","",$C89*$L89)</x:f>
       </x:c>
       <x:c r="N89" s="86" t="str">
-        <x:f>IF($M89="","",$C89+$M89)</x:f>
+        <x:f>IF($M89="","",ROUNDDOWN($C89+$M89,2))</x:f>
       </x:c>
       <x:c r="O89" s="74" t="str">
-        <x:f>IF($N89="","",ROUNDDOWN($N89*$E89,3))</x:f>
+        <x:f>IF($N89="","",ROUNDDOWN(ROUNDDOWN($N89,2)*$E89,3))</x:f>
       </x:c>
       <x:c r="P89" s="77" t="str">
         <x:f>IF($L89="","",$I89*$L89)</x:f>
@@ -5531,10 +5531,10 @@
         <x:f>IF($L90="","",$C90*$L90)</x:f>
       </x:c>
       <x:c r="N90" s="86" t="str">
-        <x:f>IF($M90="","",$C90+$M90)</x:f>
+        <x:f>IF($M90="","",ROUNDDOWN($C90+$M90,2))</x:f>
       </x:c>
       <x:c r="O90" s="74" t="str">
-        <x:f>IF($N90="","",ROUNDDOWN($N90*$E90,3))</x:f>
+        <x:f>IF($N90="","",ROUNDDOWN(ROUNDDOWN($N90,2)*$E90,3))</x:f>
       </x:c>
       <x:c r="P90" s="77" t="str">
         <x:f>IF($L90="","",$I90*$L90)</x:f>
@@ -5584,10 +5584,10 @@
         <x:f>IF($L91="","",$C91*$L91)</x:f>
       </x:c>
       <x:c r="N91" s="86" t="str">
-        <x:f>IF($M91="","",$C91+$M91)</x:f>
+        <x:f>IF($M91="","",ROUNDDOWN($C91+$M91,2))</x:f>
       </x:c>
       <x:c r="O91" s="74" t="str">
-        <x:f>IF($N91="","",ROUNDDOWN($N91*$E91,3))</x:f>
+        <x:f>IF($N91="","",ROUNDDOWN(ROUNDDOWN($N91,2)*$E91,3))</x:f>
       </x:c>
       <x:c r="P91" s="77" t="str">
         <x:f>IF($L91="","",$I91*$L91)</x:f>
@@ -5637,10 +5637,10 @@
         <x:f>IF($L92="","",$C92*$L92)</x:f>
       </x:c>
       <x:c r="N92" s="86" t="str">
-        <x:f>IF($M92="","",$C92+$M92)</x:f>
+        <x:f>IF($M92="","",ROUNDDOWN($C92+$M92,2))</x:f>
       </x:c>
       <x:c r="O92" s="74" t="str">
-        <x:f>IF($N92="","",ROUNDDOWN($N92*$E92,3))</x:f>
+        <x:f>IF($N92="","",ROUNDDOWN(ROUNDDOWN($N92,2)*$E92,3))</x:f>
       </x:c>
       <x:c r="P92" s="77" t="str">
         <x:f>IF($L92="","",$I92*$L92)</x:f>
@@ -5690,10 +5690,10 @@
         <x:f>IF($L93="","",$C93*$L93)</x:f>
       </x:c>
       <x:c r="N93" s="86" t="str">
-        <x:f>IF($M93="","",$C93+$M93)</x:f>
+        <x:f>IF($M93="","",ROUNDDOWN($C93+$M93,2))</x:f>
       </x:c>
       <x:c r="O93" s="74" t="str">
-        <x:f>IF($N93="","",ROUNDDOWN($N93*$E93,3))</x:f>
+        <x:f>IF($N93="","",ROUNDDOWN(ROUNDDOWN($N93,2)*$E93,3))</x:f>
       </x:c>
       <x:c r="P93" s="77" t="str">
         <x:f>IF($L93="","",$I93*$L93)</x:f>
@@ -5743,10 +5743,10 @@
         <x:f>IF($L94="","",$C94*$L94)</x:f>
       </x:c>
       <x:c r="N94" s="86" t="str">
-        <x:f>IF($M94="","",$C94+$M94)</x:f>
+        <x:f>IF($M94="","",ROUNDDOWN($C94+$M94,2))</x:f>
       </x:c>
       <x:c r="O94" s="74" t="str">
-        <x:f>IF($N94="","",ROUNDDOWN($N94*$E94,3))</x:f>
+        <x:f>IF($N94="","",ROUNDDOWN(ROUNDDOWN($N94,2)*$E94,3))</x:f>
       </x:c>
       <x:c r="P94" s="77" t="str">
         <x:f>IF($L94="","",$I94*$L94)</x:f>
@@ -5796,10 +5796,10 @@
         <x:f>IF($L95="","",$C95*$L95)</x:f>
       </x:c>
       <x:c r="N95" s="86" t="str">
-        <x:f>IF($M95="","",$C95+$M95)</x:f>
+        <x:f>IF($M95="","",ROUNDDOWN($C95+$M95,2))</x:f>
       </x:c>
       <x:c r="O95" s="74" t="str">
-        <x:f>IF($N95="","",ROUNDDOWN($N95*$E95,3))</x:f>
+        <x:f>IF($N95="","",ROUNDDOWN(ROUNDDOWN($N95,2)*$E95,3))</x:f>
       </x:c>
       <x:c r="P95" s="77" t="str">
         <x:f>IF($L95="","",$I95*$L95)</x:f>
@@ -5849,10 +5849,10 @@
         <x:f>IF($L96="","",$C96*$L96)</x:f>
       </x:c>
       <x:c r="N96" s="86" t="str">
-        <x:f>IF($M96="","",$C96+$M96)</x:f>
+        <x:f>IF($M96="","",ROUNDDOWN($C96+$M96,2))</x:f>
       </x:c>
       <x:c r="O96" s="74" t="str">
-        <x:f>IF($N96="","",ROUNDDOWN($N96*$E96,3))</x:f>
+        <x:f>IF($N96="","",ROUNDDOWN(ROUNDDOWN($N96,2)*$E96,3))</x:f>
       </x:c>
       <x:c r="P96" s="77" t="str">
         <x:f>IF($L96="","",$I96*$L96)</x:f>
@@ -5902,10 +5902,10 @@
         <x:f>IF($L97="","",$C97*$L97)</x:f>
       </x:c>
       <x:c r="N97" s="86" t="str">
-        <x:f>IF($M97="","",$C97+$M97)</x:f>
+        <x:f>IF($M97="","",ROUNDDOWN($C97+$M97,2))</x:f>
       </x:c>
       <x:c r="O97" s="74" t="str">
-        <x:f>IF($N97="","",ROUNDDOWN($N97*$E97,3))</x:f>
+        <x:f>IF($N97="","",ROUNDDOWN(ROUNDDOWN($N97,2)*$E97,3))</x:f>
       </x:c>
       <x:c r="P97" s="77" t="str">
         <x:f>IF($L97="","",$I97*$L97)</x:f>
@@ -5955,10 +5955,10 @@
         <x:f>IF($L98="","",$C98*$L98)</x:f>
       </x:c>
       <x:c r="N98" s="86" t="str">
-        <x:f>IF($M98="","",$C98+$M98)</x:f>
+        <x:f>IF($M98="","",ROUNDDOWN($C98+$M98,2))</x:f>
       </x:c>
       <x:c r="O98" s="74" t="str">
-        <x:f>IF($N98="","",ROUNDDOWN($N98*$E98,3))</x:f>
+        <x:f>IF($N98="","",ROUNDDOWN(ROUNDDOWN($N98,2)*$E98,3))</x:f>
       </x:c>
       <x:c r="P98" s="77" t="str">
         <x:f>IF($L98="","",$I98*$L98)</x:f>
@@ -6008,10 +6008,10 @@
         <x:f>IF($L99="","",$C99*$L99)</x:f>
       </x:c>
       <x:c r="N99" s="86" t="str">
-        <x:f>IF($M99="","",$C99+$M99)</x:f>
+        <x:f>IF($M99="","",ROUNDDOWN($C99+$M99,2))</x:f>
       </x:c>
       <x:c r="O99" s="74" t="str">
-        <x:f>IF($N99="","",ROUNDDOWN($N99*$E99,3))</x:f>
+        <x:f>IF($N99="","",ROUNDDOWN(ROUNDDOWN($N99,2)*$E99,3))</x:f>
       </x:c>
       <x:c r="P99" s="77" t="str">
         <x:f>IF($L99="","",$I99*$L99)</x:f>
@@ -6061,10 +6061,10 @@
         <x:f>IF($L100="","",$C100*$L100)</x:f>
       </x:c>
       <x:c r="N100" s="86" t="str">
-        <x:f>IF($M100="","",$C100+$M100)</x:f>
+        <x:f>IF($M100="","",ROUNDDOWN($C100+$M100,2))</x:f>
       </x:c>
       <x:c r="O100" s="74" t="str">
-        <x:f>IF($N100="","",ROUNDDOWN($N100*$E100,3))</x:f>
+        <x:f>IF($N100="","",ROUNDDOWN(ROUNDDOWN($N100,2)*$E100,3))</x:f>
       </x:c>
       <x:c r="P100" s="77" t="str">
         <x:f>IF($L100="","",$I100*$L100)</x:f>
@@ -6114,10 +6114,10 @@
         <x:f>IF($L101="","",$C101*$L101)</x:f>
       </x:c>
       <x:c r="N101" s="86" t="str">
-        <x:f>IF($M101="","",$C101+$M101)</x:f>
+        <x:f>IF($M101="","",ROUNDDOWN($C101+$M101,2))</x:f>
       </x:c>
       <x:c r="O101" s="74" t="str">
-        <x:f>IF($N101="","",ROUNDDOWN($N101*$E101,3))</x:f>
+        <x:f>IF($N101="","",ROUNDDOWN(ROUNDDOWN($N101,2)*$E101,3))</x:f>
       </x:c>
       <x:c r="P101" s="77" t="str">
         <x:f>IF($L101="","",$I101*$L101)</x:f>
@@ -6167,10 +6167,10 @@
         <x:f>IF($L102="","",$C102*$L102)</x:f>
       </x:c>
       <x:c r="N102" s="86" t="str">
-        <x:f>IF($M102="","",$C102+$M102)</x:f>
+        <x:f>IF($M102="","",ROUNDDOWN($C102+$M102,2))</x:f>
       </x:c>
       <x:c r="O102" s="74" t="str">
-        <x:f>IF($N102="","",ROUNDDOWN($N102*$E102,3))</x:f>
+        <x:f>IF($N102="","",ROUNDDOWN(ROUNDDOWN($N102,2)*$E102,3))</x:f>
       </x:c>
       <x:c r="P102" s="77" t="str">
         <x:f>IF($L102="","",$I102*$L102)</x:f>
@@ -6220,10 +6220,10 @@
         <x:f>IF($L103="","",$C103*$L103)</x:f>
       </x:c>
       <x:c r="N103" s="86" t="str">
-        <x:f>IF($M103="","",$C103+$M103)</x:f>
+        <x:f>IF($M103="","",ROUNDDOWN($C103+$M103,2))</x:f>
       </x:c>
       <x:c r="O103" s="74" t="str">
-        <x:f>IF($N103="","",ROUNDDOWN($N103*$E103,3))</x:f>
+        <x:f>IF($N103="","",ROUNDDOWN(ROUNDDOWN($N103,2)*$E103,3))</x:f>
       </x:c>
       <x:c r="P103" s="77" t="str">
         <x:f>IF($L103="","",$I103*$L103)</x:f>
@@ -6273,10 +6273,10 @@
         <x:f>IF($L104="","",$C104*$L104)</x:f>
       </x:c>
       <x:c r="N104" s="86" t="str">
-        <x:f>IF($M104="","",$C104+$M104)</x:f>
+        <x:f>IF($M104="","",ROUNDDOWN($C104+$M104,2))</x:f>
       </x:c>
       <x:c r="O104" s="74" t="str">
-        <x:f>IF($N104="","",ROUNDDOWN($N104*$E104,3))</x:f>
+        <x:f>IF($N104="","",ROUNDDOWN(ROUNDDOWN($N104,2)*$E104,3))</x:f>
       </x:c>
       <x:c r="P104" s="77" t="str">
         <x:f>IF($L104="","",$I104*$L104)</x:f>
@@ -6326,10 +6326,10 @@
         <x:f>IF($L105="","",$C105*$L105)</x:f>
       </x:c>
       <x:c r="N105" s="86" t="str">
-        <x:f>IF($M105="","",$C105+$M105)</x:f>
+        <x:f>IF($M105="","",ROUNDDOWN($C105+$M105,2))</x:f>
       </x:c>
       <x:c r="O105" s="74" t="str">
-        <x:f>IF($N105="","",ROUNDDOWN($N105*$E105,3))</x:f>
+        <x:f>IF($N105="","",ROUNDDOWN(ROUNDDOWN($N105,2)*$E105,3))</x:f>
       </x:c>
       <x:c r="P105" s="77" t="str">
         <x:f>IF($L105="","",$I105*$L105)</x:f>
@@ -6379,10 +6379,10 @@
         <x:f>IF($L106="","",$C106*$L106)</x:f>
       </x:c>
       <x:c r="N106" s="86" t="str">
-        <x:f>IF($M106="","",$C106+$M106)</x:f>
+        <x:f>IF($M106="","",ROUNDDOWN($C106+$M106,2))</x:f>
       </x:c>
       <x:c r="O106" s="74" t="str">
-        <x:f>IF($N106="","",ROUNDDOWN($N106*$E106,3))</x:f>
+        <x:f>IF($N106="","",ROUNDDOWN(ROUNDDOWN($N106,2)*$E106,3))</x:f>
       </x:c>
       <x:c r="P106" s="77" t="str">
         <x:f>IF($L106="","",$I106*$L106)</x:f>
@@ -6432,10 +6432,10 @@
         <x:f>IF($L107="","",$C107*$L107)</x:f>
       </x:c>
       <x:c r="N107" s="86" t="str">
-        <x:f>IF($M107="","",$C107+$M107)</x:f>
+        <x:f>IF($M107="","",ROUNDDOWN($C107+$M107,2))</x:f>
       </x:c>
       <x:c r="O107" s="74" t="str">
-        <x:f>IF($N107="","",ROUNDDOWN($N107*$E107,3))</x:f>
+        <x:f>IF($N107="","",ROUNDDOWN(ROUNDDOWN($N107,2)*$E107,3))</x:f>
       </x:c>
       <x:c r="P107" s="77" t="str">
         <x:f>IF($L107="","",$I107*$L107)</x:f>
@@ -6485,10 +6485,10 @@
         <x:f>IF($L108="","",$C108*$L108)</x:f>
       </x:c>
       <x:c r="N108" s="86" t="str">
-        <x:f>IF($M108="","",$C108+$M108)</x:f>
+        <x:f>IF($M108="","",ROUNDDOWN($C108+$M108,2))</x:f>
       </x:c>
       <x:c r="O108" s="74" t="str">
-        <x:f>IF($N108="","",ROUNDDOWN($N108*$E108,3))</x:f>
+        <x:f>IF($N108="","",ROUNDDOWN(ROUNDDOWN($N108,2)*$E108,3))</x:f>
       </x:c>
       <x:c r="P108" s="77" t="str">
         <x:f>IF($L108="","",$I108*$L108)</x:f>
@@ -6538,10 +6538,10 @@
         <x:f>IF($L109="","",$C109*$L109)</x:f>
       </x:c>
       <x:c r="N109" s="86" t="str">
-        <x:f>IF($M109="","",$C109+$M109)</x:f>
+        <x:f>IF($M109="","",ROUNDDOWN($C109+$M109,2))</x:f>
       </x:c>
       <x:c r="O109" s="74" t="str">
-        <x:f>IF($N109="","",ROUNDDOWN($N109*$E109,3))</x:f>
+        <x:f>IF($N109="","",ROUNDDOWN(ROUNDDOWN($N109,2)*$E109,3))</x:f>
       </x:c>
       <x:c r="P109" s="77" t="str">
         <x:f>IF($L109="","",$I109*$L109)</x:f>
@@ -6591,10 +6591,10 @@
         <x:f>IF($L110="","",$C110*$L110)</x:f>
       </x:c>
       <x:c r="N110" s="86" t="str">
-        <x:f>IF($M110="","",$C110+$M110)</x:f>
+        <x:f>IF($M110="","",ROUNDDOWN($C110+$M110,2))</x:f>
       </x:c>
       <x:c r="O110" s="74" t="str">
-        <x:f>IF($N110="","",ROUNDDOWN($N110*$E110,3))</x:f>
+        <x:f>IF($N110="","",ROUNDDOWN(ROUNDDOWN($N110,2)*$E110,3))</x:f>
       </x:c>
       <x:c r="P110" s="77" t="str">
         <x:f>IF($L110="","",$I110*$L110)</x:f>
@@ -6644,10 +6644,10 @@
         <x:f>IF($L111="","",$C111*$L111)</x:f>
       </x:c>
       <x:c r="N111" s="86" t="str">
-        <x:f>IF($M111="","",$C111+$M111)</x:f>
+        <x:f>IF($M111="","",ROUNDDOWN($C111+$M111,2))</x:f>
       </x:c>
       <x:c r="O111" s="74" t="str">
-        <x:f>IF($N111="","",ROUNDDOWN($N111*$E111,3))</x:f>
+        <x:f>IF($N111="","",ROUNDDOWN(ROUNDDOWN($N111,2)*$E111,3))</x:f>
       </x:c>
       <x:c r="P111" s="77" t="str">
         <x:f>IF($L111="","",$I111*$L111)</x:f>
@@ -6697,10 +6697,10 @@
         <x:f>IF($L112="","",$C112*$L112)</x:f>
       </x:c>
       <x:c r="N112" s="86" t="str">
-        <x:f>IF($M112="","",$C112+$M112)</x:f>
+        <x:f>IF($M112="","",ROUNDDOWN($C112+$M112,2))</x:f>
       </x:c>
       <x:c r="O112" s="74" t="str">
-        <x:f>IF($N112="","",ROUNDDOWN($N112*$E112,3))</x:f>
+        <x:f>IF($N112="","",ROUNDDOWN(ROUNDDOWN($N112,2)*$E112,3))</x:f>
       </x:c>
       <x:c r="P112" s="77" t="str">
         <x:f>IF($L112="","",$I112*$L112)</x:f>
@@ -6750,10 +6750,10 @@
         <x:f>IF($L113="","",$C113*$L113)</x:f>
       </x:c>
       <x:c r="N113" s="86" t="str">
-        <x:f>IF($M113="","",$C113+$M113)</x:f>
+        <x:f>IF($M113="","",ROUNDDOWN($C113+$M113,2))</x:f>
       </x:c>
       <x:c r="O113" s="74" t="str">
-        <x:f>IF($N113="","",ROUNDDOWN($N113*$E113,3))</x:f>
+        <x:f>IF($N113="","",ROUNDDOWN(ROUNDDOWN($N113,2)*$E113,3))</x:f>
       </x:c>
       <x:c r="P113" s="77" t="str">
         <x:f>IF($L113="","",$I113*$L113)</x:f>
@@ -6803,10 +6803,10 @@
         <x:f>IF($L114="","",$C114*$L114)</x:f>
       </x:c>
       <x:c r="N114" s="86" t="str">
-        <x:f>IF($M114="","",$C114+$M114)</x:f>
+        <x:f>IF($M114="","",ROUNDDOWN($C114+$M114,2))</x:f>
       </x:c>
       <x:c r="O114" s="74" t="str">
-        <x:f>IF($N114="","",ROUNDDOWN($N114*$E114,3))</x:f>
+        <x:f>IF($N114="","",ROUNDDOWN(ROUNDDOWN($N114,2)*$E114,3))</x:f>
       </x:c>
       <x:c r="P114" s="77" t="str">
         <x:f>IF($L114="","",$I114*$L114)</x:f>
@@ -6856,10 +6856,10 @@
         <x:f>IF($L115="","",$C115*$L115)</x:f>
       </x:c>
       <x:c r="N115" s="86" t="str">
-        <x:f>IF($M115="","",$C115+$M115)</x:f>
+        <x:f>IF($M115="","",ROUNDDOWN($C115+$M115,2))</x:f>
       </x:c>
       <x:c r="O115" s="74" t="str">
-        <x:f>IF($N115="","",ROUNDDOWN($N115*$E115,3))</x:f>
+        <x:f>IF($N115="","",ROUNDDOWN(ROUNDDOWN($N115,2)*$E115,3))</x:f>
       </x:c>
       <x:c r="P115" s="77" t="str">
         <x:f>IF($L115="","",$I115*$L115)</x:f>
@@ -6909,10 +6909,10 @@
         <x:f>IF($L116="","",$C116*$L116)</x:f>
       </x:c>
       <x:c r="N116" s="86" t="str">
-        <x:f>IF($M116="","",$C116+$M116)</x:f>
+        <x:f>IF($M116="","",ROUNDDOWN($C116+$M116,2))</x:f>
       </x:c>
       <x:c r="O116" s="74" t="str">
-        <x:f>IF($N116="","",ROUNDDOWN($N116*$E116,3))</x:f>
+        <x:f>IF($N116="","",ROUNDDOWN(ROUNDDOWN($N116,2)*$E116,3))</x:f>
       </x:c>
       <x:c r="P116" s="77" t="str">
         <x:f>IF($L116="","",$I116*$L116)</x:f>
@@ -6962,10 +6962,10 @@
         <x:f>IF($L117="","",$C117*$L117)</x:f>
       </x:c>
       <x:c r="N117" s="86" t="str">
-        <x:f>IF($M117="","",$C117+$M117)</x:f>
+        <x:f>IF($M117="","",ROUNDDOWN($C117+$M117,2))</x:f>
       </x:c>
       <x:c r="O117" s="74" t="str">
-        <x:f>IF($N117="","",ROUNDDOWN($N117*$E117,3))</x:f>
+        <x:f>IF($N117="","",ROUNDDOWN(ROUNDDOWN($N117,2)*$E117,3))</x:f>
       </x:c>
       <x:c r="P117" s="77" t="str">
         <x:f>IF($L117="","",$I117*$L117)</x:f>
@@ -7015,10 +7015,10 @@
         <x:f>IF($L118="","",$C118*$L118)</x:f>
       </x:c>
       <x:c r="N118" s="86" t="str">
-        <x:f>IF($M118="","",$C118+$M118)</x:f>
+        <x:f>IF($M118="","",ROUNDDOWN($C118+$M118,2))</x:f>
       </x:c>
       <x:c r="O118" s="74" t="str">
-        <x:f>IF($N118="","",ROUNDDOWN($N118*$E118,3))</x:f>
+        <x:f>IF($N118="","",ROUNDDOWN(ROUNDDOWN($N118,2)*$E118,3))</x:f>
       </x:c>
       <x:c r="P118" s="77" t="str">
         <x:f>IF($L118="","",$I118*$L118)</x:f>
@@ -7068,10 +7068,10 @@
         <x:f>IF($L119="","",$C119*$L119)</x:f>
       </x:c>
       <x:c r="N119" s="86" t="str">
-        <x:f>IF($M119="","",$C119+$M119)</x:f>
+        <x:f>IF($M119="","",ROUNDDOWN($C119+$M119,2))</x:f>
       </x:c>
       <x:c r="O119" s="74" t="str">
-        <x:f>IF($N119="","",ROUNDDOWN($N119*$E119,3))</x:f>
+        <x:f>IF($N119="","",ROUNDDOWN(ROUNDDOWN($N119,2)*$E119,3))</x:f>
       </x:c>
       <x:c r="P119" s="77" t="str">
         <x:f>IF($L119="","",$I119*$L119)</x:f>
@@ -7121,10 +7121,10 @@
         <x:f>IF($L120="","",$C120*$L120)</x:f>
       </x:c>
       <x:c r="N120" s="86" t="str">
-        <x:f>IF($M120="","",$C120+$M120)</x:f>
+        <x:f>IF($M120="","",ROUNDDOWN($C120+$M120,2))</x:f>
       </x:c>
       <x:c r="O120" s="74" t="str">
-        <x:f>IF($N120="","",ROUNDDOWN($N120*$E120,3))</x:f>
+        <x:f>IF($N120="","",ROUNDDOWN(ROUNDDOWN($N120,2)*$E120,3))</x:f>
       </x:c>
       <x:c r="P120" s="77" t="str">
         <x:f>IF($L120="","",$I120*$L120)</x:f>
@@ -7174,10 +7174,10 @@
         <x:f>IF($L121="","",$C121*$L121)</x:f>
       </x:c>
       <x:c r="N121" s="86" t="str">
-        <x:f>IF($M121="","",$C121+$M121)</x:f>
+        <x:f>IF($M121="","",ROUNDDOWN($C121+$M121,2))</x:f>
       </x:c>
       <x:c r="O121" s="74" t="str">
-        <x:f>IF($N121="","",ROUNDDOWN($N121*$E121,3))</x:f>
+        <x:f>IF($N121="","",ROUNDDOWN(ROUNDDOWN($N121,2)*$E121,3))</x:f>
       </x:c>
       <x:c r="P121" s="77" t="str">
         <x:f>IF($L121="","",$I121*$L121)</x:f>
@@ -7227,10 +7227,10 @@
         <x:f>IF($L122="","",$C122*$L122)</x:f>
       </x:c>
       <x:c r="N122" s="86" t="str">
-        <x:f>IF($M122="","",$C122+$M122)</x:f>
+        <x:f>IF($M122="","",ROUNDDOWN($C122+$M122,2))</x:f>
       </x:c>
       <x:c r="O122" s="74" t="str">
-        <x:f>IF($N122="","",ROUNDDOWN($N122*$E122,3))</x:f>
+        <x:f>IF($N122="","",ROUNDDOWN(ROUNDDOWN($N122,2)*$E122,3))</x:f>
       </x:c>
       <x:c r="P122" s="77" t="str">
         <x:f>IF($L122="","",$I122*$L122)</x:f>
@@ -7280,10 +7280,10 @@
         <x:f>IF($L123="","",$C123*$L123)</x:f>
       </x:c>
       <x:c r="N123" s="86" t="str">
-        <x:f>IF($M123="","",$C123+$M123)</x:f>
+        <x:f>IF($M123="","",ROUNDDOWN($C123+$M123,2))</x:f>
       </x:c>
       <x:c r="O123" s="74" t="str">
-        <x:f>IF($N123="","",ROUNDDOWN($N123*$E123,3))</x:f>
+        <x:f>IF($N123="","",ROUNDDOWN(ROUNDDOWN($N123,2)*$E123,3))</x:f>
       </x:c>
       <x:c r="P123" s="77" t="str">
         <x:f>IF($L123="","",$I123*$L123)</x:f>
@@ -7333,10 +7333,10 @@
         <x:f>IF($L124="","",$C124*$L124)</x:f>
       </x:c>
       <x:c r="N124" s="86" t="str">
-        <x:f>IF($M124="","",$C124+$M124)</x:f>
+        <x:f>IF($M124="","",ROUNDDOWN($C124+$M124,2))</x:f>
       </x:c>
       <x:c r="O124" s="74" t="str">
-        <x:f>IF($N124="","",ROUNDDOWN($N124*$E124,3))</x:f>
+        <x:f>IF($N124="","",ROUNDDOWN(ROUNDDOWN($N124,2)*$E124,3))</x:f>
       </x:c>
       <x:c r="P124" s="77" t="str">
         <x:f>IF($L124="","",$I124*$L124)</x:f>
@@ -7386,10 +7386,10 @@
         <x:f>IF($L125="","",$C125*$L125)</x:f>
       </x:c>
       <x:c r="N125" s="86" t="str">
-        <x:f>IF($M125="","",$C125+$M125)</x:f>
+        <x:f>IF($M125="","",ROUNDDOWN($C125+$M125,2))</x:f>
       </x:c>
       <x:c r="O125" s="74" t="str">
-        <x:f>IF($N125="","",ROUNDDOWN($N125*$E125,3))</x:f>
+        <x:f>IF($N125="","",ROUNDDOWN(ROUNDDOWN($N125,2)*$E125,3))</x:f>
       </x:c>
       <x:c r="P125" s="77" t="str">
         <x:f>IF($L125="","",$I125*$L125)</x:f>
@@ -7439,10 +7439,10 @@
         <x:f>IF($L126="","",$C126*$L126)</x:f>
       </x:c>
       <x:c r="N126" s="86" t="str">
-        <x:f>IF($M126="","",$C126+$M126)</x:f>
+        <x:f>IF($M126="","",ROUNDDOWN($C126+$M126,2))</x:f>
       </x:c>
       <x:c r="O126" s="74" t="str">
-        <x:f>IF($N126="","",ROUNDDOWN($N126*$E126,3))</x:f>
+        <x:f>IF($N126="","",ROUNDDOWN(ROUNDDOWN($N126,2)*$E126,3))</x:f>
       </x:c>
       <x:c r="P126" s="77" t="str">
         <x:f>IF($L126="","",$I126*$L126)</x:f>
@@ -7492,10 +7492,10 @@
         <x:f>IF($L127="","",$C127*$L127)</x:f>
       </x:c>
       <x:c r="N127" s="86" t="str">
-        <x:f>IF($M127="","",$C127+$M127)</x:f>
+        <x:f>IF($M127="","",ROUNDDOWN($C127+$M127,2))</x:f>
       </x:c>
       <x:c r="O127" s="74" t="str">
-        <x:f>IF($N127="","",ROUNDDOWN($N127*$E127,3))</x:f>
+        <x:f>IF($N127="","",ROUNDDOWN(ROUNDDOWN($N127,2)*$E127,3))</x:f>
       </x:c>
       <x:c r="P127" s="77" t="str">
         <x:f>IF($L127="","",$I127*$L127)</x:f>
@@ -7545,10 +7545,10 @@
         <x:f>IF($L128="","",$C128*$L128)</x:f>
       </x:c>
       <x:c r="N128" s="86" t="str">
-        <x:f>IF($M128="","",$C128+$M128)</x:f>
+        <x:f>IF($M128="","",ROUNDDOWN($C128+$M128,2))</x:f>
       </x:c>
       <x:c r="O128" s="74" t="str">
-        <x:f>IF($N128="","",ROUNDDOWN($N128*$E128,3))</x:f>
+        <x:f>IF($N128="","",ROUNDDOWN(ROUNDDOWN($N128,2)*$E128,3))</x:f>
       </x:c>
       <x:c r="P128" s="77" t="str">
         <x:f>IF($L128="","",$I128*$L128)</x:f>
@@ -7598,10 +7598,10 @@
         <x:f>IF($L129="","",$C129*$L129)</x:f>
       </x:c>
       <x:c r="N129" s="86" t="str">
-        <x:f>IF($M129="","",$C129+$M129)</x:f>
+        <x:f>IF($M129="","",ROUNDDOWN($C129+$M129,2))</x:f>
       </x:c>
       <x:c r="O129" s="74" t="str">
-        <x:f>IF($N129="","",ROUNDDOWN($N129*$E129,3))</x:f>
+        <x:f>IF($N129="","",ROUNDDOWN(ROUNDDOWN($N129,2)*$E129,3))</x:f>
       </x:c>
       <x:c r="P129" s="77" t="str">
         <x:f>IF($L129="","",$I129*$L129)</x:f>
@@ -7651,10 +7651,10 @@
         <x:f>IF($L130="","",$C130*$L130)</x:f>
       </x:c>
       <x:c r="N130" s="86" t="str">
-        <x:f>IF($M130="","",$C130+$M130)</x:f>
+        <x:f>IF($M130="","",ROUNDDOWN($C130+$M130,2))</x:f>
       </x:c>
       <x:c r="O130" s="74" t="str">
-        <x:f>IF($N130="","",ROUNDDOWN($N130*$E130,3))</x:f>
+        <x:f>IF($N130="","",ROUNDDOWN(ROUNDDOWN($N130,2)*$E130,3))</x:f>
       </x:c>
       <x:c r="P130" s="77" t="str">
         <x:f>IF($L130="","",$I130*$L130)</x:f>
@@ -7704,10 +7704,10 @@
         <x:f>IF($L131="","",$C131*$L131)</x:f>
       </x:c>
       <x:c r="N131" s="86" t="str">
-        <x:f>IF($M131="","",$C131+$M131)</x:f>
+        <x:f>IF($M131="","",ROUNDDOWN($C131+$M131,2))</x:f>
       </x:c>
       <x:c r="O131" s="74" t="str">
-        <x:f>IF($N131="","",ROUNDDOWN($N131*$E131,3))</x:f>
+        <x:f>IF($N131="","",ROUNDDOWN(ROUNDDOWN($N131,2)*$E131,3))</x:f>
       </x:c>
       <x:c r="P131" s="77" t="str">
         <x:f>IF($L131="","",$I131*$L131)</x:f>
@@ -7757,10 +7757,10 @@
         <x:f>IF($L132="","",$C132*$L132)</x:f>
       </x:c>
       <x:c r="N132" s="86" t="str">
-        <x:f>IF($M132="","",$C132+$M132)</x:f>
+        <x:f>IF($M132="","",ROUNDDOWN($C132+$M132,2))</x:f>
       </x:c>
       <x:c r="O132" s="74" t="str">
-        <x:f>IF($N132="","",ROUNDDOWN($N132*$E132,3))</x:f>
+        <x:f>IF($N132="","",ROUNDDOWN(ROUNDDOWN($N132,2)*$E132,3))</x:f>
       </x:c>
       <x:c r="P132" s="77" t="str">
         <x:f>IF($L132="","",$I132*$L132)</x:f>
@@ -7810,10 +7810,10 @@
         <x:f>IF($L133="","",$C133*$L133)</x:f>
       </x:c>
       <x:c r="N133" s="86" t="str">
-        <x:f>IF($M133="","",$C133+$M133)</x:f>
+        <x:f>IF($M133="","",ROUNDDOWN($C133+$M133,2))</x:f>
       </x:c>
       <x:c r="O133" s="74" t="str">
-        <x:f>IF($N133="","",ROUNDDOWN($N133*$E133,3))</x:f>
+        <x:f>IF($N133="","",ROUNDDOWN(ROUNDDOWN($N133,2)*$E133,3))</x:f>
       </x:c>
       <x:c r="P133" s="77" t="str">
         <x:f>IF($L133="","",$I133*$L133)</x:f>
@@ -7863,10 +7863,10 @@
         <x:f>IF($L134="","",$C134*$L134)</x:f>
       </x:c>
       <x:c r="N134" s="86" t="str">
-        <x:f>IF($M134="","",$C134+$M134)</x:f>
+        <x:f>IF($M134="","",ROUNDDOWN($C134+$M134,2))</x:f>
       </x:c>
       <x:c r="O134" s="74" t="str">
-        <x:f>IF($N134="","",ROUNDDOWN($N134*$E134,3))</x:f>
+        <x:f>IF($N134="","",ROUNDDOWN(ROUNDDOWN($N134,2)*$E134,3))</x:f>
       </x:c>
       <x:c r="P134" s="77" t="str">
         <x:f>IF($L134="","",$I134*$L134)</x:f>
@@ -7916,10 +7916,10 @@
         <x:f>IF($L135="","",$C135*$L135)</x:f>
       </x:c>
       <x:c r="N135" s="86" t="str">
-        <x:f>IF($M135="","",$C135+$M135)</x:f>
+        <x:f>IF($M135="","",ROUNDDOWN($C135+$M135,2))</x:f>
       </x:c>
       <x:c r="O135" s="74" t="str">
-        <x:f>IF($N135="","",ROUNDDOWN($N135*$E135,3))</x:f>
+        <x:f>IF($N135="","",ROUNDDOWN(ROUNDDOWN($N135,2)*$E135,3))</x:f>
       </x:c>
       <x:c r="P135" s="77" t="str">
         <x:f>IF($L135="","",$I135*$L135)</x:f>
@@ -7969,10 +7969,10 @@
         <x:f>IF($L136="","",$C136*$L136)</x:f>
       </x:c>
       <x:c r="N136" s="86" t="str">
-        <x:f>IF($M136="","",$C136+$M136)</x:f>
+        <x:f>IF($M136="","",ROUNDDOWN($C136+$M136,2))</x:f>
       </x:c>
       <x:c r="O136" s="74" t="str">
-        <x:f>IF($N136="","",ROUNDDOWN($N136*$E136,3))</x:f>
+        <x:f>IF($N136="","",ROUNDDOWN(ROUNDDOWN($N136,2)*$E136,3))</x:f>
       </x:c>
       <x:c r="P136" s="77" t="str">
         <x:f>IF($L136="","",$I136*$L136)</x:f>
@@ -8022,10 +8022,10 @@
         <x:f>IF($L137="","",$C137*$L137)</x:f>
       </x:c>
       <x:c r="N137" s="86" t="str">
-        <x:f>IF($M137="","",$C137+$M137)</x:f>
+        <x:f>IF($M137="","",ROUNDDOWN($C137+$M137,2))</x:f>
       </x:c>
       <x:c r="O137" s="74" t="str">
-        <x:f>IF($N137="","",ROUNDDOWN($N137*$E137,3))</x:f>
+        <x:f>IF($N137="","",ROUNDDOWN(ROUNDDOWN($N137,2)*$E137,3))</x:f>
       </x:c>
       <x:c r="P137" s="77" t="str">
         <x:f>IF($L137="","",$I137*$L137)</x:f>
@@ -8075,10 +8075,10 @@
         <x:f>IF($L138="","",$C138*$L138)</x:f>
       </x:c>
       <x:c r="N138" s="86" t="str">
-        <x:f>IF($M138="","",$C138+$M138)</x:f>
+        <x:f>IF($M138="","",ROUNDDOWN($C138+$M138,2))</x:f>
       </x:c>
       <x:c r="O138" s="74" t="str">
-        <x:f>IF($N138="","",ROUNDDOWN($N138*$E138,3))</x:f>
+        <x:f>IF($N138="","",ROUNDDOWN(ROUNDDOWN($N138,2)*$E138,3))</x:f>
       </x:c>
       <x:c r="P138" s="77" t="str">
         <x:f>IF($L138="","",$I138*$L138)</x:f>
@@ -8128,10 +8128,10 @@
         <x:f>IF($L139="","",$C139*$L139)</x:f>
       </x:c>
       <x:c r="N139" s="86" t="str">
-        <x:f>IF($M139="","",$C139+$M139)</x:f>
+        <x:f>IF($M139="","",ROUNDDOWN($C139+$M139,2))</x:f>
       </x:c>
       <x:c r="O139" s="74" t="str">
-        <x:f>IF($N139="","",ROUNDDOWN($N139*$E139,3))</x:f>
+        <x:f>IF($N139="","",ROUNDDOWN(ROUNDDOWN($N139,2)*$E139,3))</x:f>
       </x:c>
       <x:c r="P139" s="77" t="str">
         <x:f>IF($L139="","",$I139*$L139)</x:f>
@@ -8181,10 +8181,10 @@
         <x:f>IF($L140="","",$C140*$L140)</x:f>
       </x:c>
       <x:c r="N140" s="86" t="str">
-        <x:f>IF($M140="","",$C140+$M140)</x:f>
+        <x:f>IF($M140="","",ROUNDDOWN($C140+$M140,2))</x:f>
       </x:c>
       <x:c r="O140" s="74" t="str">
-        <x:f>IF($N140="","",ROUNDDOWN($N140*$E140,3))</x:f>
+        <x:f>IF($N140="","",ROUNDDOWN(ROUNDDOWN($N140,2)*$E140,3))</x:f>
       </x:c>
       <x:c r="P140" s="77" t="str">
         <x:f>IF($L140="","",$I140*$L140)</x:f>
@@ -8234,10 +8234,10 @@
         <x:f>IF($L141="","",$C141*$L141)</x:f>
       </x:c>
       <x:c r="N141" s="86" t="str">
-        <x:f>IF($M141="","",$C141+$M141)</x:f>
+        <x:f>IF($M141="","",ROUNDDOWN($C141+$M141,2))</x:f>
       </x:c>
       <x:c r="O141" s="74" t="str">
-        <x:f>IF($N141="","",ROUNDDOWN($N141*$E141,3))</x:f>
+        <x:f>IF($N141="","",ROUNDDOWN(ROUNDDOWN($N141,2)*$E141,3))</x:f>
       </x:c>
       <x:c r="P141" s="77" t="str">
         <x:f>IF($L141="","",$I141*$L141)</x:f>
@@ -8287,10 +8287,10 @@
         <x:f>IF($L142="","",$C142*$L142)</x:f>
       </x:c>
       <x:c r="N142" s="86" t="str">
-        <x:f>IF($M142="","",$C142+$M142)</x:f>
+        <x:f>IF($M142="","",ROUNDDOWN($C142+$M142,2))</x:f>
       </x:c>
       <x:c r="O142" s="74" t="str">
-        <x:f>IF($N142="","",ROUNDDOWN($N142*$E142,3))</x:f>
+        <x:f>IF($N142="","",ROUNDDOWN(ROUNDDOWN($N142,2)*$E142,3))</x:f>
       </x:c>
       <x:c r="P142" s="77" t="str">
         <x:f>IF($L142="","",$I142*$L142)</x:f>
@@ -8340,10 +8340,10 @@
         <x:f>IF($L143="","",$C143*$L143)</x:f>
       </x:c>
       <x:c r="N143" s="86" t="str">
-        <x:f>IF($M143="","",$C143+$M143)</x:f>
+        <x:f>IF($M143="","",ROUNDDOWN($C143+$M143,2))</x:f>
       </x:c>
       <x:c r="O143" s="74" t="str">
-        <x:f>IF($N143="","",ROUNDDOWN($N143*$E143,3))</x:f>
+        <x:f>IF($N143="","",ROUNDDOWN(ROUNDDOWN($N143,2)*$E143,3))</x:f>
       </x:c>
       <x:c r="P143" s="77" t="str">
         <x:f>IF($L143="","",$I143*$L143)</x:f>
@@ -8393,10 +8393,10 @@
         <x:f>IF($L144="","",$C144*$L144)</x:f>
       </x:c>
       <x:c r="N144" s="86" t="str">
-        <x:f>IF($M144="","",$C144+$M144)</x:f>
+        <x:f>IF($M144="","",ROUNDDOWN($C144+$M144,2))</x:f>
       </x:c>
       <x:c r="O144" s="74" t="str">
-        <x:f>IF($N144="","",ROUNDDOWN($N144*$E144,3))</x:f>
+        <x:f>IF($N144="","",ROUNDDOWN(ROUNDDOWN($N144,2)*$E144,3))</x:f>
       </x:c>
       <x:c r="P144" s="77" t="str">
         <x:f>IF($L144="","",$I144*$L144)</x:f>
@@ -8446,10 +8446,10 @@
         <x:f>IF($L145="","",$C145*$L145)</x:f>
       </x:c>
       <x:c r="N145" s="86" t="str">
-        <x:f>IF($M145="","",$C145+$M145)</x:f>
+        <x:f>IF($M145="","",ROUNDDOWN($C145+$M145,2))</x:f>
       </x:c>
       <x:c r="O145" s="74" t="str">
-        <x:f>IF($N145="","",ROUNDDOWN($N145*$E145,3))</x:f>
+        <x:f>IF($N145="","",ROUNDDOWN(ROUNDDOWN($N145,2)*$E145,3))</x:f>
       </x:c>
       <x:c r="P145" s="77" t="str">
         <x:f>IF($L145="","",$I145*$L145)</x:f>
@@ -8499,10 +8499,10 @@
         <x:f>IF($L146="","",$C146*$L146)</x:f>
       </x:c>
       <x:c r="N146" s="86" t="str">
-        <x:f>IF($M146="","",$C146+$M146)</x:f>
+        <x:f>IF($M146="","",ROUNDDOWN($C146+$M146,2))</x:f>
       </x:c>
       <x:c r="O146" s="74" t="str">
-        <x:f>IF($N146="","",ROUNDDOWN($N146*$E146,3))</x:f>
+        <x:f>IF($N146="","",ROUNDDOWN(ROUNDDOWN($N146,2)*$E146,3))</x:f>
       </x:c>
       <x:c r="P146" s="77" t="str">
         <x:f>IF($L146="","",$I146*$L146)</x:f>
@@ -8552,10 +8552,10 @@
         <x:f>IF($L147="","",$C147*$L147)</x:f>
       </x:c>
       <x:c r="N147" s="86" t="str">
-        <x:f>IF($M147="","",$C147+$M147)</x:f>
+        <x:f>IF($M147="","",ROUNDDOWN($C147+$M147,2))</x:f>
       </x:c>
       <x:c r="O147" s="74" t="str">
-        <x:f>IF($N147="","",ROUNDDOWN($N147*$E147,3))</x:f>
+        <x:f>IF($N147="","",ROUNDDOWN(ROUNDDOWN($N147,2)*$E147,3))</x:f>
       </x:c>
       <x:c r="P147" s="77" t="str">
         <x:f>IF($L147="","",$I147*$L147)</x:f>
@@ -8605,10 +8605,10 @@
         <x:f>IF($L148="","",$C148*$L148)</x:f>
       </x:c>
       <x:c r="N148" s="86" t="str">
-        <x:f>IF($M148="","",$C148+$M148)</x:f>
+        <x:f>IF($M148="","",ROUNDDOWN($C148+$M148,2))</x:f>
       </x:c>
       <x:c r="O148" s="74" t="str">
-        <x:f>IF($N148="","",ROUNDDOWN($N148*$E148,3))</x:f>
+        <x:f>IF($N148="","",ROUNDDOWN(ROUNDDOWN($N148,2)*$E148,3))</x:f>
       </x:c>
       <x:c r="P148" s="77" t="str">
         <x:f>IF($L148="","",$I148*$L148)</x:f>
@@ -8658,10 +8658,10 @@
         <x:f>IF($L149="","",$C149*$L149)</x:f>
       </x:c>
       <x:c r="N149" s="86" t="str">
-        <x:f>IF($M149="","",$C149+$M149)</x:f>
+        <x:f>IF($M149="","",ROUNDDOWN($C149+$M149,2))</x:f>
       </x:c>
       <x:c r="O149" s="74" t="str">
-        <x:f>IF($N149="","",ROUNDDOWN($N149*$E149,3))</x:f>
+        <x:f>IF($N149="","",ROUNDDOWN(ROUNDDOWN($N149,2)*$E149,3))</x:f>
       </x:c>
       <x:c r="P149" s="77" t="str">
         <x:f>IF($L149="","",$I149*$L149)</x:f>
@@ -8711,10 +8711,10 @@
         <x:f>IF($L150="","",$C150*$L150)</x:f>
       </x:c>
       <x:c r="N150" s="86" t="str">
-        <x:f>IF($M150="","",$C150+$M150)</x:f>
+        <x:f>IF($M150="","",ROUNDDOWN($C150+$M150,2))</x:f>
       </x:c>
       <x:c r="O150" s="74" t="str">
-        <x:f>IF($N150="","",ROUNDDOWN($N150*$E150,3))</x:f>
+        <x:f>IF($N150="","",ROUNDDOWN(ROUNDDOWN($N150,2)*$E150,3))</x:f>
       </x:c>
       <x:c r="P150" s="77" t="str">
         <x:f>IF($L150="","",$I150*$L150)</x:f>
@@ -8764,10 +8764,10 @@
         <x:f>IF($L151="","",$C151*$L151)</x:f>
       </x:c>
       <x:c r="N151" s="86" t="str">
-        <x:f>IF($M151="","",$C151+$M151)</x:f>
+        <x:f>IF($M151="","",ROUNDDOWN($C151+$M151,2))</x:f>
       </x:c>
       <x:c r="O151" s="74" t="str">
-        <x:f>IF($N151="","",ROUNDDOWN($N151*$E151,3))</x:f>
+        <x:f>IF($N151="","",ROUNDDOWN(ROUNDDOWN($N151,2)*$E151,3))</x:f>
       </x:c>
       <x:c r="P151" s="77" t="str">
         <x:f>IF($L151="","",$I151*$L151)</x:f>
@@ -8817,10 +8817,10 @@
         <x:f>IF($L152="","",$C152*$L152)</x:f>
       </x:c>
       <x:c r="N152" s="86" t="str">
-        <x:f>IF($M152="","",$C152+$M152)</x:f>
+        <x:f>IF($M152="","",ROUNDDOWN($C152+$M152,2))</x:f>
       </x:c>
       <x:c r="O152" s="74" t="str">
-        <x:f>IF($N152="","",ROUNDDOWN($N152*$E152,3))</x:f>
+        <x:f>IF($N152="","",ROUNDDOWN(ROUNDDOWN($N152,2)*$E152,3))</x:f>
       </x:c>
       <x:c r="P152" s="77" t="str">
         <x:f>IF($L152="","",$I152*$L152)</x:f>
@@ -8870,10 +8870,10 @@
         <x:f>IF($L153="","",$C153*$L153)</x:f>
       </x:c>
       <x:c r="N153" s="86" t="str">
-        <x:f>IF($M153="","",$C153+$M153)</x:f>
+        <x:f>IF($M153="","",ROUNDDOWN($C153+$M153,2))</x:f>
       </x:c>
       <x:c r="O153" s="74" t="str">
-        <x:f>IF($N153="","",ROUNDDOWN($N153*$E153,3))</x:f>
+        <x:f>IF($N153="","",ROUNDDOWN(ROUNDDOWN($N153,2)*$E153,3))</x:f>
       </x:c>
       <x:c r="P153" s="77" t="str">
         <x:f>IF($L153="","",$I153*$L153)</x:f>
@@ -8923,10 +8923,10 @@
         <x:f>IF($L154="","",$C154*$L154)</x:f>
       </x:c>
       <x:c r="N154" s="86" t="str">
-        <x:f>IF($M154="","",$C154+$M154)</x:f>
+        <x:f>IF($M154="","",ROUNDDOWN($C154+$M154,2))</x:f>
       </x:c>
       <x:c r="O154" s="74" t="str">
-        <x:f>IF($N154="","",ROUNDDOWN($N154*$E154,3))</x:f>
+        <x:f>IF($N154="","",ROUNDDOWN(ROUNDDOWN($N154,2)*$E154,3))</x:f>
       </x:c>
       <x:c r="P154" s="77" t="str">
         <x:f>IF($L154="","",$I154*$L154)</x:f>
@@ -8976,10 +8976,10 @@
         <x:f>IF($L155="","",$C155*$L155)</x:f>
       </x:c>
       <x:c r="N155" s="86" t="str">
-        <x:f>IF($M155="","",$C155+$M155)</x:f>
+        <x:f>IF($M155="","",ROUNDDOWN($C155+$M155,2))</x:f>
       </x:c>
       <x:c r="O155" s="74" t="str">
-        <x:f>IF($N155="","",ROUNDDOWN($N155*$E155,3))</x:f>
+        <x:f>IF($N155="","",ROUNDDOWN(ROUNDDOWN($N155,2)*$E155,3))</x:f>
       </x:c>
       <x:c r="P155" s="77" t="str">
         <x:f>IF($L155="","",$I155*$L155)</x:f>
@@ -9029,10 +9029,10 @@
         <x:f>IF($L156="","",$C156*$L156)</x:f>
       </x:c>
       <x:c r="N156" s="86" t="str">
-        <x:f>IF($M156="","",$C156+$M156)</x:f>
+        <x:f>IF($M156="","",ROUNDDOWN($C156+$M156,2))</x:f>
       </x:c>
       <x:c r="O156" s="74" t="str">
-        <x:f>IF($N156="","",ROUNDDOWN($N156*$E156,3))</x:f>
+        <x:f>IF($N156="","",ROUNDDOWN(ROUNDDOWN($N156,2)*$E156,3))</x:f>
       </x:c>
       <x:c r="P156" s="77" t="str">
         <x:f>IF($L156="","",$I156*$L156)</x:f>
@@ -9082,10 +9082,10 @@
         <x:f>IF($L157="","",$C157*$L157)</x:f>
       </x:c>
       <x:c r="N157" s="86" t="str">
-        <x:f>IF($M157="","",$C157+$M157)</x:f>
+        <x:f>IF($M157="","",ROUNDDOWN($C157+$M157,2))</x:f>
       </x:c>
       <x:c r="O157" s="74" t="str">
-        <x:f>IF($N157="","",ROUNDDOWN($N157*$E157,3))</x:f>
+        <x:f>IF($N157="","",ROUNDDOWN(ROUNDDOWN($N157,2)*$E157,3))</x:f>
       </x:c>
       <x:c r="P157" s="77" t="str">
         <x:f>IF($L157="","",$I157*$L157)</x:f>
@@ -9135,10 +9135,10 @@
         <x:f>IF($L158="","",$C158*$L158)</x:f>
       </x:c>
       <x:c r="N158" s="86" t="str">
-        <x:f>IF($M158="","",$C158+$M158)</x:f>
+        <x:f>IF($M158="","",ROUNDDOWN($C158+$M158,2))</x:f>
       </x:c>
       <x:c r="O158" s="74" t="str">
-        <x:f>IF($N158="","",ROUNDDOWN($N158*$E158,3))</x:f>
+        <x:f>IF($N158="","",ROUNDDOWN(ROUNDDOWN($N158,2)*$E158,3))</x:f>
       </x:c>
       <x:c r="P158" s="77" t="str">
         <x:f>IF($L158="","",$I158*$L158)</x:f>
@@ -9188,10 +9188,10 @@
         <x:f>IF($L159="","",$C159*$L159)</x:f>
       </x:c>
       <x:c r="N159" s="86" t="str">
-        <x:f>IF($M159="","",$C159+$M159)</x:f>
+        <x:f>IF($M159="","",ROUNDDOWN($C159+$M159,2))</x:f>
       </x:c>
       <x:c r="O159" s="74" t="str">
-        <x:f>IF($N159="","",ROUNDDOWN($N159*$E159,3))</x:f>
+        <x:f>IF($N159="","",ROUNDDOWN(ROUNDDOWN($N159,2)*$E159,3))</x:f>
       </x:c>
       <x:c r="P159" s="77" t="str">
         <x:f>IF($L159="","",$I159*$L159)</x:f>
@@ -9241,10 +9241,10 @@
         <x:f>IF($L160="","",$C160*$L160)</x:f>
       </x:c>
       <x:c r="N160" s="86" t="str">
-        <x:f>IF($M160="","",$C160+$M160)</x:f>
+        <x:f>IF($M160="","",ROUNDDOWN($C160+$M160,2))</x:f>
       </x:c>
       <x:c r="O160" s="74" t="str">
-        <x:f>IF($N160="","",ROUNDDOWN($N160*$E160,3))</x:f>
+        <x:f>IF($N160="","",ROUNDDOWN(ROUNDDOWN($N160,2)*$E160,3))</x:f>
       </x:c>
       <x:c r="P160" s="77" t="str">
         <x:f>IF($L160="","",$I160*$L160)</x:f>
@@ -9294,10 +9294,10 @@
         <x:f>IF($L161="","",$C161*$L161)</x:f>
       </x:c>
       <x:c r="N161" s="86" t="str">
-        <x:f>IF($M161="","",$C161+$M161)</x:f>
+        <x:f>IF($M161="","",ROUNDDOWN($C161+$M161,2))</x:f>
       </x:c>
       <x:c r="O161" s="74" t="str">
-        <x:f>IF($N161="","",ROUNDDOWN($N161*$E161,3))</x:f>
+        <x:f>IF($N161="","",ROUNDDOWN(ROUNDDOWN($N161,2)*$E161,3))</x:f>
       </x:c>
       <x:c r="P161" s="77" t="str">
         <x:f>IF($L161="","",$I161*$L161)</x:f>
@@ -9347,10 +9347,10 @@
         <x:f>IF($L162="","",$C162*$L162)</x:f>
       </x:c>
       <x:c r="N162" s="86" t="str">
-        <x:f>IF($M162="","",$C162+$M162)</x:f>
+        <x:f>IF($M162="","",ROUNDDOWN($C162+$M162,2))</x:f>
       </x:c>
       <x:c r="O162" s="74" t="str">
-        <x:f>IF($N162="","",ROUNDDOWN($N162*$E162,3))</x:f>
+        <x:f>IF($N162="","",ROUNDDOWN(ROUNDDOWN($N162,2)*$E162,3))</x:f>
       </x:c>
       <x:c r="P162" s="77" t="str">
         <x:f>IF($L162="","",$I162*$L162)</x:f>
@@ -9400,10 +9400,10 @@
         <x:f>IF($L163="","",$C163*$L163)</x:f>
       </x:c>
       <x:c r="N163" s="86" t="str">
-        <x:f>IF($M163="","",$C163+$M163)</x:f>
+        <x:f>IF($M163="","",ROUNDDOWN($C163+$M163,2))</x:f>
       </x:c>
       <x:c r="O163" s="74" t="str">
-        <x:f>IF($N163="","",ROUNDDOWN($N163*$E163,3))</x:f>
+        <x:f>IF($N163="","",ROUNDDOWN(ROUNDDOWN($N163,2)*$E163,3))</x:f>
       </x:c>
       <x:c r="P163" s="77" t="str">
         <x:f>IF($L163="","",$I163*$L163)</x:f>
@@ -9453,10 +9453,10 @@
         <x:f>IF($L164="","",$C164*$L164)</x:f>
       </x:c>
       <x:c r="N164" s="86" t="str">
-        <x:f>IF($M164="","",$C164+$M164)</x:f>
+        <x:f>IF($M164="","",ROUNDDOWN($C164+$M164,2))</x:f>
       </x:c>
       <x:c r="O164" s="74" t="str">
-        <x:f>IF($N164="","",ROUNDDOWN($N164*$E164,3))</x:f>
+        <x:f>IF($N164="","",ROUNDDOWN(ROUNDDOWN($N164,2)*$E164,3))</x:f>
       </x:c>
       <x:c r="P164" s="77" t="str">
         <x:f>IF($L164="","",$I164*$L164)</x:f>
@@ -9506,10 +9506,10 @@
         <x:f>IF($L165="","",$C165*$L165)</x:f>
       </x:c>
       <x:c r="N165" s="86" t="str">
-        <x:f>IF($M165="","",$C165+$M165)</x:f>
+        <x:f>IF($M165="","",ROUNDDOWN($C165+$M165,2))</x:f>
       </x:c>
       <x:c r="O165" s="74" t="str">
-        <x:f>IF($N165="","",ROUNDDOWN($N165*$E165,3))</x:f>
+        <x:f>IF($N165="","",ROUNDDOWN(ROUNDDOWN($N165,2)*$E165,3))</x:f>
       </x:c>
       <x:c r="P165" s="77" t="str">
         <x:f>IF($L165="","",$I165*$L165)</x:f>
@@ -9559,10 +9559,10 @@
         <x:f>IF($L166="","",$C166*$L166)</x:f>
       </x:c>
       <x:c r="N166" s="86" t="str">
-        <x:f>IF($M166="","",$C166+$M166)</x:f>
+        <x:f>IF($M166="","",ROUNDDOWN($C166+$M166,2))</x:f>
       </x:c>
       <x:c r="O166" s="74" t="str">
-        <x:f>IF($N166="","",ROUNDDOWN($N166*$E166,3))</x:f>
+        <x:f>IF($N166="","",ROUNDDOWN(ROUNDDOWN($N166,2)*$E166,3))</x:f>
       </x:c>
       <x:c r="P166" s="77" t="str">
         <x:f>IF($L166="","",$I166*$L166)</x:f>
@@ -9612,10 +9612,10 @@
         <x:f>IF($L167="","",$C167*$L167)</x:f>
       </x:c>
       <x:c r="N167" s="86" t="str">
-        <x:f>IF($M167="","",$C167+$M167)</x:f>
+        <x:f>IF($M167="","",ROUNDDOWN($C167+$M167,2))</x:f>
       </x:c>
       <x:c r="O167" s="74" t="str">
-        <x:f>IF($N167="","",ROUNDDOWN($N167*$E167,3))</x:f>
+        <x:f>IF($N167="","",ROUNDDOWN(ROUNDDOWN($N167,2)*$E167,3))</x:f>
       </x:c>
       <x:c r="P167" s="77" t="str">
         <x:f>IF($L167="","",$I167*$L167)</x:f>
@@ -9665,10 +9665,10 @@
         <x:f>IF($L168="","",$C168*$L168)</x:f>
       </x:c>
       <x:c r="N168" s="86" t="str">
-        <x:f>IF($M168="","",$C168+$M168)</x:f>
+        <x:f>IF($M168="","",ROUNDDOWN($C168+$M168,2))</x:f>
       </x:c>
       <x:c r="O168" s="74" t="str">
-        <x:f>IF($N168="","",ROUNDDOWN($N168*$E168,3))</x:f>
+        <x:f>IF($N168="","",ROUNDDOWN(ROUNDDOWN($N168,2)*$E168,3))</x:f>
       </x:c>
       <x:c r="P168" s="77" t="str">
         <x:f>IF($L168="","",$I168*$L168)</x:f>
@@ -9718,10 +9718,10 @@
         <x:f>IF($L169="","",$C169*$L169)</x:f>
       </x:c>
       <x:c r="N169" s="86" t="str">
-        <x:f>IF($M169="","",$C169+$M169)</x:f>
+        <x:f>IF($M169="","",ROUNDDOWN($C169+$M169,2))</x:f>
       </x:c>
       <x:c r="O169" s="74" t="str">
-        <x:f>IF($N169="","",ROUNDDOWN($N169*$E169,3))</x:f>
+        <x:f>IF($N169="","",ROUNDDOWN(ROUNDDOWN($N169,2)*$E169,3))</x:f>
       </x:c>
       <x:c r="P169" s="77" t="str">
         <x:f>IF($L169="","",$I169*$L169)</x:f>
@@ -9771,10 +9771,10 @@
         <x:f>IF($L170="","",$C170*$L170)</x:f>
       </x:c>
       <x:c r="N170" s="86" t="str">
-        <x:f>IF($M170="","",$C170+$M170)</x:f>
+        <x:f>IF($M170="","",ROUNDDOWN($C170+$M170,2))</x:f>
       </x:c>
       <x:c r="O170" s="74" t="str">
-        <x:f>IF($N170="","",ROUNDDOWN($N170*$E170,3))</x:f>
+        <x:f>IF($N170="","",ROUNDDOWN(ROUNDDOWN($N170,2)*$E170,3))</x:f>
       </x:c>
       <x:c r="P170" s="77" t="str">
         <x:f>IF($L170="","",$I170*$L170)</x:f>
@@ -9824,10 +9824,10 @@
         <x:f>IF($L171="","",$C171*$L171)</x:f>
       </x:c>
       <x:c r="N171" s="86" t="str">
-        <x:f>IF($M171="","",$C171+$M171)</x:f>
+        <x:f>IF($M171="","",ROUNDDOWN($C171+$M171,2))</x:f>
       </x:c>
       <x:c r="O171" s="74" t="str">
-        <x:f>IF($N171="","",ROUNDDOWN($N171*$E171,3))</x:f>
+        <x:f>IF($N171="","",ROUNDDOWN(ROUNDDOWN($N171,2)*$E171,3))</x:f>
       </x:c>
       <x:c r="P171" s="77" t="str">
         <x:f>IF($L171="","",$I171*$L171)</x:f>
@@ -9877,10 +9877,10 @@
         <x:f>IF($L172="","",$C172*$L172)</x:f>
       </x:c>
       <x:c r="N172" s="86" t="str">
-        <x:f>IF($M172="","",$C172+$M172)</x:f>
+        <x:f>IF($M172="","",ROUNDDOWN($C172+$M172,2))</x:f>
       </x:c>
       <x:c r="O172" s="74" t="str">
-        <x:f>IF($N172="","",ROUNDDOWN($N172*$E172,3))</x:f>
+        <x:f>IF($N172="","",ROUNDDOWN(ROUNDDOWN($N172,2)*$E172,3))</x:f>
       </x:c>
       <x:c r="P172" s="77" t="str">
         <x:f>IF($L172="","",$I172*$L172)</x:f>
@@ -9930,10 +9930,10 @@
         <x:f>IF($L173="","",$C173*$L173)</x:f>
       </x:c>
       <x:c r="N173" s="86" t="str">
-        <x:f>IF($M173="","",$C173+$M173)</x:f>
+        <x:f>IF($M173="","",ROUNDDOWN($C173+$M173,2))</x:f>
       </x:c>
       <x:c r="O173" s="74" t="str">
-        <x:f>IF($N173="","",ROUNDDOWN($N173*$E173,3))</x:f>
+        <x:f>IF($N173="","",ROUNDDOWN(ROUNDDOWN($N173,2)*$E173,3))</x:f>
       </x:c>
       <x:c r="P173" s="77" t="str">
         <x:f>IF($L173="","",$I173*$L173)</x:f>
@@ -9983,10 +9983,10 @@
         <x:f>IF($L174="","",$C174*$L174)</x:f>
       </x:c>
       <x:c r="N174" s="86" t="str">
-        <x:f>IF($M174="","",$C174+$M174)</x:f>
+        <x:f>IF($M174="","",ROUNDDOWN($C174+$M174,2))</x:f>
       </x:c>
       <x:c r="O174" s="74" t="str">
-        <x:f>IF($N174="","",ROUNDDOWN($N174*$E174,3))</x:f>
+        <x:f>IF($N174="","",ROUNDDOWN(ROUNDDOWN($N174,2)*$E174,3))</x:f>
       </x:c>
       <x:c r="P174" s="77" t="str">
         <x:f>IF($L174="","",$I174*$L174)</x:f>
@@ -10036,10 +10036,10 @@
         <x:f>IF($L175="","",$C175*$L175)</x:f>
       </x:c>
       <x:c r="N175" s="86" t="str">
-        <x:f>IF($M175="","",$C175+$M175)</x:f>
+        <x:f>IF($M175="","",ROUNDDOWN($C175+$M175,2))</x:f>
       </x:c>
       <x:c r="O175" s="74" t="str">
-        <x:f>IF($N175="","",ROUNDDOWN($N175*$E175,3))</x:f>
+        <x:f>IF($N175="","",ROUNDDOWN(ROUNDDOWN($N175,2)*$E175,3))</x:f>
       </x:c>
       <x:c r="P175" s="77" t="str">
         <x:f>IF($L175="","",$I175*$L175)</x:f>
@@ -10089,10 +10089,10 @@
         <x:f>IF($L176="","",$C176*$L176)</x:f>
       </x:c>
       <x:c r="N176" s="86" t="str">
-        <x:f>IF($M176="","",$C176+$M176)</x:f>
+        <x:f>IF($M176="","",ROUNDDOWN($C176+$M176,2))</x:f>
       </x:c>
       <x:c r="O176" s="74" t="str">
-        <x:f>IF($N176="","",ROUNDDOWN($N176*$E176,3))</x:f>
+        <x:f>IF($N176="","",ROUNDDOWN(ROUNDDOWN($N176,2)*$E176,3))</x:f>
       </x:c>
       <x:c r="P176" s="77" t="str">
         <x:f>IF($L176="","",$I176*$L176)</x:f>
@@ -10142,10 +10142,10 @@
         <x:f>IF($L177="","",$C177*$L177)</x:f>
       </x:c>
       <x:c r="N177" s="86" t="str">
-        <x:f>IF($M177="","",$C177+$M177)</x:f>
+        <x:f>IF($M177="","",ROUNDDOWN($C177+$M177,2))</x:f>
       </x:c>
       <x:c r="O177" s="74" t="str">
-        <x:f>IF($N177="","",ROUNDDOWN($N177*$E177,3))</x:f>
+        <x:f>IF($N177="","",ROUNDDOWN(ROUNDDOWN($N177,2)*$E177,3))</x:f>
       </x:c>
       <x:c r="P177" s="77" t="str">
         <x:f>IF($L177="","",$I177*$L177)</x:f>
@@ -10195,10 +10195,10 @@
         <x:f>IF($L178="","",$C178*$L178)</x:f>
       </x:c>
       <x:c r="N178" s="86" t="str">
-        <x:f>IF($M178="","",$C178+$M178)</x:f>
+        <x:f>IF($M178="","",ROUNDDOWN($C178+$M178,2))</x:f>
       </x:c>
       <x:c r="O178" s="74" t="str">
-        <x:f>IF($N178="","",ROUNDDOWN($N178*$E178,3))</x:f>
+        <x:f>IF($N178="","",ROUNDDOWN(ROUNDDOWN($N178,2)*$E178,3))</x:f>
       </x:c>
       <x:c r="P178" s="77" t="str">
         <x:f>IF($L178="","",$I178*$L178)</x:f>
@@ -10248,10 +10248,10 @@
         <x:f>IF($L179="","",$C179*$L179)</x:f>
       </x:c>
       <x:c r="N179" s="86" t="str">
-        <x:f>IF($M179="","",$C179+$M179)</x:f>
+        <x:f>IF($M179="","",ROUNDDOWN($C179+$M179,2))</x:f>
       </x:c>
       <x:c r="O179" s="74" t="str">
-        <x:f>IF($N179="","",ROUNDDOWN($N179*$E179,3))</x:f>
+        <x:f>IF($N179="","",ROUNDDOWN(ROUNDDOWN($N179,2)*$E179,3))</x:f>
       </x:c>
       <x:c r="P179" s="77" t="str">
         <x:f>IF($L179="","",$I179*$L179)</x:f>
@@ -10301,10 +10301,10 @@
         <x:f>IF($L180="","",$C180*$L180)</x:f>
       </x:c>
       <x:c r="N180" s="86" t="str">
-        <x:f>IF($M180="","",$C180+$M180)</x:f>
+        <x:f>IF($M180="","",ROUNDDOWN($C180+$M180,2))</x:f>
       </x:c>
       <x:c r="O180" s="74" t="str">
-        <x:f>IF($N180="","",ROUNDDOWN($N180*$E180,3))</x:f>
+        <x:f>IF($N180="","",ROUNDDOWN(ROUNDDOWN($N180,2)*$E180,3))</x:f>
       </x:c>
       <x:c r="P180" s="77" t="str">
         <x:f>IF($L180="","",$I180*$L180)</x:f>
@@ -10354,10 +10354,10 @@
         <x:f>IF($L181="","",$C181*$L181)</x:f>
       </x:c>
       <x:c r="N181" s="86" t="str">
-        <x:f>IF($M181="","",$C181+$M181)</x:f>
+        <x:f>IF($M181="","",ROUNDDOWN($C181+$M181,2))</x:f>
       </x:c>
       <x:c r="O181" s="74" t="str">
-        <x:f>IF($N181="","",ROUNDDOWN($N181*$E181,3))</x:f>
+        <x:f>IF($N181="","",ROUNDDOWN(ROUNDDOWN($N181,2)*$E181,3))</x:f>
       </x:c>
       <x:c r="P181" s="77" t="str">
         <x:f>IF($L181="","",$I181*$L181)</x:f>
@@ -10407,10 +10407,10 @@
         <x:f>IF($L182="","",$C182*$L182)</x:f>
       </x:c>
       <x:c r="N182" s="86" t="str">
-        <x:f>IF($M182="","",$C182+$M182)</x:f>
+        <x:f>IF($M182="","",ROUNDDOWN($C182+$M182,2))</x:f>
       </x:c>
       <x:c r="O182" s="74" t="str">
-        <x:f>IF($N182="","",ROUNDDOWN($N182*$E182,3))</x:f>
+        <x:f>IF($N182="","",ROUNDDOWN(ROUNDDOWN($N182,2)*$E182,3))</x:f>
       </x:c>
       <x:c r="P182" s="77" t="str">
         <x:f>IF($L182="","",$I182*$L182)</x:f>
@@ -10460,10 +10460,10 @@
         <x:f>IF($L183="","",$C183*$L183)</x:f>
       </x:c>
       <x:c r="N183" s="86" t="str">
-        <x:f>IF($M183="","",$C183+$M183)</x:f>
+        <x:f>IF($M183="","",ROUNDDOWN($C183+$M183,2))</x:f>
       </x:c>
       <x:c r="O183" s="74" t="str">
-        <x:f>IF($N183="","",ROUNDDOWN($N183*$E183,3))</x:f>
+        <x:f>IF($N183="","",ROUNDDOWN(ROUNDDOWN($N183,2)*$E183,3))</x:f>
       </x:c>
       <x:c r="P183" s="77" t="str">
         <x:f>IF($L183="","",$I183*$L183)</x:f>
@@ -10513,10 +10513,10 @@
         <x:f>IF($L184="","",$C184*$L184)</x:f>
       </x:c>
       <x:c r="N184" s="86" t="str">
-        <x:f>IF($M184="","",$C184+$M184)</x:f>
+        <x:f>IF($M184="","",ROUNDDOWN($C184+$M184,2))</x:f>
       </x:c>
       <x:c r="O184" s="74" t="str">
-        <x:f>IF($N184="","",ROUNDDOWN($N184*$E184,3))</x:f>
+        <x:f>IF($N184="","",ROUNDDOWN(ROUNDDOWN($N184,2)*$E184,3))</x:f>
       </x:c>
       <x:c r="P184" s="77" t="str">
         <x:f>IF($L184="","",$I184*$L184)</x:f>
@@ -10566,10 +10566,10 @@
         <x:f>IF($L185="","",$C185*$L185)</x:f>
       </x:c>
       <x:c r="N185" s="86" t="str">
-        <x:f>IF($M185="","",$C185+$M185)</x:f>
+        <x:f>IF($M185="","",ROUNDDOWN($C185+$M185,2))</x:f>
       </x:c>
       <x:c r="O185" s="74" t="str">
-        <x:f>IF($N185="","",ROUNDDOWN($N185*$E185,3))</x:f>
+        <x:f>IF($N185="","",ROUNDDOWN(ROUNDDOWN($N185,2)*$E185,3))</x:f>
       </x:c>
       <x:c r="P185" s="77" t="str">
         <x:f>IF($L185="","",$I185*$L185)</x:f>
@@ -10619,10 +10619,10 @@
         <x:f>IF($L186="","",$C186*$L186)</x:f>
       </x:c>
       <x:c r="N186" s="86" t="str">
-        <x:f>IF($M186="","",$C186+$M186)</x:f>
+        <x:f>IF($M186="","",ROUNDDOWN($C186+$M186,2))</x:f>
       </x:c>
       <x:c r="O186" s="74" t="str">
-        <x:f>IF($N186="","",ROUNDDOWN($N186*$E186,3))</x:f>
+        <x:f>IF($N186="","",ROUNDDOWN(ROUNDDOWN($N186,2)*$E186,3))</x:f>
       </x:c>
       <x:c r="P186" s="77" t="str">
         <x:f>IF($L186="","",$I186*$L186)</x:f>
@@ -10672,10 +10672,10 @@
         <x:f>IF($L187="","",$C187*$L187)</x:f>
       </x:c>
       <x:c r="N187" s="86" t="str">
-        <x:f>IF($M187="","",$C187+$M187)</x:f>
+        <x:f>IF($M187="","",ROUNDDOWN($C187+$M187,2))</x:f>
       </x:c>
       <x:c r="O187" s="74" t="str">
-        <x:f>IF($N187="","",ROUNDDOWN($N187*$E187,3))</x:f>
+        <x:f>IF($N187="","",ROUNDDOWN(ROUNDDOWN($N187,2)*$E187,3))</x:f>
       </x:c>
       <x:c r="P187" s="77" t="str">
         <x:f>IF($L187="","",$I187*$L187)</x:f>
@@ -10725,10 +10725,10 @@
         <x:f>IF($L188="","",$C188*$L188)</x:f>
       </x:c>
       <x:c r="N188" s="86" t="str">
-        <x:f>IF($M188="","",$C188+$M188)</x:f>
+        <x:f>IF($M188="","",ROUNDDOWN($C188+$M188,2))</x:f>
       </x:c>
       <x:c r="O188" s="74" t="str">
-        <x:f>IF($N188="","",ROUNDDOWN($N188*$E188,3))</x:f>
+        <x:f>IF($N188="","",ROUNDDOWN(ROUNDDOWN($N188,2)*$E188,3))</x:f>
       </x:c>
       <x:c r="P188" s="77" t="str">
         <x:f>IF($L188="","",$I188*$L188)</x:f>
@@ -10778,10 +10778,10 @@
         <x:f>IF($L189="","",$C189*$L189)</x:f>
       </x:c>
       <x:c r="N189" s="86" t="str">
-        <x:f>IF($M189="","",$C189+$M189)</x:f>
+        <x:f>IF($M189="","",ROUNDDOWN($C189+$M189,2))</x:f>
       </x:c>
       <x:c r="O189" s="74" t="str">
-        <x:f>IF($N189="","",ROUNDDOWN($N189*$E189,3))</x:f>
+        <x:f>IF($N189="","",ROUNDDOWN(ROUNDDOWN($N189,2)*$E189,3))</x:f>
       </x:c>
       <x:c r="P189" s="77" t="str">
         <x:f>IF($L189="","",$I189*$L189)</x:f>
@@ -10831,10 +10831,10 @@
         <x:f>IF($L190="","",$C190*$L190)</x:f>
       </x:c>
       <x:c r="N190" s="86" t="str">
-        <x:f>IF($M190="","",$C190+$M190)</x:f>
+        <x:f>IF($M190="","",ROUNDDOWN($C190+$M190,2))</x:f>
       </x:c>
       <x:c r="O190" s="74" t="str">
-        <x:f>IF($N190="","",ROUNDDOWN($N190*$E190,3))</x:f>
+        <x:f>IF($N190="","",ROUNDDOWN(ROUNDDOWN($N190,2)*$E190,3))</x:f>
       </x:c>
       <x:c r="P190" s="77" t="str">
         <x:f>IF($L190="","",$I190*$L190)</x:f>
@@ -10884,10 +10884,10 @@
         <x:f>IF($L191="","",$C191*$L191)</x:f>
       </x:c>
       <x:c r="N191" s="86" t="str">
-        <x:f>IF($M191="","",$C191+$M191)</x:f>
+        <x:f>IF($M191="","",ROUNDDOWN($C191+$M191,2))</x:f>
       </x:c>
       <x:c r="O191" s="74" t="str">
-        <x:f>IF($N191="","",ROUNDDOWN($N191*$E191,3))</x:f>
+        <x:f>IF($N191="","",ROUNDDOWN(ROUNDDOWN($N191,2)*$E191,3))</x:f>
       </x:c>
       <x:c r="P191" s="77" t="str">
         <x:f>IF($L191="","",$I191*$L191)</x:f>
@@ -10937,10 +10937,10 @@
         <x:f>IF($L192="","",$C192*$L192)</x:f>
       </x:c>
       <x:c r="N192" s="86" t="str">
-        <x:f>IF($M192="","",$C192+$M192)</x:f>
+        <x:f>IF($M192="","",ROUNDDOWN($C192+$M192,2))</x:f>
       </x:c>
       <x:c r="O192" s="74" t="str">
-        <x:f>IF($N192="","",ROUNDDOWN($N192*$E192,3))</x:f>
+        <x:f>IF($N192="","",ROUNDDOWN(ROUNDDOWN($N192,2)*$E192,3))</x:f>
       </x:c>
       <x:c r="P192" s="77" t="str">
         <x:f>IF($L192="","",$I192*$L192)</x:f>
@@ -10990,10 +10990,10 @@
         <x:f>IF($L193="","",$C193*$L193)</x:f>
       </x:c>
       <x:c r="N193" s="86" t="str">
-        <x:f>IF($M193="","",$C193+$M193)</x:f>
+        <x:f>IF($M193="","",ROUNDDOWN($C193+$M193,2))</x:f>
       </x:c>
       <x:c r="O193" s="74" t="str">
-        <x:f>IF($N193="","",ROUNDDOWN($N193*$E193,3))</x:f>
+        <x:f>IF($N193="","",ROUNDDOWN(ROUNDDOWN($N193,2)*$E193,3))</x:f>
       </x:c>
       <x:c r="P193" s="77" t="str">
         <x:f>IF($L193="","",$I193*$L193)</x:f>
@@ -11043,10 +11043,10 @@
         <x:f>IF($L194="","",$C194*$L194)</x:f>
       </x:c>
       <x:c r="N194" s="86" t="str">
-        <x:f>IF($M194="","",$C194+$M194)</x:f>
+        <x:f>IF($M194="","",ROUNDDOWN($C194+$M194,2))</x:f>
       </x:c>
       <x:c r="O194" s="74" t="str">
-        <x:f>IF($N194="","",ROUNDDOWN($N194*$E194,3))</x:f>
+        <x:f>IF($N194="","",ROUNDDOWN(ROUNDDOWN($N194,2)*$E194,3))</x:f>
       </x:c>
       <x:c r="P194" s="77" t="str">
         <x:f>IF($L194="","",$I194*$L194)</x:f>
@@ -11096,10 +11096,10 @@
         <x:f>IF($L195="","",$C195*$L195)</x:f>
       </x:c>
       <x:c r="N195" s="86" t="str">
-        <x:f>IF($M195="","",$C195+$M195)</x:f>
+        <x:f>IF($M195="","",ROUNDDOWN($C195+$M195,2))</x:f>
       </x:c>
       <x:c r="O195" s="74" t="str">
-        <x:f>IF($N195="","",ROUNDDOWN($N195*$E195,3))</x:f>
+        <x:f>IF($N195="","",ROUNDDOWN(ROUNDDOWN($N195,2)*$E195,3))</x:f>
       </x:c>
       <x:c r="P195" s="77" t="str">
         <x:f>IF($L195="","",$I195*$L195)</x:f>
@@ -11149,10 +11149,10 @@
         <x:f>IF($L196="","",$C196*$L196)</x:f>
       </x:c>
       <x:c r="N196" s="86" t="str">
-        <x:f>IF($M196="","",$C196+$M196)</x:f>
+        <x:f>IF($M196="","",ROUNDDOWN($C196+$M196,2))</x:f>
       </x:c>
       <x:c r="O196" s="74" t="str">
-        <x:f>IF($N196="","",ROUNDDOWN($N196*$E196,3))</x:f>
+        <x:f>IF($N196="","",ROUNDDOWN(ROUNDDOWN($N196,2)*$E196,3))</x:f>
       </x:c>
       <x:c r="P196" s="77" t="str">
         <x:f>IF($L196="","",$I196*$L196)</x:f>
@@ -11202,10 +11202,10 @@
         <x:f>IF($L197="","",$C197*$L197)</x:f>
       </x:c>
       <x:c r="N197" s="86" t="str">
-        <x:f>IF($M197="","",$C197+$M197)</x:f>
+        <x:f>IF($M197="","",ROUNDDOWN($C197+$M197,2))</x:f>
       </x:c>
       <x:c r="O197" s="74" t="str">
-        <x:f>IF($N197="","",ROUNDDOWN($N197*$E197,3))</x:f>
+        <x:f>IF($N197="","",ROUNDDOWN(ROUNDDOWN($N197,2)*$E197,3))</x:f>
       </x:c>
       <x:c r="P197" s="77" t="str">
         <x:f>IF($L197="","",$I197*$L197)</x:f>
@@ -11255,10 +11255,10 @@
         <x:f>IF($L198="","",$C198*$L198)</x:f>
       </x:c>
       <x:c r="N198" s="86" t="str">
-        <x:f>IF($M198="","",$C198+$M198)</x:f>
+        <x:f>IF($M198="","",ROUNDDOWN($C198+$M198,2))</x:f>
       </x:c>
       <x:c r="O198" s="74" t="str">
-        <x:f>IF($N198="","",ROUNDDOWN($N198*$E198,3))</x:f>
+        <x:f>IF($N198="","",ROUNDDOWN(ROUNDDOWN($N198,2)*$E198,3))</x:f>
       </x:c>
       <x:c r="P198" s="77" t="str">
         <x:f>IF($L198="","",$I198*$L198)</x:f>
@@ -11308,10 +11308,10 @@
         <x:f>IF($L199="","",$C199*$L199)</x:f>
       </x:c>
       <x:c r="N199" s="86" t="str">
-        <x:f>IF($M199="","",$C199+$M199)</x:f>
+        <x:f>IF($M199="","",ROUNDDOWN($C199+$M199,2))</x:f>
       </x:c>
       <x:c r="O199" s="74" t="str">
-        <x:f>IF($N199="","",ROUNDDOWN($N199*$E199,3))</x:f>
+        <x:f>IF($N199="","",ROUNDDOWN(ROUNDDOWN($N199,2)*$E199,3))</x:f>
       </x:c>
       <x:c r="P199" s="77" t="str">
         <x:f>IF($L199="","",$I199*$L199)</x:f>
@@ -11361,10 +11361,10 @@
         <x:f>IF($L200="","",$C200*$L200)</x:f>
       </x:c>
       <x:c r="N200" s="86" t="str">
-        <x:f>IF($M200="","",$C200+$M200)</x:f>
+        <x:f>IF($M200="","",ROUNDDOWN($C200+$M200,2))</x:f>
       </x:c>
       <x:c r="O200" s="74" t="str">
-        <x:f>IF($N200="","",ROUNDDOWN($N200*$E200,3))</x:f>
+        <x:f>IF($N200="","",ROUNDDOWN(ROUNDDOWN($N200,2)*$E200,3))</x:f>
       </x:c>
       <x:c r="P200" s="77" t="str">
         <x:f>IF($L200="","",$I200*$L200)</x:f>
@@ -11414,10 +11414,10 @@
         <x:f>IF($L201="","",$C201*$L201)</x:f>
       </x:c>
       <x:c r="N201" s="86" t="str">
-        <x:f>IF($M201="","",$C201+$M201)</x:f>
+        <x:f>IF($M201="","",ROUNDDOWN($C201+$M201,2))</x:f>
       </x:c>
       <x:c r="O201" s="74" t="str">
-        <x:f>IF($N201="","",ROUNDDOWN($N201*$E201,3))</x:f>
+        <x:f>IF($N201="","",ROUNDDOWN(ROUNDDOWN($N201,2)*$E201,3))</x:f>
       </x:c>
       <x:c r="P201" s="77" t="str">
         <x:f>IF($L201="","",$I201*$L201)</x:f>
@@ -11467,10 +11467,10 @@
         <x:f>IF($L202="","",$C202*$L202)</x:f>
       </x:c>
       <x:c r="N202" s="86" t="str">
-        <x:f>IF($M202="","",$C202+$M202)</x:f>
+        <x:f>IF($M202="","",ROUNDDOWN($C202+$M202,2))</x:f>
       </x:c>
       <x:c r="O202" s="74" t="str">
-        <x:f>IF($N202="","",ROUNDDOWN($N202*$E202,3))</x:f>
+        <x:f>IF($N202="","",ROUNDDOWN(ROUNDDOWN($N202,2)*$E202,3))</x:f>
       </x:c>
       <x:c r="P202" s="77" t="str">
         <x:f>IF($L202="","",$I202*$L202)</x:f>
@@ -11520,10 +11520,10 @@
         <x:f>IF($L203="","",$C203*$L203)</x:f>
       </x:c>
       <x:c r="N203" s="86" t="str">
-        <x:f>IF($M203="","",$C203+$M203)</x:f>
+        <x:f>IF($M203="","",ROUNDDOWN($C203+$M203,2))</x:f>
       </x:c>
       <x:c r="O203" s="74" t="str">
-        <x:f>IF($N203="","",ROUNDDOWN($N203*$E203,3))</x:f>
+        <x:f>IF($N203="","",ROUNDDOWN(ROUNDDOWN($N203,2)*$E203,3))</x:f>
       </x:c>
       <x:c r="P203" s="77" t="str">
         <x:f>IF($L203="","",$I203*$L203)</x:f>
@@ -11573,10 +11573,10 @@
         <x:f>IF($L204="","",$C204*$L204)</x:f>
       </x:c>
       <x:c r="N204" s="86" t="str">
-        <x:f>IF($M204="","",$C204+$M204)</x:f>
+        <x:f>IF($M204="","",ROUNDDOWN($C204+$M204,2))</x:f>
       </x:c>
       <x:c r="O204" s="74" t="str">
-        <x:f>IF($N204="","",ROUNDDOWN($N204*$E204,3))</x:f>
+        <x:f>IF($N204="","",ROUNDDOWN(ROUNDDOWN($N204,2)*$E204,3))</x:f>
       </x:c>
       <x:c r="P204" s="77" t="str">
         <x:f>IF($L204="","",$I204*$L204)</x:f>
@@ -11626,10 +11626,10 @@
         <x:f>IF($L205="","",$C205*$L205)</x:f>
       </x:c>
       <x:c r="N205" s="86" t="str">
-        <x:f>IF($M205="","",$C205+$M205)</x:f>
+        <x:f>IF($M205="","",ROUNDDOWN($C205+$M205,2))</x:f>
       </x:c>
       <x:c r="O205" s="74" t="str">
-        <x:f>IF($N205="","",ROUNDDOWN($N205*$E205,3))</x:f>
+        <x:f>IF($N205="","",ROUNDDOWN(ROUNDDOWN($N205,2)*$E205,3))</x:f>
       </x:c>
       <x:c r="P205" s="77" t="str">
         <x:f>IF($L205="","",$I205*$L205)</x:f>
@@ -11679,10 +11679,10 @@
         <x:f>IF($L206="","",$C206*$L206)</x:f>
       </x:c>
       <x:c r="N206" s="86" t="str">
-        <x:f>IF($M206="","",$C206+$M206)</x:f>
+        <x:f>IF($M206="","",ROUNDDOWN($C206+$M206,2))</x:f>
       </x:c>
       <x:c r="O206" s="74" t="str">
-        <x:f>IF($N206="","",ROUNDDOWN($N206*$E206,3))</x:f>
+        <x:f>IF($N206="","",ROUNDDOWN(ROUNDDOWN($N206,2)*$E206,3))</x:f>
       </x:c>
       <x:c r="P206" s="77" t="str">
         <x:f>IF($L206="","",$I206*$L206)</x:f>
@@ -11732,10 +11732,10 @@
         <x:f>IF($L207="","",$C207*$L207)</x:f>
       </x:c>
       <x:c r="N207" s="86" t="str">
-        <x:f>IF($M207="","",$C207+$M207)</x:f>
+        <x:f>IF($M207="","",ROUNDDOWN($C207+$M207,2))</x:f>
       </x:c>
       <x:c r="O207" s="74" t="str">
-        <x:f>IF($N207="","",ROUNDDOWN($N207*$E207,3))</x:f>
+        <x:f>IF($N207="","",ROUNDDOWN(ROUNDDOWN($N207,2)*$E207,3))</x:f>
       </x:c>
       <x:c r="P207" s="77" t="str">
         <x:f>IF($L207="","",$I207*$L207)</x:f>
@@ -11785,10 +11785,10 @@
         <x:f>IF($L208="","",$C208*$L208)</x:f>
       </x:c>
       <x:c r="N208" s="86" t="str">
-        <x:f>IF($M208="","",$C208+$M208)</x:f>
+        <x:f>IF($M208="","",ROUNDDOWN($C208+$M208,2))</x:f>
       </x:c>
       <x:c r="O208" s="74" t="str">
-        <x:f>IF($N208="","",ROUNDDOWN($N208*$E208,3))</x:f>
+        <x:f>IF($N208="","",ROUNDDOWN(ROUNDDOWN($N208,2)*$E208,3))</x:f>
       </x:c>
       <x:c r="P208" s="77" t="str">
         <x:f>IF($L208="","",$I208*$L208)</x:f>
@@ -11838,10 +11838,10 @@
         <x:f>IF($L209="","",$C209*$L209)</x:f>
       </x:c>
       <x:c r="N209" s="86" t="str">
-        <x:f>IF($M209="","",$C209+$M209)</x:f>
+        <x:f>IF($M209="","",ROUNDDOWN($C209+$M209,2))</x:f>
       </x:c>
       <x:c r="O209" s="74" t="str">
-        <x:f>IF($N209="","",ROUNDDOWN($N209*$E209,3))</x:f>
+        <x:f>IF($N209="","",ROUNDDOWN(ROUNDDOWN($N209,2)*$E209,3))</x:f>
       </x:c>
       <x:c r="P209" s="77" t="str">
         <x:f>IF($L209="","",$I209*$L209)</x:f>
@@ -11891,10 +11891,10 @@
         <x:f>IF($L210="","",$C210*$L210)</x:f>
       </x:c>
       <x:c r="N210" s="86" t="str">
-        <x:f>IF($M210="","",$C210+$M210)</x:f>
+        <x:f>IF($M210="","",ROUNDDOWN($C210+$M210,2))</x:f>
       </x:c>
       <x:c r="O210" s="74" t="str">
-        <x:f>IF($N210="","",ROUNDDOWN($N210*$E210,3))</x:f>
+        <x:f>IF($N210="","",ROUNDDOWN(ROUNDDOWN($N210,2)*$E210,3))</x:f>
       </x:c>
       <x:c r="P210" s="77" t="str">
         <x:f>IF($L210="","",$I210*$L210)</x:f>
@@ -11944,10 +11944,10 @@
         <x:f>IF($L211="","",$C211*$L211)</x:f>
       </x:c>
       <x:c r="N211" s="86" t="str">
-        <x:f>IF($M211="","",$C211+$M211)</x:f>
+        <x:f>IF($M211="","",ROUNDDOWN($C211+$M211,2))</x:f>
       </x:c>
       <x:c r="O211" s="74" t="str">
-        <x:f>IF($N211="","",ROUNDDOWN($N211*$E211,3))</x:f>
+        <x:f>IF($N211="","",ROUNDDOWN(ROUNDDOWN($N211,2)*$E211,3))</x:f>
       </x:c>
       <x:c r="P211" s="77" t="str">
         <x:f>IF($L211="","",$I211*$L211)</x:f>
@@ -11997,10 +11997,10 @@
         <x:f>IF($L212="","",$C212*$L212)</x:f>
       </x:c>
       <x:c r="N212" s="86" t="str">
-        <x:f>IF($M212="","",$C212+$M212)</x:f>
+        <x:f>IF($M212="","",ROUNDDOWN($C212+$M212,2))</x:f>
       </x:c>
       <x:c r="O212" s="74" t="str">
-        <x:f>IF($N212="","",ROUNDDOWN($N212*$E212,3))</x:f>
+        <x:f>IF($N212="","",ROUNDDOWN(ROUNDDOWN($N212,2)*$E212,3))</x:f>
       </x:c>
       <x:c r="P212" s="77" t="str">
         <x:f>IF($L212="","",$I212*$L212)</x:f>
@@ -12050,10 +12050,10 @@
         <x:f>IF($L213="","",$C213*$L213)</x:f>
       </x:c>
       <x:c r="N213" s="86" t="str">
-        <x:f>IF($M213="","",$C213+$M213)</x:f>
+        <x:f>IF($M213="","",ROUNDDOWN($C213+$M213,2))</x:f>
       </x:c>
       <x:c r="O213" s="74" t="str">
-        <x:f>IF($N213="","",ROUNDDOWN($N213*$E213,3))</x:f>
+        <x:f>IF($N213="","",ROUNDDOWN(ROUNDDOWN($N213,2)*$E213,3))</x:f>
       </x:c>
       <x:c r="P213" s="77" t="str">
         <x:f>IF($L213="","",$I213*$L213)</x:f>
@@ -12103,10 +12103,10 @@
         <x:f>IF($L214="","",$C214*$L214)</x:f>
       </x:c>
       <x:c r="N214" s="86" t="str">
-        <x:f>IF($M214="","",$C214+$M214)</x:f>
+        <x:f>IF($M214="","",ROUNDDOWN($C214+$M214,2))</x:f>
       </x:c>
       <x:c r="O214" s="74" t="str">
-        <x:f>IF($N214="","",ROUNDDOWN($N214*$E214,3))</x:f>
+        <x:f>IF($N214="","",ROUNDDOWN(ROUNDDOWN($N214,2)*$E214,3))</x:f>
       </x:c>
       <x:c r="P214" s="77" t="str">
         <x:f>IF($L214="","",$I214*$L214)</x:f>
@@ -12156,10 +12156,10 @@
         <x:f>IF($L215="","",$C215*$L215)</x:f>
       </x:c>
       <x:c r="N215" s="86" t="str">
-        <x:f>IF($M215="","",$C215+$M215)</x:f>
+        <x:f>IF($M215="","",ROUNDDOWN($C215+$M215,2))</x:f>
       </x:c>
       <x:c r="O215" s="74" t="str">
-        <x:f>IF($N215="","",ROUNDDOWN($N215*$E215,3))</x:f>
+        <x:f>IF($N215="","",ROUNDDOWN(ROUNDDOWN($N215,2)*$E215,3))</x:f>
       </x:c>
       <x:c r="P215" s="77" t="str">
         <x:f>IF($L215="","",$I215*$L215)</x:f>
@@ -12209,10 +12209,10 @@
         <x:f>IF($L216="","",$C216*$L216)</x:f>
       </x:c>
       <x:c r="N216" s="86" t="str">
-        <x:f>IF($M216="","",$C216+$M216)</x:f>
+        <x:f>IF($M216="","",ROUNDDOWN($C216+$M216,2))</x:f>
       </x:c>
       <x:c r="O216" s="74" t="str">
-        <x:f>IF($N216="","",ROUNDDOWN($N216*$E216,3))</x:f>
+        <x:f>IF($N216="","",ROUNDDOWN(ROUNDDOWN($N216,2)*$E216,3))</x:f>
       </x:c>
       <x:c r="P216" s="77" t="str">
         <x:f>IF($L216="","",$I216*$L216)</x:f>
@@ -12262,10 +12262,10 @@
         <x:f>IF($L217="","",$C217*$L217)</x:f>
       </x:c>
       <x:c r="N217" s="86" t="str">
-        <x:f>IF($M217="","",$C217+$M217)</x:f>
+        <x:f>IF($M217="","",ROUNDDOWN($C217+$M217,2))</x:f>
       </x:c>
       <x:c r="O217" s="74" t="str">
-        <x:f>IF($N217="","",ROUNDDOWN($N217*$E217,3))</x:f>
+        <x:f>IF($N217="","",ROUNDDOWN(ROUNDDOWN($N217,2)*$E217,3))</x:f>
       </x:c>
       <x:c r="P217" s="77" t="str">
         <x:f>IF($L217="","",$I217*$L217)</x:f>
@@ -12315,10 +12315,10 @@
         <x:f>IF($L218="","",$C218*$L218)</x:f>
       </x:c>
       <x:c r="N218" s="86" t="str">
-        <x:f>IF($M218="","",$C218+$M218)</x:f>
+        <x:f>IF($M218="","",ROUNDDOWN($C218+$M218,2))</x:f>
       </x:c>
       <x:c r="O218" s="74" t="str">
-        <x:f>IF($N218="","",ROUNDDOWN($N218*$E218,3))</x:f>
+        <x:f>IF($N218="","",ROUNDDOWN(ROUNDDOWN($N218,2)*$E218,3))</x:f>
       </x:c>
       <x:c r="P218" s="77" t="str">
         <x:f>IF($L218="","",$I218*$L218)</x:f>
@@ -12368,10 +12368,10 @@
         <x:f>IF($L219="","",$C219*$L219)</x:f>
       </x:c>
       <x:c r="N219" s="86" t="str">
-        <x:f>IF($M219="","",$C219+$M219)</x:f>
+        <x:f>IF($M219="","",ROUNDDOWN($C219+$M219,2))</x:f>
       </x:c>
       <x:c r="O219" s="74" t="str">
-        <x:f>IF($N219="","",ROUNDDOWN($N219*$E219,3))</x:f>
+        <x:f>IF($N219="","",ROUNDDOWN(ROUNDDOWN($N219,2)*$E219,3))</x:f>
       </x:c>
       <x:c r="P219" s="77" t="str">
         <x:f>IF($L219="","",$I219*$L219)</x:f>
@@ -12421,10 +12421,10 @@
         <x:f>IF($L220="","",$C220*$L220)</x:f>
       </x:c>
       <x:c r="N220" s="86" t="str">
-        <x:f>IF($M220="","",$C220+$M220)</x:f>
+        <x:f>IF($M220="","",ROUNDDOWN($C220+$M220,2))</x:f>
       </x:c>
       <x:c r="O220" s="74" t="str">
-        <x:f>IF($N220="","",ROUNDDOWN($N220*$E220,3))</x:f>
+        <x:f>IF($N220="","",ROUNDDOWN(ROUNDDOWN($N220,2)*$E220,3))</x:f>
       </x:c>
       <x:c r="P220" s="77" t="str">
         <x:f>IF($L220="","",$I220*$L220)</x:f>
@@ -12474,10 +12474,10 @@
         <x:f>IF($L221="","",$C221*$L221)</x:f>
       </x:c>
       <x:c r="N221" s="86" t="str">
-        <x:f>IF($M221="","",$C221+$M221)</x:f>
+        <x:f>IF($M221="","",ROUNDDOWN($C221+$M221,2))</x:f>
       </x:c>
       <x:c r="O221" s="74" t="str">
-        <x:f>IF($N221="","",ROUNDDOWN($N221*$E221,3))</x:f>
+        <x:f>IF($N221="","",ROUNDDOWN(ROUNDDOWN($N221,2)*$E221,3))</x:f>
       </x:c>
       <x:c r="P221" s="77" t="str">
         <x:f>IF($L221="","",$I221*$L221)</x:f>
@@ -12527,10 +12527,10 @@
         <x:f>IF($L222="","",$C222*$L222)</x:f>
       </x:c>
       <x:c r="N222" s="86" t="str">
-        <x:f>IF($M222="","",$C222+$M222)</x:f>
+        <x:f>IF($M222="","",ROUNDDOWN($C222+$M222,2))</x:f>
       </x:c>
       <x:c r="O222" s="74" t="str">
-        <x:f>IF($N222="","",ROUNDDOWN($N222*$E222,3))</x:f>
+        <x:f>IF($N222="","",ROUNDDOWN(ROUNDDOWN($N222,2)*$E222,3))</x:f>
       </x:c>
       <x:c r="P222" s="77" t="str">
         <x:f>IF($L222="","",$I222*$L222)</x:f>
@@ -12580,10 +12580,10 @@
         <x:f>IF($L223="","",$C223*$L223)</x:f>
       </x:c>
       <x:c r="N223" s="86" t="str">
-        <x:f>IF($M223="","",$C223+$M223)</x:f>
+        <x:f>IF($M223="","",ROUNDDOWN($C223+$M223,2))</x:f>
       </x:c>
       <x:c r="O223" s="74" t="str">
-        <x:f>IF($N223="","",ROUNDDOWN($N223*$E223,3))</x:f>
+        <x:f>IF($N223="","",ROUNDDOWN(ROUNDDOWN($N223,2)*$E223,3))</x:f>
       </x:c>
       <x:c r="P223" s="77" t="str">
         <x:f>IF($L223="","",$I223*$L223)</x:f>
@@ -12633,10 +12633,10 @@
         <x:f>IF($L224="","",$C224*$L224)</x:f>
       </x:c>
       <x:c r="N224" s="86" t="str">
-        <x:f>IF($M224="","",$C224+$M224)</x:f>
+        <x:f>IF($M224="","",ROUNDDOWN($C224+$M224,2))</x:f>
       </x:c>
       <x:c r="O224" s="74" t="str">
-        <x:f>IF($N224="","",ROUNDDOWN($N224*$E224,3))</x:f>
+        <x:f>IF($N224="","",ROUNDDOWN(ROUNDDOWN($N224,2)*$E224,3))</x:f>
       </x:c>
       <x:c r="P224" s="77" t="str">
         <x:f>IF($L224="","",$I224*$L224)</x:f>
@@ -12686,10 +12686,10 @@
         <x:f>IF($L225="","",$C225*$L225)</x:f>
       </x:c>
       <x:c r="N225" s="86" t="str">
-        <x:f>IF($M225="","",$C225+$M225)</x:f>
+        <x:f>IF($M225="","",ROUNDDOWN($C225+$M225,2))</x:f>
       </x:c>
       <x:c r="O225" s="74" t="str">
-        <x:f>IF($N225="","",ROUNDDOWN($N225*$E225,3))</x:f>
+        <x:f>IF($N225="","",ROUNDDOWN(ROUNDDOWN($N225,2)*$E225,3))</x:f>
       </x:c>
       <x:c r="P225" s="77" t="str">
         <x:f>IF($L225="","",$I225*$L225)</x:f>
@@ -12739,10 +12739,10 @@
         <x:f>IF($L226="","",$C226*$L226)</x:f>
       </x:c>
       <x:c r="N226" s="86" t="str">
-        <x:f>IF($M226="","",$C226+$M226)</x:f>
+        <x:f>IF($M226="","",ROUNDDOWN($C226+$M226,2))</x:f>
       </x:c>
       <x:c r="O226" s="74" t="str">
-        <x:f>IF($N226="","",ROUNDDOWN($N226*$E226,3))</x:f>
+        <x:f>IF($N226="","",ROUNDDOWN(ROUNDDOWN($N226,2)*$E226,3))</x:f>
       </x:c>
       <x:c r="P226" s="77" t="str">
         <x:f>IF($L226="","",$I226*$L226)</x:f>
@@ -12792,10 +12792,10 @@
         <x:f>IF($L227="","",$C227*$L227)</x:f>
       </x:c>
       <x:c r="N227" s="86" t="str">
-        <x:f>IF($M227="","",$C227+$M227)</x:f>
+        <x:f>IF($M227="","",ROUNDDOWN($C227+$M227,2))</x:f>
       </x:c>
       <x:c r="O227" s="74" t="str">
-        <x:f>IF($N227="","",ROUNDDOWN($N227*$E227,3))</x:f>
+        <x:f>IF($N227="","",ROUNDDOWN(ROUNDDOWN($N227,2)*$E227,3))</x:f>
       </x:c>
       <x:c r="P227" s="77" t="str">
         <x:f>IF($L227="","",$I227*$L227)</x:f>
@@ -12845,10 +12845,10 @@
         <x:f>IF($L228="","",$C228*$L228)</x:f>
       </x:c>
       <x:c r="N228" s="86" t="str">
-        <x:f>IF($M228="","",$C228+$M228)</x:f>
+        <x:f>IF($M228="","",ROUNDDOWN($C228+$M228,2))</x:f>
       </x:c>
       <x:c r="O228" s="74" t="str">
-        <x:f>IF($N228="","",ROUNDDOWN($N228*$E228,3))</x:f>
+        <x:f>IF($N228="","",ROUNDDOWN(ROUNDDOWN($N228,2)*$E228,3))</x:f>
       </x:c>
       <x:c r="P228" s="77" t="str">
         <x:f>IF($L228="","",$I228*$L228)</x:f>
@@ -12898,10 +12898,10 @@
         <x:f>IF($L229="","",$C229*$L229)</x:f>
       </x:c>
       <x:c r="N229" s="86" t="str">
-        <x:f>IF($M229="","",$C229+$M229)</x:f>
+        <x:f>IF($M229="","",ROUNDDOWN($C229+$M229,2))</x:f>
       </x:c>
       <x:c r="O229" s="74" t="str">
-        <x:f>IF($N229="","",ROUNDDOWN($N229*$E229,3))</x:f>
+        <x:f>IF($N229="","",ROUNDDOWN(ROUNDDOWN($N229,2)*$E229,3))</x:f>
       </x:c>
       <x:c r="P229" s="77" t="str">
         <x:f>IF($L229="","",$I229*$L229)</x:f>
@@ -12951,10 +12951,10 @@
         <x:f>IF($L230="","",$C230*$L230)</x:f>
       </x:c>
       <x:c r="N230" s="86" t="str">
-        <x:f>IF($M230="","",$C230+$M230)</x:f>
+        <x:f>IF($M230="","",ROUNDDOWN($C230+$M230,2))</x:f>
       </x:c>
       <x:c r="O230" s="74" t="str">
-        <x:f>IF($N230="","",ROUNDDOWN($N230*$E230,3))</x:f>
+        <x:f>IF($N230="","",ROUNDDOWN(ROUNDDOWN($N230,2)*$E230,3))</x:f>
       </x:c>
       <x:c r="P230" s="77" t="str">
         <x:f>IF($L230="","",$I230*$L230)</x:f>
@@ -13004,10 +13004,10 @@
         <x:f>IF($L231="","",$C231*$L231)</x:f>
       </x:c>
       <x:c r="N231" s="86" t="str">
-        <x:f>IF($M231="","",$C231+$M231)</x:f>
+        <x:f>IF($M231="","",ROUNDDOWN($C231+$M231,2))</x:f>
       </x:c>
       <x:c r="O231" s="74" t="str">
-        <x:f>IF($N231="","",ROUNDDOWN($N231*$E231,3))</x:f>
+        <x:f>IF($N231="","",ROUNDDOWN(ROUNDDOWN($N231,2)*$E231,3))</x:f>
       </x:c>
       <x:c r="P231" s="77" t="str">
         <x:f>IF($L231="","",$I231*$L231)</x:f>
@@ -13057,10 +13057,10 @@
         <x:f>IF($L232="","",$C232*$L232)</x:f>
       </x:c>
       <x:c r="N232" s="86" t="str">
-        <x:f>IF($M232="","",$C232+$M232)</x:f>
+        <x:f>IF($M232="","",ROUNDDOWN($C232+$M232,2))</x:f>
       </x:c>
       <x:c r="O232" s="74" t="str">
-        <x:f>IF($N232="","",ROUNDDOWN($N232*$E232,3))</x:f>
+        <x:f>IF($N232="","",ROUNDDOWN(ROUNDDOWN($N232,2)*$E232,3))</x:f>
       </x:c>
       <x:c r="P232" s="77" t="str">
         <x:f>IF($L232="","",$I232*$L232)</x:f>
@@ -13110,10 +13110,10 @@
         <x:f>IF($L233="","",$C233*$L233)</x:f>
       </x:c>
       <x:c r="N233" s="86" t="str">
-        <x:f>IF($M233="","",$C233+$M233)</x:f>
+        <x:f>IF($M233="","",ROUNDDOWN($C233+$M233,2))</x:f>
       </x:c>
       <x:c r="O233" s="74" t="str">
-        <x:f>IF($N233="","",ROUNDDOWN($N233*$E233,3))</x:f>
+        <x:f>IF($N233="","",ROUNDDOWN(ROUNDDOWN($N233,2)*$E233,3))</x:f>
       </x:c>
       <x:c r="P233" s="77" t="str">
         <x:f>IF($L233="","",$I233*$L233)</x:f>
@@ -13163,10 +13163,10 @@
         <x:f>IF($L234="","",$C234*$L234)</x:f>
       </x:c>
       <x:c r="N234" s="86" t="str">
-        <x:f>IF($M234="","",$C234+$M234)</x:f>
+        <x:f>IF($M234="","",ROUNDDOWN($C234+$M234,2))</x:f>
       </x:c>
       <x:c r="O234" s="74" t="str">
-        <x:f>IF($N234="","",ROUNDDOWN($N234*$E234,3))</x:f>
+        <x:f>IF($N234="","",ROUNDDOWN(ROUNDDOWN($N234,2)*$E234,3))</x:f>
       </x:c>
       <x:c r="P234" s="77" t="str">
         <x:f>IF($L234="","",$I234*$L234)</x:f>
@@ -13216,10 +13216,10 @@
         <x:f>IF($L235="","",$C235*$L235)</x:f>
       </x:c>
       <x:c r="N235" s="86" t="str">
-        <x:f>IF($M235="","",$C235+$M235)</x:f>
+        <x:f>IF($M235="","",ROUNDDOWN($C235+$M235,2))</x:f>
       </x:c>
       <x:c r="O235" s="74" t="str">
-        <x:f>IF($N235="","",ROUNDDOWN($N235*$E235,3))</x:f>
+        <x:f>IF($N235="","",ROUNDDOWN(ROUNDDOWN($N235,2)*$E235,3))</x:f>
       </x:c>
       <x:c r="P235" s="77" t="str">
         <x:f>IF($L235="","",$I235*$L235)</x:f>
@@ -13269,10 +13269,10 @@
         <x:f>IF($L236="","",$C236*$L236)</x:f>
       </x:c>
       <x:c r="N236" s="86" t="str">
-        <x:f>IF($M236="","",$C236+$M236)</x:f>
+        <x:f>IF($M236="","",ROUNDDOWN($C236+$M236,2))</x:f>
       </x:c>
       <x:c r="O236" s="74" t="str">
-        <x:f>IF($N236="","",ROUNDDOWN($N236*$E236,3))</x:f>
+        <x:f>IF($N236="","",ROUNDDOWN(ROUNDDOWN($N236,2)*$E236,3))</x:f>
       </x:c>
       <x:c r="P236" s="77" t="str">
         <x:f>IF($L236="","",$I236*$L236)</x:f>
@@ -13322,10 +13322,10 @@
         <x:f>IF($L237="","",$C237*$L237)</x:f>
       </x:c>
       <x:c r="N237" s="86" t="str">
-        <x:f>IF($M237="","",$C237+$M237)</x:f>
+        <x:f>IF($M237="","",ROUNDDOWN($C237+$M237,2))</x:f>
       </x:c>
       <x:c r="O237" s="74" t="str">
-        <x:f>IF($N237="","",ROUNDDOWN($N237*$E237,3))</x:f>
+        <x:f>IF($N237="","",ROUNDDOWN(ROUNDDOWN($N237,2)*$E237,3))</x:f>
       </x:c>
       <x:c r="P237" s="77" t="str">
         <x:f>IF($L237="","",$I237*$L237)</x:f>
@@ -13375,10 +13375,10 @@
         <x:f>IF($L238="","",$C238*$L238)</x:f>
       </x:c>
       <x:c r="N238" s="86" t="str">
-        <x:f>IF($M238="","",$C238+$M238)</x:f>
+        <x:f>IF($M238="","",ROUNDDOWN($C238+$M238,2))</x:f>
       </x:c>
       <x:c r="O238" s="74" t="str">
-        <x:f>IF($N238="","",ROUNDDOWN($N238*$E238,3))</x:f>
+        <x:f>IF($N238="","",ROUNDDOWN(ROUNDDOWN($N238,2)*$E238,3))</x:f>
       </x:c>
       <x:c r="P238" s="77" t="str">
         <x:f>IF($L238="","",$I238*$L238)</x:f>
@@ -13428,10 +13428,10 @@
         <x:f>IF($L239="","",$C239*$L239)</x:f>
       </x:c>
       <x:c r="N239" s="86" t="str">
-        <x:f>IF($M239="","",$C239+$M239)</x:f>
+        <x:f>IF($M239="","",ROUNDDOWN($C239+$M239,2))</x:f>
       </x:c>
       <x:c r="O239" s="74" t="str">
-        <x:f>IF($N239="","",ROUNDDOWN($N239*$E239,3))</x:f>
+        <x:f>IF($N239="","",ROUNDDOWN(ROUNDDOWN($N239,2)*$E239,3))</x:f>
       </x:c>
       <x:c r="P239" s="77" t="str">
         <x:f>IF($L239="","",$I239*$L239)</x:f>
@@ -13481,10 +13481,10 @@
         <x:f>IF($L240="","",$C240*$L240)</x:f>
       </x:c>
       <x:c r="N240" s="86" t="str">
-        <x:f>IF($M240="","",$C240+$M240)</x:f>
+        <x:f>IF($M240="","",ROUNDDOWN($C240+$M240,2))</x:f>
       </x:c>
       <x:c r="O240" s="74" t="str">
-        <x:f>IF($N240="","",ROUNDDOWN($N240*$E240,3))</x:f>
+        <x:f>IF($N240="","",ROUNDDOWN(ROUNDDOWN($N240,2)*$E240,3))</x:f>
       </x:c>
       <x:c r="P240" s="77" t="str">
         <x:f>IF($L240="","",$I240*$L240)</x:f>
@@ -13534,10 +13534,10 @@
         <x:f>IF($L241="","",$C241*$L241)</x:f>
       </x:c>
       <x:c r="N241" s="86" t="str">
-        <x:f>IF($M241="","",$C241+$M241)</x:f>
+        <x:f>IF($M241="","",ROUNDDOWN($C241+$M241,2))</x:f>
       </x:c>
       <x:c r="O241" s="74" t="str">
-        <x:f>IF($N241="","",ROUNDDOWN($N241*$E241,3))</x:f>
+        <x:f>IF($N241="","",ROUNDDOWN(ROUNDDOWN($N241,2)*$E241,3))</x:f>
       </x:c>
       <x:c r="P241" s="77" t="str">
         <x:f>IF($L241="","",$I241*$L241)</x:f>
@@ -13587,10 +13587,10 @@
         <x:f>IF($L242="","",$C242*$L242)</x:f>
       </x:c>
       <x:c r="N242" s="86" t="str">
-        <x:f>IF($M242="","",$C242+$M242)</x:f>
+        <x:f>IF($M242="","",ROUNDDOWN($C242+$M242,2))</x:f>
       </x:c>
       <x:c r="O242" s="74" t="str">
-        <x:f>IF($N242="","",ROUNDDOWN($N242*$E242,3))</x:f>
+        <x:f>IF($N242="","",ROUNDDOWN(ROUNDDOWN($N242,2)*$E242,3))</x:f>
       </x:c>
       <x:c r="P242" s="77" t="str">
         <x:f>IF($L242="","",$I242*$L242)</x:f>
@@ -13640,10 +13640,10 @@
         <x:f>IF($L243="","",$C243*$L243)</x:f>
       </x:c>
       <x:c r="N243" s="86" t="str">
-        <x:f>IF($M243="","",$C243+$M243)</x:f>
+        <x:f>IF($M243="","",ROUNDDOWN($C243+$M243,2))</x:f>
       </x:c>
       <x:c r="O243" s="74" t="str">
-        <x:f>IF($N243="","",ROUNDDOWN($N243*$E243,3))</x:f>
+        <x:f>IF($N243="","",ROUNDDOWN(ROUNDDOWN($N243,2)*$E243,3))</x:f>
       </x:c>
       <x:c r="P243" s="77" t="str">
         <x:f>IF($L243="","",$I243*$L243)</x:f>
@@ -13693,10 +13693,10 @@
         <x:f>IF($L244="","",$C244*$L244)</x:f>
       </x:c>
       <x:c r="N244" s="86" t="str">
-        <x:f>IF($M244="","",$C244+$M244)</x:f>
+        <x:f>IF($M244="","",ROUNDDOWN($C244+$M244,2))</x:f>
       </x:c>
       <x:c r="O244" s="74" t="str">
-        <x:f>IF($N244="","",ROUNDDOWN($N244*$E244,3))</x:f>
+        <x:f>IF($N244="","",ROUNDDOWN(ROUNDDOWN($N244,2)*$E244,3))</x:f>
       </x:c>
       <x:c r="P244" s="77" t="str">
         <x:f>IF($L244="","",$I244*$L244)</x:f>
@@ -13746,10 +13746,10 @@
         <x:f>IF($L245="","",$C245*$L245)</x:f>
       </x:c>
       <x:c r="N245" s="86" t="str">
-        <x:f>IF($M245="","",$C245+$M245)</x:f>
+        <x:f>IF($M245="","",ROUNDDOWN($C245+$M245,2))</x:f>
       </x:c>
       <x:c r="O245" s="74" t="str">
-        <x:f>IF($N245="","",ROUNDDOWN($N245*$E245,3))</x:f>
+        <x:f>IF($N245="","",ROUNDDOWN(ROUNDDOWN($N245,2)*$E245,3))</x:f>
       </x:c>
       <x:c r="P245" s="77" t="str">
         <x:f>IF($L245="","",$I245*$L245)</x:f>
@@ -13799,10 +13799,10 @@
         <x:f>IF($L246="","",$C246*$L246)</x:f>
       </x:c>
       <x:c r="N246" s="86" t="str">
-        <x:f>IF($M246="","",$C246+$M246)</x:f>
+        <x:f>IF($M246="","",ROUNDDOWN($C246+$M246,2))</x:f>
       </x:c>
       <x:c r="O246" s="74" t="str">
-        <x:f>IF($N246="","",ROUNDDOWN($N246*$E246,3))</x:f>
+        <x:f>IF($N246="","",ROUNDDOWN(ROUNDDOWN($N246,2)*$E246,3))</x:f>
       </x:c>
       <x:c r="P246" s="77" t="str">
         <x:f>IF($L246="","",$I246*$L246)</x:f>
@@ -13852,10 +13852,10 @@
         <x:f>IF($L247="","",$C247*$L247)</x:f>
       </x:c>
       <x:c r="N247" s="86" t="str">
-        <x:f>IF($M247="","",$C247+$M247)</x:f>
+        <x:f>IF($M247="","",ROUNDDOWN($C247+$M247,2))</x:f>
       </x:c>
       <x:c r="O247" s="74" t="str">
-        <x:f>IF($N247="","",ROUNDDOWN($N247*$E247,3))</x:f>
+        <x:f>IF($N247="","",ROUNDDOWN(ROUNDDOWN($N247,2)*$E247,3))</x:f>
       </x:c>
       <x:c r="P247" s="77" t="str">
         <x:f>IF($L247="","",$I247*$L247)</x:f>
@@ -13905,10 +13905,10 @@
         <x:f>IF($L248="","",$C248*$L248)</x:f>
       </x:c>
       <x:c r="N248" s="86" t="str">
-        <x:f>IF($M248="","",$C248+$M248)</x:f>
+        <x:f>IF($M248="","",ROUNDDOWN($C248+$M248,2))</x:f>
       </x:c>
       <x:c r="O248" s="74" t="str">
-        <x:f>IF($N248="","",ROUNDDOWN($N248*$E248,3))</x:f>
+        <x:f>IF($N248="","",ROUNDDOWN(ROUNDDOWN($N248,2)*$E248,3))</x:f>
       </x:c>
       <x:c r="P248" s="77" t="str">
         <x:f>IF($L248="","",$I248*$L248)</x:f>
@@ -13958,10 +13958,10 @@
         <x:f>IF($L249="","",$C249*$L249)</x:f>
       </x:c>
       <x:c r="N249" s="86" t="str">
-        <x:f>IF($M249="","",$C249+$M249)</x:f>
+        <x:f>IF($M249="","",ROUNDDOWN($C249+$M249,2))</x:f>
       </x:c>
       <x:c r="O249" s="74" t="str">
-        <x:f>IF($N249="","",ROUNDDOWN($N249*$E249,3))</x:f>
+        <x:f>IF($N249="","",ROUNDDOWN(ROUNDDOWN($N249,2)*$E249,3))</x:f>
       </x:c>
       <x:c r="P249" s="77" t="str">
         <x:f>IF($L249="","",$I249*$L249)</x:f>
@@ -14011,10 +14011,10 @@
         <x:f>IF($L250="","",$C250*$L250)</x:f>
       </x:c>
       <x:c r="N250" s="86" t="str">
-        <x:f>IF($M250="","",$C250+$M250)</x:f>
+        <x:f>IF($M250="","",ROUNDDOWN($C250+$M250,2))</x:f>
       </x:c>
       <x:c r="O250" s="74" t="str">
-        <x:f>IF($N250="","",ROUNDDOWN($N250*$E250,3))</x:f>
+        <x:f>IF($N250="","",ROUNDDOWN(ROUNDDOWN($N250,2)*$E250,3))</x:f>
       </x:c>
       <x:c r="P250" s="77" t="str">
         <x:f>IF($L250="","",$I250*$L250)</x:f>
@@ -14064,10 +14064,10 @@
         <x:f>IF($L251="","",$C251*$L251)</x:f>
       </x:c>
       <x:c r="N251" s="86" t="str">
-        <x:f>IF($M251="","",$C251+$M251)</x:f>
+        <x:f>IF($M251="","",ROUNDDOWN($C251+$M251,2))</x:f>
       </x:c>
       <x:c r="O251" s="74" t="str">
-        <x:f>IF($N251="","",ROUNDDOWN($N251*$E251,3))</x:f>
+        <x:f>IF($N251="","",ROUNDDOWN(ROUNDDOWN($N251,2)*$E251,3))</x:f>
       </x:c>
       <x:c r="P251" s="77" t="str">
         <x:f>IF($L251="","",$I251*$L251)</x:f>
@@ -14117,10 +14117,10 @@
         <x:f>IF($L252="","",$C252*$L252)</x:f>
       </x:c>
       <x:c r="N252" s="86" t="str">
-        <x:f>IF($M252="","",$C252+$M252)</x:f>
+        <x:f>IF($M252="","",ROUNDDOWN($C252+$M252,2))</x:f>
       </x:c>
       <x:c r="O252" s="74" t="str">
-        <x:f>IF($N252="","",ROUNDDOWN($N252*$E252,3))</x:f>
+        <x:f>IF($N252="","",ROUNDDOWN(ROUNDDOWN($N252,2)*$E252,3))</x:f>
       </x:c>
       <x:c r="P252" s="77" t="str">
         <x:f>IF($L252="","",$I252*$L252)</x:f>
@@ -14170,10 +14170,10 @@
         <x:f>IF($L253="","",$C253*$L253)</x:f>
       </x:c>
       <x:c r="N253" s="86" t="str">
-        <x:f>IF($M253="","",$C253+$M253)</x:f>
+        <x:f>IF($M253="","",ROUNDDOWN($C253+$M253,2))</x:f>
       </x:c>
       <x:c r="O253" s="74" t="str">
-        <x:f>IF($N253="","",ROUNDDOWN($N253*$E253,3))</x:f>
+        <x:f>IF($N253="","",ROUNDDOWN(ROUNDDOWN($N253,2)*$E253,3))</x:f>
       </x:c>
       <x:c r="P253" s="77" t="str">
         <x:f>IF($L253="","",$I253*$L253)</x:f>
@@ -14223,10 +14223,10 @@
         <x:f>IF($L254="","",$C254*$L254)</x:f>
       </x:c>
       <x:c r="N254" s="86" t="str">
-        <x:f>IF($M254="","",$C254+$M254)</x:f>
+        <x:f>IF($M254="","",ROUNDDOWN($C254+$M254,2))</x:f>
       </x:c>
       <x:c r="O254" s="74" t="str">
-        <x:f>IF($N254="","",ROUNDDOWN($N254*$E254,3))</x:f>
+        <x:f>IF($N254="","",ROUNDDOWN(ROUNDDOWN($N254,2)*$E254,3))</x:f>
       </x:c>
       <x:c r="P254" s="77" t="str">
         <x:f>IF($L254="","",$I254*$L254)</x:f>
@@ -14276,10 +14276,10 @@
         <x:f>IF($L255="","",$C255*$L255)</x:f>
       </x:c>
       <x:c r="N255" s="86" t="str">
-        <x:f>IF($M255="","",$C255+$M255)</x:f>
+        <x:f>IF($M255="","",ROUNDDOWN($C255+$M255,2))</x:f>
       </x:c>
       <x:c r="O255" s="74" t="str">
-        <x:f>IF($N255="","",ROUNDDOWN($N255*$E255,3))</x:f>
+        <x:f>IF($N255="","",ROUNDDOWN(ROUNDDOWN($N255,2)*$E255,3))</x:f>
       </x:c>
       <x:c r="P255" s="77" t="str">
         <x:f>IF($L255="","",$I255*$L255)</x:f>
@@ -14329,10 +14329,10 @@
         <x:f>IF($L256="","",$C256*$L256)</x:f>
       </x:c>
       <x:c r="N256" s="86" t="str">
-        <x:f>IF($M256="","",$C256+$M256)</x:f>
+        <x:f>IF($M256="","",ROUNDDOWN($C256+$M256,2))</x:f>
       </x:c>
       <x:c r="O256" s="74" t="str">
-        <x:f>IF($N256="","",ROUNDDOWN($N256*$E256,3))</x:f>
+        <x:f>IF($N256="","",ROUNDDOWN(ROUNDDOWN($N256,2)*$E256,3))</x:f>
       </x:c>
       <x:c r="P256" s="77" t="str">
         <x:f>IF($L256="","",$I256*$L256)</x:f>
@@ -14382,10 +14382,10 @@
         <x:f>IF($L257="","",$C257*$L257)</x:f>
       </x:c>
       <x:c r="N257" s="86" t="str">
-        <x:f>IF($M257="","",$C257+$M257)</x:f>
+        <x:f>IF($M257="","",ROUNDDOWN($C257+$M257,2))</x:f>
       </x:c>
       <x:c r="O257" s="74" t="str">
-        <x:f>IF($N257="","",ROUNDDOWN($N257*$E257,3))</x:f>
+        <x:f>IF($N257="","",ROUNDDOWN(ROUNDDOWN($N257,2)*$E257,3))</x:f>
       </x:c>
       <x:c r="P257" s="77" t="str">
         <x:f>IF($L257="","",$I257*$L257)</x:f>
@@ -14435,10 +14435,10 @@
         <x:f>IF($L258="","",$C258*$L258)</x:f>
       </x:c>
       <x:c r="N258" s="86" t="str">
-        <x:f>IF($M258="","",$C258+$M258)</x:f>
+        <x:f>IF($M258="","",ROUNDDOWN($C258+$M258,2))</x:f>
       </x:c>
       <x:c r="O258" s="74" t="str">
-        <x:f>IF($N258="","",ROUNDDOWN($N258*$E258,3))</x:f>
+        <x:f>IF($N258="","",ROUNDDOWN(ROUNDDOWN($N258,2)*$E258,3))</x:f>
       </x:c>
       <x:c r="P258" s="77" t="str">
         <x:f>IF($L258="","",$I258*$L258)</x:f>
@@ -14488,10 +14488,10 @@
         <x:f>IF($L259="","",$C259*$L259)</x:f>
       </x:c>
       <x:c r="N259" s="86" t="str">
-        <x:f>IF($M259="","",$C259+$M259)</x:f>
+        <x:f>IF($M259="","",ROUNDDOWN($C259+$M259,2))</x:f>
       </x:c>
       <x:c r="O259" s="74" t="str">
-        <x:f>IF($N259="","",ROUNDDOWN($N259*$E259,3))</x:f>
+        <x:f>IF($N259="","",ROUNDDOWN(ROUNDDOWN($N259,2)*$E259,3))</x:f>
       </x:c>
       <x:c r="P259" s="77" t="str">
         <x:f>IF($L259="","",$I259*$L259)</x:f>
@@ -14541,10 +14541,10 @@
         <x:f>IF($L260="","",$C260*$L260)</x:f>
       </x:c>
       <x:c r="N260" s="86" t="str">
-        <x:f>IF($M260="","",$C260+$M260)</x:f>
+        <x:f>IF($M260="","",ROUNDDOWN($C260+$M260,2))</x:f>
       </x:c>
       <x:c r="O260" s="74" t="str">
-        <x:f>IF($N260="","",ROUNDDOWN($N260*$E260,3))</x:f>
+        <x:f>IF($N260="","",ROUNDDOWN(ROUNDDOWN($N260,2)*$E260,3))</x:f>
       </x:c>
       <x:c r="P260" s="77" t="str">
         <x:f>IF($L260="","",$I260*$L260)</x:f>
@@ -14594,10 +14594,10 @@
         <x:f>IF($L261="","",$C261*$L261)</x:f>
       </x:c>
       <x:c r="N261" s="86" t="str">
-        <x:f>IF($M261="","",$C261+$M261)</x:f>
+        <x:f>IF($M261="","",ROUNDDOWN($C261+$M261,2))</x:f>
       </x:c>
       <x:c r="O261" s="74" t="str">
-        <x:f>IF($N261="","",ROUNDDOWN($N261*$E261,3))</x:f>
+        <x:f>IF($N261="","",ROUNDDOWN(ROUNDDOWN($N261,2)*$E261,3))</x:f>
       </x:c>
       <x:c r="P261" s="77" t="str">
         <x:f>IF($L261="","",$I261*$L261)</x:f>
@@ -14647,10 +14647,10 @@
         <x:f>IF($L262="","",$C262*$L262)</x:f>
       </x:c>
       <x:c r="N262" s="86" t="str">
-        <x:f>IF($M262="","",$C262+$M262)</x:f>
+        <x:f>IF($M262="","",ROUNDDOWN($C262+$M262,2))</x:f>
       </x:c>
       <x:c r="O262" s="74" t="str">
-        <x:f>IF($N262="","",ROUNDDOWN($N262*$E262,3))</x:f>
+        <x:f>IF($N262="","",ROUNDDOWN(ROUNDDOWN($N262,2)*$E262,3))</x:f>
       </x:c>
       <x:c r="P262" s="77" t="str">
         <x:f>IF($L262="","",$I262*$L262)</x:f>
@@ -14700,10 +14700,10 @@
         <x:f>IF($L263="","",$C263*$L263)</x:f>
       </x:c>
       <x:c r="N263" s="86" t="str">
-        <x:f>IF($M263="","",$C263+$M263)</x:f>
+        <x:f>IF($M263="","",ROUNDDOWN($C263+$M263,2))</x:f>
       </x:c>
       <x:c r="O263" s="74" t="str">
-        <x:f>IF($N263="","",ROUNDDOWN($N263*$E263,3))</x:f>
+        <x:f>IF($N263="","",ROUNDDOWN(ROUNDDOWN($N263,2)*$E263,3))</x:f>
       </x:c>
       <x:c r="P263" s="77" t="str">
         <x:f>IF($L263="","",$I263*$L263)</x:f>
@@ -14753,10 +14753,10 @@
         <x:f>IF($L264="","",$C264*$L264)</x:f>
       </x:c>
       <x:c r="N264" s="86" t="str">
-        <x:f>IF($M264="","",$C264+$M264)</x:f>
+        <x:f>IF($M264="","",ROUNDDOWN($C264+$M264,2))</x:f>
       </x:c>
       <x:c r="O264" s="74" t="str">
-        <x:f>IF($N264="","",ROUNDDOWN($N264*$E264,3))</x:f>
+        <x:f>IF($N264="","",ROUNDDOWN(ROUNDDOWN($N264,2)*$E264,3))</x:f>
       </x:c>
       <x:c r="P264" s="77" t="str">
         <x:f>IF($L264="","",$I264*$L264)</x:f>
@@ -14806,10 +14806,10 @@
         <x:f>IF($L265="","",$C265*$L265)</x:f>
       </x:c>
       <x:c r="N265" s="86" t="str">
-        <x:f>IF($M265="","",$C265+$M265)</x:f>
+        <x:f>IF($M265="","",ROUNDDOWN($C265+$M265,2))</x:f>
       </x:c>
       <x:c r="O265" s="74" t="str">
-        <x:f>IF($N265="","",ROUNDDOWN($N265*$E265,3))</x:f>
+        <x:f>IF($N265="","",ROUNDDOWN(ROUNDDOWN($N265,2)*$E265,3))</x:f>
       </x:c>
       <x:c r="P265" s="77" t="str">
         <x:f>IF($L265="","",$I265*$L265)</x:f>
@@ -14859,10 +14859,10 @@
         <x:f>IF($L266="","",$C266*$L266)</x:f>
       </x:c>
       <x:c r="N266" s="86" t="str">
-        <x:f>IF($M266="","",$C266+$M266)</x:f>
+        <x:f>IF($M266="","",ROUNDDOWN($C266+$M266,2))</x:f>
       </x:c>
       <x:c r="O266" s="74" t="str">
-        <x:f>IF($N266="","",ROUNDDOWN($N266*$E266,3))</x:f>
+        <x:f>IF($N266="","",ROUNDDOWN(ROUNDDOWN($N266,2)*$E266,3))</x:f>
       </x:c>
       <x:c r="P266" s="77" t="str">
         <x:f>IF($L266="","",$I266*$L266)</x:f>
@@ -14912,10 +14912,10 @@
         <x:f>IF($L267="","",$C267*$L267)</x:f>
       </x:c>
       <x:c r="N267" s="86" t="str">
-        <x:f>IF($M267="","",$C267+$M267)</x:f>
+        <x:f>IF($M267="","",ROUNDDOWN($C267+$M267,2))</x:f>
       </x:c>
       <x:c r="O267" s="74" t="str">
-        <x:f>IF($N267="","",ROUNDDOWN($N267*$E267,3))</x:f>
+        <x:f>IF($N267="","",ROUNDDOWN(ROUNDDOWN($N267,2)*$E267,3))</x:f>
       </x:c>
       <x:c r="P267" s="77" t="str">
         <x:f>IF($L267="","",$I267*$L267)</x:f>
@@ -14965,10 +14965,10 @@
         <x:f>IF($L268="","",$C268*$L268)</x:f>
       </x:c>
       <x:c r="N268" s="86" t="str">
-        <x:f>IF($M268="","",$C268+$M268)</x:f>
+        <x:f>IF($M268="","",ROUNDDOWN($C268+$M268,2))</x:f>
       </x:c>
       <x:c r="O268" s="74" t="str">
-        <x:f>IF($N268="","",ROUNDDOWN($N268*$E268,3))</x:f>
+        <x:f>IF($N268="","",ROUNDDOWN(ROUNDDOWN($N268,2)*$E268,3))</x:f>
       </x:c>
       <x:c r="P268" s="77" t="str">
         <x:f>IF($L268="","",$I268*$L268)</x:f>
@@ -15018,10 +15018,10 @@
         <x:f>IF($L269="","",$C269*$L269)</x:f>
       </x:c>
       <x:c r="N269" s="86" t="str">
-        <x:f>IF($M269="","",$C269+$M269)</x:f>
+        <x:f>IF($M269="","",ROUNDDOWN($C269+$M269,2))</x:f>
       </x:c>
       <x:c r="O269" s="74" t="str">
-        <x:f>IF($N269="","",ROUNDDOWN($N269*$E269,3))</x:f>
+        <x:f>IF($N269="","",ROUNDDOWN(ROUNDDOWN($N269,2)*$E269,3))</x:f>
       </x:c>
       <x:c r="P269" s="77" t="str">
         <x:f>IF($L269="","",$I269*$L269)</x:f>
@@ -15071,10 +15071,10 @@
         <x:f>IF($L270="","",$C270*$L270)</x:f>
       </x:c>
       <x:c r="N270" s="86" t="str">
-        <x:f>IF($M270="","",$C270+$M270)</x:f>
+        <x:f>IF($M270="","",ROUNDDOWN($C270+$M270,2))</x:f>
       </x:c>
       <x:c r="O270" s="74" t="str">
-        <x:f>IF($N270="","",ROUNDDOWN($N270*$E270,3))</x:f>
+        <x:f>IF($N270="","",ROUNDDOWN(ROUNDDOWN($N270,2)*$E270,3))</x:f>
       </x:c>
       <x:c r="P270" s="77" t="str">
         <x:f>IF($L270="","",$I270*$L270)</x:f>
@@ -15124,10 +15124,10 @@
         <x:f>IF($L271="","",$C271*$L271)</x:f>
       </x:c>
       <x:c r="N271" s="86" t="str">
-        <x:f>IF($M271="","",$C271+$M271)</x:f>
+        <x:f>IF($M271="","",ROUNDDOWN($C271+$M271,2))</x:f>
       </x:c>
       <x:c r="O271" s="74" t="str">
-        <x:f>IF($N271="","",ROUNDDOWN($N271*$E271,3))</x:f>
+        <x:f>IF($N271="","",ROUNDDOWN(ROUNDDOWN($N271,2)*$E271,3))</x:f>
       </x:c>
       <x:c r="P271" s="77" t="str">
         <x:f>IF($L271="","",$I271*$L271)</x:f>
@@ -15177,10 +15177,10 @@
         <x:f>IF($L272="","",$C272*$L272)</x:f>
       </x:c>
       <x:c r="N272" s="86" t="str">
-        <x:f>IF($M272="","",$C272+$M272)</x:f>
+        <x:f>IF($M272="","",ROUNDDOWN($C272+$M272,2))</x:f>
       </x:c>
       <x:c r="O272" s="74" t="str">
-        <x:f>IF($N272="","",ROUNDDOWN($N272*$E272,3))</x:f>
+        <x:f>IF($N272="","",ROUNDDOWN(ROUNDDOWN($N272,2)*$E272,3))</x:f>
       </x:c>
       <x:c r="P272" s="77" t="str">
         <x:f>IF($L272="","",$I272*$L272)</x:f>
@@ -15230,10 +15230,10 @@
         <x:f>IF($L273="","",$C273*$L273)</x:f>
       </x:c>
       <x:c r="N273" s="86" t="str">
-        <x:f>IF($M273="","",$C273+$M273)</x:f>
+        <x:f>IF($M273="","",ROUNDDOWN($C273+$M273,2))</x:f>
       </x:c>
       <x:c r="O273" s="74" t="str">
-        <x:f>IF($N273="","",ROUNDDOWN($N273*$E273,3))</x:f>
+        <x:f>IF($N273="","",ROUNDDOWN(ROUNDDOWN($N273,2)*$E273,3))</x:f>
       </x:c>
       <x:c r="P273" s="77" t="str">
         <x:f>IF($L273="","",$I273*$L273)</x:f>
@@ -15283,10 +15283,10 @@
         <x:f>IF($L274="","",$C274*$L274)</x:f>
       </x:c>
       <x:c r="N274" s="86" t="str">
-        <x:f>IF($M274="","",$C274+$M274)</x:f>
+        <x:f>IF($M274="","",ROUNDDOWN($C274+$M274,2))</x:f>
       </x:c>
       <x:c r="O274" s="74" t="str">
-        <x:f>IF($N274="","",ROUNDDOWN($N274*$E274,3))</x:f>
+        <x:f>IF($N274="","",ROUNDDOWN(ROUNDDOWN($N274,2)*$E274,3))</x:f>
       </x:c>
       <x:c r="P274" s="77" t="str">
         <x:f>IF($L274="","",$I274*$L274)</x:f>
@@ -15336,10 +15336,10 @@
         <x:f>IF($L275="","",$C275*$L275)</x:f>
       </x:c>
       <x:c r="N275" s="86" t="str">
-        <x:f>IF($M275="","",$C275+$M275)</x:f>
+        <x:f>IF($M275="","",ROUNDDOWN($C275+$M275,2))</x:f>
       </x:c>
       <x:c r="O275" s="74" t="str">
-        <x:f>IF($N275="","",ROUNDDOWN($N275*$E275,3))</x:f>
+        <x:f>IF($N275="","",ROUNDDOWN(ROUNDDOWN($N275,2)*$E275,3))</x:f>
       </x:c>
       <x:c r="P275" s="77" t="str">
         <x:f>IF($L275="","",$I275*$L275)</x:f>
@@ -15389,10 +15389,10 @@
         <x:f>IF($L276="","",$C276*$L276)</x:f>
       </x:c>
       <x:c r="N276" s="86" t="str">
-        <x:f>IF($M276="","",$C276+$M276)</x:f>
+        <x:f>IF($M276="","",ROUNDDOWN($C276+$M276,2))</x:f>
       </x:c>
       <x:c r="O276" s="74" t="str">
-        <x:f>IF($N276="","",ROUNDDOWN($N276*$E276,3))</x:f>
+        <x:f>IF($N276="","",ROUNDDOWN(ROUNDDOWN($N276,2)*$E276,3))</x:f>
       </x:c>
       <x:c r="P276" s="77" t="str">
         <x:f>IF($L276="","",$I276*$L276)</x:f>
@@ -15442,10 +15442,10 @@
         <x:f>IF($L277="","",$C277*$L277)</x:f>
       </x:c>
       <x:c r="N277" s="86" t="str">
-        <x:f>IF($M277="","",$C277+$M277)</x:f>
+        <x:f>IF($M277="","",ROUNDDOWN($C277+$M277,2))</x:f>
       </x:c>
       <x:c r="O277" s="74" t="str">
-        <x:f>IF($N277="","",ROUNDDOWN($N277*$E277,3))</x:f>
+        <x:f>IF($N277="","",ROUNDDOWN(ROUNDDOWN($N277,2)*$E277,3))</x:f>
       </x:c>
       <x:c r="P277" s="77" t="str">
         <x:f>IF($L277="","",$I277*$L277)</x:f>
@@ -15495,10 +15495,10 @@
         <x:f>IF($L278="","",$C278*$L278)</x:f>
       </x:c>
       <x:c r="N278" s="86" t="str">
-        <x:f>IF($M278="","",$C278+$M278)</x:f>
+        <x:f>IF($M278="","",ROUNDDOWN($C278+$M278,2))</x:f>
       </x:c>
       <x:c r="O278" s="74" t="str">
-        <x:f>IF($N278="","",ROUNDDOWN($N278*$E278,3))</x:f>
+        <x:f>IF($N278="","",ROUNDDOWN(ROUNDDOWN($N278,2)*$E278,3))</x:f>
       </x:c>
       <x:c r="P278" s="77" t="str">
         <x:f>IF($L278="","",$I278*$L278)</x:f>
@@ -15548,10 +15548,10 @@
         <x:f>IF($L279="","",$C279*$L279)</x:f>
       </x:c>
       <x:c r="N279" s="86" t="str">
-        <x:f>IF($M279="","",$C279+$M279)</x:f>
+        <x:f>IF($M279="","",ROUNDDOWN($C279+$M279,2))</x:f>
       </x:c>
       <x:c r="O279" s="74" t="str">
-        <x:f>IF($N279="","",ROUNDDOWN($N279*$E279,3))</x:f>
+        <x:f>IF($N279="","",ROUNDDOWN(ROUNDDOWN($N279,2)*$E279,3))</x:f>
       </x:c>
       <x:c r="P279" s="77" t="str">
         <x:f>IF($L279="","",$I279*$L279)</x:f>
@@ -15601,10 +15601,10 @@
         <x:f>IF($L280="","",$C280*$L280)</x:f>
       </x:c>
       <x:c r="N280" s="86" t="str">
-        <x:f>IF($M280="","",$C280+$M280)</x:f>
+        <x:f>IF($M280="","",ROUNDDOWN($C280+$M280,2))</x:f>
       </x:c>
       <x:c r="O280" s="74" t="str">
-        <x:f>IF($N280="","",ROUNDDOWN($N280*$E280,3))</x:f>
+        <x:f>IF($N280="","",ROUNDDOWN(ROUNDDOWN($N280,2)*$E280,3))</x:f>
       </x:c>
       <x:c r="P280" s="77" t="str">
         <x:f>IF($L280="","",$I280*$L280)</x:f>
@@ -15654,10 +15654,10 @@
         <x:f>IF($L281="","",$C281*$L281)</x:f>
       </x:c>
       <x:c r="N281" s="86" t="str">
-        <x:f>IF($M281="","",$C281+$M281)</x:f>
+        <x:f>IF($M281="","",ROUNDDOWN($C281+$M281,2))</x:f>
       </x:c>
       <x:c r="O281" s="74" t="str">
-        <x:f>IF($N281="","",ROUNDDOWN($N281*$E281,3))</x:f>
+        <x:f>IF($N281="","",ROUNDDOWN(ROUNDDOWN($N281,2)*$E281,3))</x:f>
       </x:c>
       <x:c r="P281" s="77" t="str">
         <x:f>IF($L281="","",$I281*$L281)</x:f>
@@ -15707,10 +15707,10 @@
         <x:f>IF($L282="","",$C282*$L282)</x:f>
       </x:c>
       <x:c r="N282" s="86" t="str">
-        <x:f>IF($M282="","",$C282+$M282)</x:f>
+        <x:f>IF($M282="","",ROUNDDOWN($C282+$M282,2))</x:f>
       </x:c>
       <x:c r="O282" s="74" t="str">
-        <x:f>IF($N282="","",ROUNDDOWN($N282*$E282,3))</x:f>
+        <x:f>IF($N282="","",ROUNDDOWN(ROUNDDOWN($N282,2)*$E282,3))</x:f>
       </x:c>
       <x:c r="P282" s="77" t="str">
         <x:f>IF($L282="","",$I282*$L282)</x:f>
@@ -15760,10 +15760,10 @@
         <x:f>IF($L283="","",$C283*$L283)</x:f>
       </x:c>
       <x:c r="N283" s="86" t="str">
-        <x:f>IF($M283="","",$C283+$M283)</x:f>
+        <x:f>IF($M283="","",ROUNDDOWN($C283+$M283,2))</x:f>
       </x:c>
       <x:c r="O283" s="74" t="str">
-        <x:f>IF($N283="","",ROUNDDOWN($N283*$E283,3))</x:f>
+        <x:f>IF($N283="","",ROUNDDOWN(ROUNDDOWN($N283,2)*$E283,3))</x:f>
       </x:c>
       <x:c r="P283" s="77" t="str">
         <x:f>IF($L283="","",$I283*$L283)</x:f>
@@ -15813,10 +15813,10 @@
         <x:f>IF($L284="","",$C284*$L284)</x:f>
       </x:c>
       <x:c r="N284" s="86" t="str">
-        <x:f>IF($M284="","",$C284+$M284)</x:f>
+        <x:f>IF($M284="","",ROUNDDOWN($C284+$M284,2))</x:f>
       </x:c>
       <x:c r="O284" s="74" t="str">
-        <x:f>IF($N284="","",ROUNDDOWN($N284*$E284,3))</x:f>
+        <x:f>IF($N284="","",ROUNDDOWN(ROUNDDOWN($N284,2)*$E284,3))</x:f>
       </x:c>
       <x:c r="P284" s="77" t="str">
         <x:f>IF($L284="","",$I284*$L284)</x:f>
@@ -15866,10 +15866,10 @@
         <x:f>IF($L285="","",$C285*$L285)</x:f>
       </x:c>
       <x:c r="N285" s="86" t="str">
-        <x:f>IF($M285="","",$C285+$M285)</x:f>
+        <x:f>IF($M285="","",ROUNDDOWN($C285+$M285,2))</x:f>
       </x:c>
       <x:c r="O285" s="74" t="str">
-        <x:f>IF($N285="","",ROUNDDOWN($N285*$E285,3))</x:f>
+        <x:f>IF($N285="","",ROUNDDOWN(ROUNDDOWN($N285,2)*$E285,3))</x:f>
       </x:c>
       <x:c r="P285" s="77" t="str">
         <x:f>IF($L285="","",$I285*$L285)</x:f>
@@ -15919,10 +15919,10 @@
         <x:f>IF($L286="","",$C286*$L286)</x:f>
       </x:c>
       <x:c r="N286" s="86" t="str">
-        <x:f>IF($M286="","",$C286+$M286)</x:f>
+        <x:f>IF($M286="","",ROUNDDOWN($C286+$M286,2))</x:f>
       </x:c>
       <x:c r="O286" s="74" t="str">
-        <x:f>IF($N286="","",ROUNDDOWN($N286*$E286,3))</x:f>
+        <x:f>IF($N286="","",ROUNDDOWN(ROUNDDOWN($N286,2)*$E286,3))</x:f>
       </x:c>
       <x:c r="P286" s="77" t="str">
         <x:f>IF($L286="","",$I286*$L286)</x:f>
@@ -15972,10 +15972,10 @@
         <x:f>IF($L287="","",$C287*$L287)</x:f>
       </x:c>
       <x:c r="N287" s="86" t="str">
-        <x:f>IF($M287="","",$C287+$M287)</x:f>
+        <x:f>IF($M287="","",ROUNDDOWN($C287+$M287,2))</x:f>
       </x:c>
       <x:c r="O287" s="74" t="str">
-        <x:f>IF($N287="","",ROUNDDOWN($N287*$E287,3))</x:f>
+        <x:f>IF($N287="","",ROUNDDOWN(ROUNDDOWN($N287,2)*$E287,3))</x:f>
       </x:c>
       <x:c r="P287" s="77" t="str">
         <x:f>IF($L287="","",$I287*$L287)</x:f>
@@ -16025,10 +16025,10 @@
         <x:f>IF($L288="","",$C288*$L288)</x:f>
       </x:c>
       <x:c r="N288" s="86" t="str">
-        <x:f>IF($M288="","",$C288+$M288)</x:f>
+        <x:f>IF($M288="","",ROUNDDOWN($C288+$M288,2))</x:f>
       </x:c>
       <x:c r="O288" s="74" t="str">
-        <x:f>IF($N288="","",ROUNDDOWN($N288*$E288,3))</x:f>
+        <x:f>IF($N288="","",ROUNDDOWN(ROUNDDOWN($N288,2)*$E288,3))</x:f>
       </x:c>
       <x:c r="P288" s="77" t="str">
         <x:f>IF($L288="","",$I288*$L288)</x:f>
@@ -16078,10 +16078,10 @@
         <x:f>IF($L289="","",$C289*$L289)</x:f>
       </x:c>
       <x:c r="N289" s="86" t="str">
-        <x:f>IF($M289="","",$C289+$M289)</x:f>
+        <x:f>IF($M289="","",ROUNDDOWN($C289+$M289,2))</x:f>
       </x:c>
       <x:c r="O289" s="74" t="str">
-        <x:f>IF($N289="","",ROUNDDOWN($N289*$E289,3))</x:f>
+        <x:f>IF($N289="","",ROUNDDOWN(ROUNDDOWN($N289,2)*$E289,3))</x:f>
       </x:c>
       <x:c r="P289" s="77" t="str">
         <x:f>IF($L289="","",$I289*$L289)</x:f>
@@ -16131,10 +16131,10 @@
         <x:f>IF($L290="","",$C290*$L290)</x:f>
       </x:c>
       <x:c r="N290" s="86" t="str">
-        <x:f>IF($M290="","",$C290+$M290)</x:f>
+        <x:f>IF($M290="","",ROUNDDOWN($C290+$M290,2))</x:f>
       </x:c>
       <x:c r="O290" s="74" t="str">
-        <x:f>IF($N290="","",ROUNDDOWN($N290*$E290,3))</x:f>
+        <x:f>IF($N290="","",ROUNDDOWN(ROUNDDOWN($N290,2)*$E290,3))</x:f>
       </x:c>
       <x:c r="P290" s="77" t="str">
         <x:f>IF($L290="","",$I290*$L290)</x:f>
@@ -16184,10 +16184,10 @@
         <x:f>IF($L291="","",$C291*$L291)</x:f>
       </x:c>
       <x:c r="N291" s="86" t="str">
-        <x:f>IF($M291="","",$C291+$M291)</x:f>
+        <x:f>IF($M291="","",ROUNDDOWN($C291+$M291,2))</x:f>
       </x:c>
       <x:c r="O291" s="74" t="str">
-        <x:f>IF($N291="","",ROUNDDOWN($N291*$E291,3))</x:f>
+        <x:f>IF($N291="","",ROUNDDOWN(ROUNDDOWN($N291,2)*$E291,3))</x:f>
       </x:c>
       <x:c r="P291" s="77" t="str">
         <x:f>IF($L291="","",$I291*$L291)</x:f>
@@ -16237,10 +16237,10 @@
         <x:f>IF($L292="","",$C292*$L292)</x:f>
       </x:c>
       <x:c r="N292" s="86" t="str">
-        <x:f>IF($M292="","",$C292+$M292)</x:f>
+        <x:f>IF($M292="","",ROUNDDOWN($C292+$M292,2))</x:f>
       </x:c>
       <x:c r="O292" s="74" t="str">
-        <x:f>IF($N292="","",ROUNDDOWN($N292*$E292,3))</x:f>
+        <x:f>IF($N292="","",ROUNDDOWN(ROUNDDOWN($N292,2)*$E292,3))</x:f>
       </x:c>
       <x:c r="P292" s="77" t="str">
         <x:f>IF($L292="","",$I292*$L292)</x:f>
@@ -16290,10 +16290,10 @@
         <x:f>IF($L293="","",$C293*$L293)</x:f>
       </x:c>
       <x:c r="N293" s="86" t="str">
-        <x:f>IF($M293="","",$C293+$M293)</x:f>
+        <x:f>IF($M293="","",ROUNDDOWN($C293+$M293,2))</x:f>
       </x:c>
       <x:c r="O293" s="74" t="str">
-        <x:f>IF($N293="","",ROUNDDOWN($N293*$E293,3))</x:f>
+        <x:f>IF($N293="","",ROUNDDOWN(ROUNDDOWN($N293,2)*$E293,3))</x:f>
       </x:c>
       <x:c r="P293" s="77" t="str">
         <x:f>IF($L293="","",$I293*$L293)</x:f>
@@ -16343,10 +16343,10 @@
         <x:f>IF($L294="","",$C294*$L294)</x:f>
       </x:c>
       <x:c r="N294" s="86" t="str">
-        <x:f>IF($M294="","",$C294+$M294)</x:f>
+        <x:f>IF($M294="","",ROUNDDOWN($C294+$M294,2))</x:f>
       </x:c>
       <x:c r="O294" s="74" t="str">
-        <x:f>IF($N294="","",ROUNDDOWN($N294*$E294,3))</x:f>
+        <x:f>IF($N294="","",ROUNDDOWN(ROUNDDOWN($N294,2)*$E294,3))</x:f>
       </x:c>
       <x:c r="P294" s="77" t="str">
         <x:f>IF($L294="","",$I294*$L294)</x:f>
@@ -16396,10 +16396,10 @@
         <x:f>IF($L295="","",$C295*$L295)</x:f>
       </x:c>
       <x:c r="N295" s="86" t="str">
-        <x:f>IF($M295="","",$C295+$M295)</x:f>
+        <x:f>IF($M295="","",ROUNDDOWN($C295+$M295,2))</x:f>
       </x:c>
       <x:c r="O295" s="74" t="str">
-        <x:f>IF($N295="","",ROUNDDOWN($N295*$E295,3))</x:f>
+        <x:f>IF($N295="","",ROUNDDOWN(ROUNDDOWN($N295,2)*$E295,3))</x:f>
       </x:c>
       <x:c r="P295" s="77" t="str">
         <x:f>IF($L295="","",$I295*$L295)</x:f>
@@ -16449,10 +16449,10 @@
         <x:f>IF($L296="","",$C296*$L296)</x:f>
       </x:c>
       <x:c r="N296" s="86" t="str">
-        <x:f>IF($M296="","",$C296+$M296)</x:f>
+        <x:f>IF($M296="","",ROUNDDOWN($C296+$M296,2))</x:f>
       </x:c>
       <x:c r="O296" s="74" t="str">
-        <x:f>IF($N296="","",ROUNDDOWN($N296*$E296,3))</x:f>
+        <x:f>IF($N296="","",ROUNDDOWN(ROUNDDOWN($N296,2)*$E296,3))</x:f>
       </x:c>
       <x:c r="P296" s="77" t="str">
         <x:f>IF($L296="","",$I296*$L296)</x:f>
@@ -16502,10 +16502,10 @@
         <x:f>IF($L297="","",$C297*$L297)</x:f>
       </x:c>
       <x:c r="N297" s="86" t="str">
-        <x:f>IF($M297="","",$C297+$M297)</x:f>
+        <x:f>IF($M297="","",ROUNDDOWN($C297+$M297,2))</x:f>
       </x:c>
       <x:c r="O297" s="74" t="str">
-        <x:f>IF($N297="","",ROUNDDOWN($N297*$E297,3))</x:f>
+        <x:f>IF($N297="","",ROUNDDOWN(ROUNDDOWN($N297,2)*$E297,3))</x:f>
       </x:c>
       <x:c r="P297" s="77" t="str">
         <x:f>IF($L297="","",$I297*$L297)</x:f>
@@ -16555,10 +16555,10 @@
         <x:f>IF($L298="","",$C298*$L298)</x:f>
       </x:c>
       <x:c r="N298" s="86" t="str">
-        <x:f>IF($M298="","",$C298+$M298)</x:f>
+        <x:f>IF($M298="","",ROUNDDOWN($C298+$M298,2))</x:f>
       </x:c>
       <x:c r="O298" s="74" t="str">
-        <x:f>IF($N298="","",ROUNDDOWN($N298*$E298,3))</x:f>
+        <x:f>IF($N298="","",ROUNDDOWN(ROUNDDOWN($N298,2)*$E298,3))</x:f>
       </x:c>
       <x:c r="P298" s="77" t="str">
         <x:f>IF($L298="","",$I298*$L298)</x:f>
@@ -16608,10 +16608,10 @@
         <x:f>IF($L299="","",$C299*$L299)</x:f>
       </x:c>
       <x:c r="N299" s="86" t="str">
-        <x:f>IF($M299="","",$C299+$M299)</x:f>
+        <x:f>IF($M299="","",ROUNDDOWN($C299+$M299,2))</x:f>
       </x:c>
       <x:c r="O299" s="74" t="str">
-        <x:f>IF($N299="","",ROUNDDOWN($N299*$E299,3))</x:f>
+        <x:f>IF($N299="","",ROUNDDOWN(ROUNDDOWN($N299,2)*$E299,3))</x:f>
       </x:c>
       <x:c r="P299" s="77" t="str">
         <x:f>IF($L299="","",$I299*$L299)</x:f>
@@ -16661,10 +16661,10 @@
         <x:f>IF($L300="","",$C300*$L300)</x:f>
       </x:c>
       <x:c r="N300" s="86" t="str">
-        <x:f>IF($M300="","",$C300+$M300)</x:f>
+        <x:f>IF($M300="","",ROUNDDOWN($C300+$M300,2))</x:f>
       </x:c>
       <x:c r="O300" s="74" t="str">
-        <x:f>IF($N300="","",ROUNDDOWN($N300*$E300,3))</x:f>
+        <x:f>IF($N300="","",ROUNDDOWN(ROUNDDOWN($N300,2)*$E300,3))</x:f>
       </x:c>
       <x:c r="P300" s="77" t="str">
         <x:f>IF($L300="","",$I300*$L300)</x:f>
@@ -16714,10 +16714,10 @@
         <x:f>IF($L301="","",$C301*$L301)</x:f>
       </x:c>
       <x:c r="N301" s="86" t="str">
-        <x:f>IF($M301="","",$C301+$M301)</x:f>
+        <x:f>IF($M301="","",ROUNDDOWN($C301+$M301,2))</x:f>
       </x:c>
       <x:c r="O301" s="74" t="str">
-        <x:f>IF($N301="","",ROUNDDOWN($N301*$E301,3))</x:f>
+        <x:f>IF($N301="","",ROUNDDOWN(ROUNDDOWN($N301,2)*$E301,3))</x:f>
       </x:c>
       <x:c r="P301" s="77" t="str">
         <x:f>IF($L301="","",$I301*$L301)</x:f>
@@ -16767,10 +16767,10 @@
         <x:f>IF($L302="","",$C302*$L302)</x:f>
       </x:c>
       <x:c r="N302" s="86" t="str">
-        <x:f>IF($M302="","",$C302+$M302)</x:f>
+        <x:f>IF($M302="","",ROUNDDOWN($C302+$M302,2))</x:f>
       </x:c>
       <x:c r="O302" s="74" t="str">
-        <x:f>IF($N302="","",ROUNDDOWN($N302*$E302,3))</x:f>
+        <x:f>IF($N302="","",ROUNDDOWN(ROUNDDOWN($N302,2)*$E302,3))</x:f>
       </x:c>
       <x:c r="P302" s="77" t="str">
         <x:f>IF($L302="","",$I302*$L302)</x:f>
@@ -16820,10 +16820,10 @@
         <x:f>IF($L303="","",$C303*$L303)</x:f>
       </x:c>
       <x:c r="N303" s="86" t="str">
-        <x:f>IF($M303="","",$C303+$M303)</x:f>
+        <x:f>IF($M303="","",ROUNDDOWN($C303+$M303,2))</x:f>
       </x:c>
       <x:c r="O303" s="74" t="str">
-        <x:f>IF($N303="","",ROUNDDOWN($N303*$E303,3))</x:f>
+        <x:f>IF($N303="","",ROUNDDOWN(ROUNDDOWN($N303,2)*$E303,3))</x:f>
       </x:c>
       <x:c r="P303" s="77" t="str">
         <x:f>IF($L303="","",$I303*$L303)</x:f>
@@ -16873,10 +16873,10 @@
         <x:f>IF($L304="","",$C304*$L304)</x:f>
       </x:c>
       <x:c r="N304" s="86" t="str">
-        <x:f>IF($M304="","",$C304+$M304)</x:f>
+        <x:f>IF($M304="","",ROUNDDOWN($C304+$M304,2))</x:f>
       </x:c>
       <x:c r="O304" s="74" t="str">
-        <x:f>IF($N304="","",ROUNDDOWN($N304*$E304,3))</x:f>
+        <x:f>IF($N304="","",ROUNDDOWN(ROUNDDOWN($N304,2)*$E304,3))</x:f>
       </x:c>
       <x:c r="P304" s="77" t="str">
         <x:f>IF($L304="","",$I304*$L304)</x:f>
@@ -16926,10 +16926,10 @@
         <x:f>IF($L305="","",$C305*$L305)</x:f>
       </x:c>
       <x:c r="N305" s="86" t="str">
-        <x:f>IF($M305="","",$C305+$M305)</x:f>
+        <x:f>IF($M305="","",ROUNDDOWN($C305+$M305,2))</x:f>
       </x:c>
       <x:c r="O305" s="74" t="str">
-        <x:f>IF($N305="","",ROUNDDOWN($N305*$E305,3))</x:f>
+        <x:f>IF($N305="","",ROUNDDOWN(ROUNDDOWN($N305,2)*$E305,3))</x:f>
       </x:c>
       <x:c r="P305" s="77" t="str">
         <x:f>IF($L305="","",$I305*$L305)</x:f>
@@ -16979,10 +16979,10 @@
         <x:f>IF($L306="","",$C306*$L306)</x:f>
       </x:c>
       <x:c r="N306" s="86" t="str">
-        <x:f>IF($M306="","",$C306+$M306)</x:f>
+        <x:f>IF($M306="","",ROUNDDOWN($C306+$M306,2))</x:f>
       </x:c>
       <x:c r="O306" s="74" t="str">
-        <x:f>IF($N306="","",ROUNDDOWN($N306*$E306,3))</x:f>
+        <x:f>IF($N306="","",ROUNDDOWN(ROUNDDOWN($N306,2)*$E306,3))</x:f>
       </x:c>
       <x:c r="P306" s="77" t="str">
         <x:f>IF($L306="","",$I306*$L306)</x:f>
@@ -17032,10 +17032,10 @@
         <x:f>IF($L307="","",$C307*$L307)</x:f>
       </x:c>
       <x:c r="N307" s="86" t="str">
-        <x:f>IF($M307="","",$C307+$M307)</x:f>
+        <x:f>IF($M307="","",ROUNDDOWN($C307+$M307,2))</x:f>
       </x:c>
       <x:c r="O307" s="74" t="str">
-        <x:f>IF($N307="","",ROUNDDOWN($N307*$E307,3))</x:f>
+        <x:f>IF($N307="","",ROUNDDOWN(ROUNDDOWN($N307,2)*$E307,3))</x:f>
       </x:c>
       <x:c r="P307" s="77" t="str">
         <x:f>IF($L307="","",$I307*$L307)</x:f>
@@ -17085,10 +17085,10 @@
         <x:f>IF($L308="","",$C308*$L308)</x:f>
       </x:c>
       <x:c r="N308" s="86" t="str">
-        <x:f>IF($M308="","",$C308+$M308)</x:f>
+        <x:f>IF($M308="","",ROUNDDOWN($C308+$M308,2))</x:f>
       </x:c>
       <x:c r="O308" s="74" t="str">
-        <x:f>IF($N308="","",ROUNDDOWN($N308*$E308,3))</x:f>
+        <x:f>IF($N308="","",ROUNDDOWN(ROUNDDOWN($N308,2)*$E308,3))</x:f>
       </x:c>
       <x:c r="P308" s="77" t="str">
         <x:f>IF($L308="","",$I308*$L308)</x:f>
@@ -17138,10 +17138,10 @@
         <x:f>IF($L309="","",$C309*$L309)</x:f>
       </x:c>
       <x:c r="N309" s="86" t="str">
-        <x:f>IF($M309="","",$C309+$M309)</x:f>
+        <x:f>IF($M309="","",ROUNDDOWN($C309+$M309,2))</x:f>
       </x:c>
       <x:c r="O309" s="74" t="str">
-        <x:f>IF($N309="","",ROUNDDOWN($N309*$E309,3))</x:f>
+        <x:f>IF($N309="","",ROUNDDOWN(ROUNDDOWN($N309,2)*$E309,3))</x:f>
       </x:c>
       <x:c r="P309" s="77" t="str">
         <x:f>IF($L309="","",$I309*$L309)</x:f>
@@ -17191,10 +17191,10 @@
         <x:f>IF($L310="","",$C310*$L310)</x:f>
       </x:c>
       <x:c r="N310" s="86" t="str">
-        <x:f>IF($M310="","",$C310+$M310)</x:f>
+        <x:f>IF($M310="","",ROUNDDOWN($C310+$M310,2))</x:f>
       </x:c>
       <x:c r="O310" s="74" t="str">
-        <x:f>IF($N310="","",ROUNDDOWN($N310*$E310,3))</x:f>
+        <x:f>IF($N310="","",ROUNDDOWN(ROUNDDOWN($N310,2)*$E310,3))</x:f>
       </x:c>
       <x:c r="P310" s="77" t="str">
         <x:f>IF($L310="","",$I310*$L310)</x:f>
@@ -17244,10 +17244,10 @@
         <x:f>IF($L311="","",$C311*$L311)</x:f>
       </x:c>
       <x:c r="N311" s="86" t="str">
-        <x:f>IF($M311="","",$C311+$M311)</x:f>
+        <x:f>IF($M311="","",ROUNDDOWN($C311+$M311,2))</x:f>
       </x:c>
       <x:c r="O311" s="74" t="str">
-        <x:f>IF($N311="","",ROUNDDOWN($N311*$E311,3))</x:f>
+        <x:f>IF($N311="","",ROUNDDOWN(ROUNDDOWN($N311,2)*$E311,3))</x:f>
       </x:c>
       <x:c r="P311" s="77" t="str">
         <x:f>IF($L311="","",$I311*$L311)</x:f>
@@ -17297,10 +17297,10 @@
         <x:f>IF($L312="","",$C312*$L312)</x:f>
       </x:c>
       <x:c r="N312" s="86" t="str">
-        <x:f>IF($M312="","",$C312+$M312)</x:f>
+        <x:f>IF($M312="","",ROUNDDOWN($C312+$M312,2))</x:f>
       </x:c>
       <x:c r="O312" s="74" t="str">
-        <x:f>IF($N312="","",ROUNDDOWN($N312*$E312,3))</x:f>
+        <x:f>IF($N312="","",ROUNDDOWN(ROUNDDOWN($N312,2)*$E312,3))</x:f>
       </x:c>
       <x:c r="P312" s="77" t="str">
         <x:f>IF($L312="","",$I312*$L312)</x:f>
@@ -17350,10 +17350,10 @@
         <x:f>IF($L313="","",$C313*$L313)</x:f>
       </x:c>
       <x:c r="N313" s="86" t="str">
-        <x:f>IF($M313="","",$C313+$M313)</x:f>
+        <x:f>IF($M313="","",ROUNDDOWN($C313+$M313,2))</x:f>
       </x:c>
       <x:c r="O313" s="74" t="str">
-        <x:f>IF($N313="","",ROUNDDOWN($N313*$E313,3))</x:f>
+        <x:f>IF($N313="","",ROUNDDOWN(ROUNDDOWN($N313,2)*$E313,3))</x:f>
       </x:c>
       <x:c r="P313" s="77" t="str">
         <x:f>IF($L313="","",$I313*$L313)</x:f>
@@ -17403,10 +17403,10 @@
         <x:f>IF($L314="","",$C314*$L314)</x:f>
       </x:c>
       <x:c r="N314" s="86" t="str">
-        <x:f>IF($M314="","",$C314+$M314)</x:f>
+        <x:f>IF($M314="","",ROUNDDOWN($C314+$M314,2))</x:f>
       </x:c>
       <x:c r="O314" s="74" t="str">
-        <x:f>IF($N314="","",ROUNDDOWN($N314*$E314,3))</x:f>
+        <x:f>IF($N314="","",ROUNDDOWN(ROUNDDOWN($N314,2)*$E314,3))</x:f>
       </x:c>
       <x:c r="P314" s="77" t="str">
         <x:f>IF($L314="","",$I314*$L314)</x:f>
@@ -17456,10 +17456,10 @@
         <x:f>IF($L315="","",$C315*$L315)</x:f>
       </x:c>
       <x:c r="N315" s="86" t="str">
-        <x:f>IF($M315="","",$C315+$M315)</x:f>
+        <x:f>IF($M315="","",ROUNDDOWN($C315+$M315,2))</x:f>
       </x:c>
       <x:c r="O315" s="74" t="str">
-        <x:f>IF($N315="","",ROUNDDOWN($N315*$E315,3))</x:f>
+        <x:f>IF($N315="","",ROUNDDOWN(ROUNDDOWN($N315,2)*$E315,3))</x:f>
       </x:c>
       <x:c r="P315" s="77" t="str">
         <x:f>IF($L315="","",$I315*$L315)</x:f>
@@ -17509,10 +17509,10 @@
         <x:f>IF($L316="","",$C316*$L316)</x:f>
       </x:c>
       <x:c r="N316" s="86" t="str">
-        <x:f>IF($M316="","",$C316+$M316)</x:f>
+        <x:f>IF($M316="","",ROUNDDOWN($C316+$M316,2))</x:f>
       </x:c>
       <x:c r="O316" s="74" t="str">
-        <x:f>IF($N316="","",ROUNDDOWN($N316*$E316,3))</x:f>
+        <x:f>IF($N316="","",ROUNDDOWN(ROUNDDOWN($N316,2)*$E316,3))</x:f>
       </x:c>
       <x:c r="P316" s="77" t="str">
         <x:f>IF($L316="","",$I316*$L316)</x:f>
@@ -17562,10 +17562,10 @@
         <x:f>IF($L317="","",$C317*$L317)</x:f>
       </x:c>
       <x:c r="N317" s="86" t="str">
-        <x:f>IF($M317="","",$C317+$M317)</x:f>
+        <x:f>IF($M317="","",ROUNDDOWN($C317+$M317,2))</x:f>
       </x:c>
       <x:c r="O317" s="74" t="str">
-        <x:f>IF($N317="","",ROUNDDOWN($N317*$E317,3))</x:f>
+        <x:f>IF($N317="","",ROUNDDOWN(ROUNDDOWN($N317,2)*$E317,3))</x:f>
       </x:c>
       <x:c r="P317" s="77" t="str">
         <x:f>IF($L317="","",$I317*$L317)</x:f>
@@ -17615,10 +17615,10 @@
         <x:f>IF($L318="","",$C318*$L318)</x:f>
       </x:c>
       <x:c r="N318" s="86" t="str">
-        <x:f>IF($M318="","",$C318+$M318)</x:f>
+        <x:f>IF($M318="","",ROUNDDOWN($C318+$M318,2))</x:f>
       </x:c>
       <x:c r="O318" s="74" t="str">
-        <x:f>IF($N318="","",ROUNDDOWN($N318*$E318,3))</x:f>
+        <x:f>IF($N318="","",ROUNDDOWN(ROUNDDOWN($N318,2)*$E318,3))</x:f>
       </x:c>
       <x:c r="P318" s="77" t="str">
         <x:f>IF($L318="","",$I318*$L318)</x:f>
@@ -17668,10 +17668,10 @@
         <x:f>IF($L319="","",$C319*$L319)</x:f>
       </x:c>
       <x:c r="N319" s="86" t="str">
-        <x:f>IF($M319="","",$C319+$M319)</x:f>
+        <x:f>IF($M319="","",ROUNDDOWN($C319+$M319,2))</x:f>
       </x:c>
       <x:c r="O319" s="74" t="str">
-        <x:f>IF($N319="","",ROUNDDOWN($N319*$E319,3))</x:f>
+        <x:f>IF($N319="","",ROUNDDOWN(ROUNDDOWN($N319,2)*$E319,3))</x:f>
       </x:c>
       <x:c r="P319" s="77" t="str">
         <x:f>IF($L319="","",$I319*$L319)</x:f>
@@ -17721,10 +17721,10 @@
         <x:f>IF($L320="","",$C320*$L320)</x:f>
       </x:c>
       <x:c r="N320" s="86" t="str">
-        <x:f>IF($M320="","",$C320+$M320)</x:f>
+        <x:f>IF($M320="","",ROUNDDOWN($C320+$M320,2))</x:f>
       </x:c>
       <x:c r="O320" s="74" t="str">
-        <x:f>IF($N320="","",ROUNDDOWN($N320*$E320,3))</x:f>
+        <x:f>IF($N320="","",ROUNDDOWN(ROUNDDOWN($N320,2)*$E320,3))</x:f>
       </x:c>
       <x:c r="P320" s="77" t="str">
         <x:f>IF($L320="","",$I320*$L320)</x:f>
@@ -17774,10 +17774,10 @@
         <x:f>IF($L321="","",$C321*$L321)</x:f>
       </x:c>
       <x:c r="N321" s="86" t="str">
-        <x:f>IF($M321="","",$C321+$M321)</x:f>
+        <x:f>IF($M321="","",ROUNDDOWN($C321+$M321,2))</x:f>
       </x:c>
       <x:c r="O321" s="74" t="str">
-        <x:f>IF($N321="","",ROUNDDOWN($N321*$E321,3))</x:f>
+        <x:f>IF($N321="","",ROUNDDOWN(ROUNDDOWN($N321,2)*$E321,3))</x:f>
       </x:c>
       <x:c r="P321" s="77" t="str">
         <x:f>IF($L321="","",$I321*$L321)</x:f>
@@ -17827,10 +17827,10 @@
         <x:f>IF($L322="","",$C322*$L322)</x:f>
       </x:c>
       <x:c r="N322" s="86" t="str">
-        <x:f>IF($M322="","",$C322+$M322)</x:f>
+        <x:f>IF($M322="","",ROUNDDOWN($C322+$M322,2))</x:f>
       </x:c>
       <x:c r="O322" s="74" t="str">
-        <x:f>IF($N322="","",ROUNDDOWN($N322*$E322,3))</x:f>
+        <x:f>IF($N322="","",ROUNDDOWN(ROUNDDOWN($N322,2)*$E322,3))</x:f>
       </x:c>
       <x:c r="P322" s="77" t="str">
         <x:f>IF($L322="","",$I322*$L322)</x:f>
@@ -17880,10 +17880,10 @@
         <x:f>IF($L323="","",$C323*$L323)</x:f>
       </x:c>
       <x:c r="N323" s="86" t="str">
-        <x:f>IF($M323="","",$C323+$M323)</x:f>
+        <x:f>IF($M323="","",ROUNDDOWN($C323+$M323,2))</x:f>
       </x:c>
       <x:c r="O323" s="74" t="str">
-        <x:f>IF($N323="","",ROUNDDOWN($N323*$E323,3))</x:f>
+        <x:f>IF($N323="","",ROUNDDOWN(ROUNDDOWN($N323,2)*$E323,3))</x:f>
       </x:c>
       <x:c r="P323" s="77" t="str">
         <x:f>IF($L323="","",$I323*$L323)</x:f>
@@ -17933,10 +17933,10 @@
         <x:f>IF($L324="","",$C324*$L324)</x:f>
       </x:c>
       <x:c r="N324" s="86" t="str">
-        <x:f>IF($M324="","",$C324+$M324)</x:f>
+        <x:f>IF($M324="","",ROUNDDOWN($C324+$M324,2))</x:f>
       </x:c>
       <x:c r="O324" s="74" t="str">
-        <x:f>IF($N324="","",ROUNDDOWN($N324*$E324,3))</x:f>
+        <x:f>IF($N324="","",ROUNDDOWN(ROUNDDOWN($N324,2)*$E324,3))</x:f>
       </x:c>
       <x:c r="P324" s="77" t="str">
         <x:f>IF($L324="","",$I324*$L324)</x:f>
@@ -17986,10 +17986,10 @@
         <x:f>IF($L325="","",$C325*$L325)</x:f>
       </x:c>
       <x:c r="N325" s="86" t="str">
-        <x:f>IF($M325="","",$C325+$M325)</x:f>
+        <x:f>IF($M325="","",ROUNDDOWN($C325+$M325,2))</x:f>
       </x:c>
       <x:c r="O325" s="74" t="str">
-        <x:f>IF($N325="","",ROUNDDOWN($N325*$E325,3))</x:f>
+        <x:f>IF($N325="","",ROUNDDOWN(ROUNDDOWN($N325,2)*$E325,3))</x:f>
       </x:c>
       <x:c r="P325" s="77" t="str">
         <x:f>IF($L325="","",$I325*$L325)</x:f>
@@ -18039,10 +18039,10 @@
         <x:f>IF($L326="","",$C326*$L326)</x:f>
       </x:c>
       <x:c r="N326" s="86" t="str">
-        <x:f>IF($M326="","",$C326+$M326)</x:f>
+        <x:f>IF($M326="","",ROUNDDOWN($C326+$M326,2))</x:f>
       </x:c>
       <x:c r="O326" s="74" t="str">
-        <x:f>IF($N326="","",ROUNDDOWN($N326*$E326,3))</x:f>
+        <x:f>IF($N326="","",ROUNDDOWN(ROUNDDOWN($N326,2)*$E326,3))</x:f>
       </x:c>
       <x:c r="P326" s="77" t="str">
         <x:f>IF($L326="","",$I326*$L326)</x:f>
@@ -18092,10 +18092,10 @@
         <x:f>IF($L327="","",$C327*$L327)</x:f>
       </x:c>
       <x:c r="N327" s="86" t="str">
-        <x:f>IF($M327="","",$C327+$M327)</x:f>
+        <x:f>IF($M327="","",ROUNDDOWN($C327+$M327,2))</x:f>
       </x:c>
       <x:c r="O327" s="74" t="str">
-        <x:f>IF($N327="","",ROUNDDOWN($N327*$E327,3))</x:f>
+        <x:f>IF($N327="","",ROUNDDOWN(ROUNDDOWN($N327,2)*$E327,3))</x:f>
       </x:c>
       <x:c r="P327" s="77" t="str">
         <x:f>IF($L327="","",$I327*$L327)</x:f>
@@ -18145,10 +18145,10 @@
         <x:f>IF($L328="","",$C328*$L328)</x:f>
       </x:c>
       <x:c r="N328" s="86" t="str">
-        <x:f>IF($M328="","",$C328+$M328)</x:f>
+        <x:f>IF($M328="","",ROUNDDOWN($C328+$M328,2))</x:f>
       </x:c>
       <x:c r="O328" s="74" t="str">
-        <x:f>IF($N328="","",ROUNDDOWN($N328*$E328,3))</x:f>
+        <x:f>IF($N328="","",ROUNDDOWN(ROUNDDOWN($N328,2)*$E328,3))</x:f>
       </x:c>
       <x:c r="P328" s="77" t="str">
         <x:f>IF($L328="","",$I328*$L328)</x:f>
@@ -18198,10 +18198,10 @@
         <x:f>IF($L329="","",$C329*$L329)</x:f>
       </x:c>
       <x:c r="N329" s="86" t="str">
-        <x:f>IF($M329="","",$C329+$M329)</x:f>
+        <x:f>IF($M329="","",ROUNDDOWN($C329+$M329,2))</x:f>
       </x:c>
       <x:c r="O329" s="74" t="str">
-        <x:f>IF($N329="","",ROUNDDOWN($N329*$E329,3))</x:f>
+        <x:f>IF($N329="","",ROUNDDOWN(ROUNDDOWN($N329,2)*$E329,3))</x:f>
       </x:c>
       <x:c r="P329" s="77" t="str">
         <x:f>IF($L329="","",$I329*$L329)</x:f>
@@ -18251,10 +18251,10 @@
         <x:f>IF($L330="","",$C330*$L330)</x:f>
       </x:c>
       <x:c r="N330" s="86" t="str">
-        <x:f>IF($M330="","",$C330+$M330)</x:f>
+        <x:f>IF($M330="","",ROUNDDOWN($C330+$M330,2))</x:f>
       </x:c>
       <x:c r="O330" s="74" t="str">
-        <x:f>IF($N330="","",ROUNDDOWN($N330*$E330,3))</x:f>
+        <x:f>IF($N330="","",ROUNDDOWN(ROUNDDOWN($N330,2)*$E330,3))</x:f>
       </x:c>
       <x:c r="P330" s="77" t="str">
         <x:f>IF($L330="","",$I330*$L330)</x:f>
@@ -18304,10 +18304,10 @@
         <x:f>IF($L331="","",$C331*$L331)</x:f>
       </x:c>
       <x:c r="N331" s="86" t="str">
-        <x:f>IF($M331="","",$C331+$M331)</x:f>
+        <x:f>IF($M331="","",ROUNDDOWN($C331+$M331,2))</x:f>
       </x:c>
       <x:c r="O331" s="74" t="str">
-        <x:f>IF($N331="","",ROUNDDOWN($N331*$E331,3))</x:f>
+        <x:f>IF($N331="","",ROUNDDOWN(ROUNDDOWN($N331,2)*$E331,3))</x:f>
       </x:c>
       <x:c r="P331" s="77" t="str">
         <x:f>IF($L331="","",$I331*$L331)</x:f>
@@ -18357,10 +18357,10 @@
         <x:f>IF($L332="","",$C332*$L332)</x:f>
       </x:c>
       <x:c r="N332" s="86" t="str">
-        <x:f>IF($M332="","",$C332+$M332)</x:f>
+        <x:f>IF($M332="","",ROUNDDOWN($C332+$M332,2))</x:f>
       </x:c>
       <x:c r="O332" s="74" t="str">
-        <x:f>IF($N332="","",ROUNDDOWN($N332*$E332,3))</x:f>
+        <x:f>IF($N332="","",ROUNDDOWN(ROUNDDOWN($N332,2)*$E332,3))</x:f>
       </x:c>
       <x:c r="P332" s="77" t="str">
         <x:f>IF($L332="","",$I332*$L332)</x:f>
@@ -18410,10 +18410,10 @@
         <x:f>IF($L333="","",$C333*$L333)</x:f>
       </x:c>
       <x:c r="N333" s="86" t="str">
-        <x:f>IF($M333="","",$C333+$M333)</x:f>
+        <x:f>IF($M333="","",ROUNDDOWN($C333+$M333,2))</x:f>
       </x:c>
       <x:c r="O333" s="74" t="str">
-        <x:f>IF($N333="","",ROUNDDOWN($N333*$E333,3))</x:f>
+        <x:f>IF($N333="","",ROUNDDOWN(ROUNDDOWN($N333,2)*$E333,3))</x:f>
       </x:c>
       <x:c r="P333" s="77" t="str">
         <x:f>IF($L333="","",$I333*$L333)</x:f>
@@ -18463,10 +18463,10 @@
         <x:f>IF($L334="","",$C334*$L334)</x:f>
       </x:c>
       <x:c r="N334" s="86" t="str">
-        <x:f>IF($M334="","",$C334+$M334)</x:f>
+        <x:f>IF($M334="","",ROUNDDOWN($C334+$M334,2))</x:f>
       </x:c>
       <x:c r="O334" s="74" t="str">
-        <x:f>IF($N334="","",ROUNDDOWN($N334*$E334,3))</x:f>
+        <x:f>IF($N334="","",ROUNDDOWN(ROUNDDOWN($N334,2)*$E334,3))</x:f>
       </x:c>
       <x:c r="P334" s="77" t="str">
         <x:f>IF($L334="","",$I334*$L334)</x:f>
@@ -18516,10 +18516,10 @@
         <x:f>IF($L335="","",$C335*$L335)</x:f>
       </x:c>
       <x:c r="N335" s="86" t="str">
-        <x:f>IF($M335="","",$C335+$M335)</x:f>
+        <x:f>IF($M335="","",ROUNDDOWN($C335+$M335,2))</x:f>
       </x:c>
       <x:c r="O335" s="74" t="str">
-        <x:f>IF($N335="","",ROUNDDOWN($N335*$E335,3))</x:f>
+        <x:f>IF($N335="","",ROUNDDOWN(ROUNDDOWN($N335,2)*$E335,3))</x:f>
       </x:c>
       <x:c r="P335" s="77" t="str">
         <x:f>IF($L335="","",$I335*$L335)</x:f>
@@ -18569,10 +18569,10 @@
         <x:f>IF($L336="","",$C336*$L336)</x:f>
       </x:c>
       <x:c r="N336" s="86" t="str">
-        <x:f>IF($M336="","",$C336+$M336)</x:f>
+        <x:f>IF($M336="","",ROUNDDOWN($C336+$M336,2))</x:f>
       </x:c>
       <x:c r="O336" s="74" t="str">
-        <x:f>IF($N336="","",ROUNDDOWN($N336*$E336,3))</x:f>
+        <x:f>IF($N336="","",ROUNDDOWN(ROUNDDOWN($N336,2)*$E336,3))</x:f>
       </x:c>
       <x:c r="P336" s="77" t="str">
         <x:f>IF($L336="","",$I336*$L336)</x:f>
@@ -18622,10 +18622,10 @@
         <x:f>IF($L337="","",$C337*$L337)</x:f>
       </x:c>
       <x:c r="N337" s="86" t="str">
-        <x:f>IF($M337="","",$C337+$M337)</x:f>
+        <x:f>IF($M337="","",ROUNDDOWN($C337+$M337,2))</x:f>
       </x:c>
       <x:c r="O337" s="74" t="str">
-        <x:f>IF($N337="","",ROUNDDOWN($N337*$E337,3))</x:f>
+        <x:f>IF($N337="","",ROUNDDOWN(ROUNDDOWN($N337,2)*$E337,3))</x:f>
       </x:c>
       <x:c r="P337" s="77" t="str">
         <x:f>IF($L337="","",$I337*$L337)</x:f>
@@ -18675,10 +18675,10 @@
         <x:f>IF($L338="","",$C338*$L338)</x:f>
       </x:c>
       <x:c r="N338" s="86" t="str">
-        <x:f>IF($M338="","",$C338+$M338)</x:f>
+        <x:f>IF($M338="","",ROUNDDOWN($C338+$M338,2))</x:f>
       </x:c>
       <x:c r="O338" s="74" t="str">
-        <x:f>IF($N338="","",ROUNDDOWN($N338*$E338,3))</x:f>
+        <x:f>IF($N338="","",ROUNDDOWN(ROUNDDOWN($N338,2)*$E338,3))</x:f>
       </x:c>
       <x:c r="P338" s="77" t="str">
         <x:f>IF($L338="","",$I338*$L338)</x:f>
@@ -18728,10 +18728,10 @@
         <x:f>IF($L339="","",$C339*$L339)</x:f>
       </x:c>
       <x:c r="N339" s="86" t="str">
-        <x:f>IF($M339="","",$C339+$M339)</x:f>
+        <x:f>IF($M339="","",ROUNDDOWN($C339+$M339,2))</x:f>
       </x:c>
       <x:c r="O339" s="74" t="str">
-        <x:f>IF($N339="","",ROUNDDOWN($N339*$E339,3))</x:f>
+        <x:f>IF($N339="","",ROUNDDOWN(ROUNDDOWN($N339,2)*$E339,3))</x:f>
       </x:c>
       <x:c r="P339" s="77" t="str">
         <x:f>IF($L339="","",$I339*$L339)</x:f>
@@ -18781,10 +18781,10 @@
         <x:f>IF($L340="","",$C340*$L340)</x:f>
       </x:c>
       <x:c r="N340" s="86" t="str">
-        <x:f>IF($M340="","",$C340+$M340)</x:f>
+        <x:f>IF($M340="","",ROUNDDOWN($C340+$M340,2))</x:f>
       </x:c>
       <x:c r="O340" s="74" t="str">
-        <x:f>IF($N340="","",ROUNDDOWN($N340*$E340,3))</x:f>
+        <x:f>IF($N340="","",ROUNDDOWN(ROUNDDOWN($N340,2)*$E340,3))</x:f>
       </x:c>
       <x:c r="P340" s="77" t="str">
         <x:f>IF($L340="","",$I340*$L340)</x:f>
@@ -18834,10 +18834,10 @@
         <x:f>IF($L341="","",$C341*$L341)</x:f>
       </x:c>
       <x:c r="N341" s="86" t="str">
-        <x:f>IF($M341="","",$C341+$M341)</x:f>
+        <x:f>IF($M341="","",ROUNDDOWN($C341+$M341,2))</x:f>
       </x:c>
       <x:c r="O341" s="74" t="str">
-        <x:f>IF($N341="","",ROUNDDOWN($N341*$E341,3))</x:f>
+        <x:f>IF($N341="","",ROUNDDOWN(ROUNDDOWN($N341,2)*$E341,3))</x:f>
       </x:c>
       <x:c r="P341" s="77" t="str">
         <x:f>IF($L341="","",$I341*$L341)</x:f>
@@ -18887,10 +18887,10 @@
         <x:f>IF($L342="","",$C342*$L342)</x:f>
       </x:c>
       <x:c r="N342" s="86" t="str">
-        <x:f>IF($M342="","",$C342+$M342)</x:f>
+        <x:f>IF($M342="","",ROUNDDOWN($C342+$M342,2))</x:f>
       </x:c>
       <x:c r="O342" s="74" t="str">
-        <x:f>IF($N342="","",ROUNDDOWN($N342*$E342,3))</x:f>
+        <x:f>IF($N342="","",ROUNDDOWN(ROUNDDOWN($N342,2)*$E342,3))</x:f>
       </x:c>
       <x:c r="P342" s="77" t="str">
         <x:f>IF($L342="","",$I342*$L342)</x:f>
@@ -18940,10 +18940,10 @@
         <x:f>IF($L343="","",$C343*$L343)</x:f>
       </x:c>
       <x:c r="N343" s="86" t="str">
-        <x:f>IF($M343="","",$C343+$M343)</x:f>
+        <x:f>IF($M343="","",ROUNDDOWN($C343+$M343,2))</x:f>
       </x:c>
       <x:c r="O343" s="74" t="str">
-        <x:f>IF($N343="","",ROUNDDOWN($N343*$E343,3))</x:f>
+        <x:f>IF($N343="","",ROUNDDOWN(ROUNDDOWN($N343,2)*$E343,3))</x:f>
       </x:c>
       <x:c r="P343" s="77" t="str">
         <x:f>IF($L343="","",$I343*$L343)</x:f>
@@ -18993,10 +18993,10 @@
         <x:f>IF($L344="","",$C344*$L344)</x:f>
       </x:c>
       <x:c r="N344" s="86" t="str">
-        <x:f>IF($M344="","",$C344+$M344)</x:f>
+        <x:f>IF($M344="","",ROUNDDOWN($C344+$M344,2))</x:f>
       </x:c>
       <x:c r="O344" s="74" t="str">
-        <x:f>IF($N344="","",ROUNDDOWN($N344*$E344,3))</x:f>
+        <x:f>IF($N344="","",ROUNDDOWN(ROUNDDOWN($N344,2)*$E344,3))</x:f>
       </x:c>
       <x:c r="P344" s="77" t="str">
         <x:f>IF($L344="","",$I344*$L344)</x:f>
@@ -19046,10 +19046,10 @@
         <x:f>IF($L345="","",$C345*$L345)</x:f>
       </x:c>
       <x:c r="N345" s="86" t="str">
-        <x:f>IF($M345="","",$C345+$M345)</x:f>
+        <x:f>IF($M345="","",ROUNDDOWN($C345+$M345,2))</x:f>
       </x:c>
       <x:c r="O345" s="74" t="str">
-        <x:f>IF($N345="","",ROUNDDOWN($N345*$E345,3))</x:f>
+        <x:f>IF($N345="","",ROUNDDOWN(ROUNDDOWN($N345,2)*$E345,3))</x:f>
       </x:c>
       <x:c r="P345" s="77" t="str">
         <x:f>IF($L345="","",$I345*$L345)</x:f>
@@ -19099,10 +19099,10 @@
         <x:f>IF($L346="","",$C346*$L346)</x:f>
       </x:c>
       <x:c r="N346" s="86" t="str">
-        <x:f>IF($M346="","",$C346+$M346)</x:f>
+        <x:f>IF($M346="","",ROUNDDOWN($C346+$M346,2))</x:f>
       </x:c>
       <x:c r="O346" s="74" t="str">
-        <x:f>IF($N346="","",ROUNDDOWN($N346*$E346,3))</x:f>
+        <x:f>IF($N346="","",ROUNDDOWN(ROUNDDOWN($N346,2)*$E346,3))</x:f>
       </x:c>
       <x:c r="P346" s="77" t="str">
         <x:f>IF($L346="","",$I346*$L346)</x:f>
@@ -19152,10 +19152,10 @@
         <x:f>IF($L347="","",$C347*$L347)</x:f>
       </x:c>
       <x:c r="N347" s="86" t="str">
-        <x:f>IF($M347="","",$C347+$M347)</x:f>
+        <x:f>IF($M347="","",ROUNDDOWN($C347+$M347,2))</x:f>
       </x:c>
       <x:c r="O347" s="74" t="str">
-        <x:f>IF($N347="","",ROUNDDOWN($N347*$E347,3))</x:f>
+        <x:f>IF($N347="","",ROUNDDOWN(ROUNDDOWN($N347,2)*$E347,3))</x:f>
       </x:c>
       <x:c r="P347" s="77" t="str">
         <x:f>IF($L347="","",$I347*$L347)</x:f>
@@ -19205,10 +19205,10 @@
         <x:f>IF($L348="","",$C348*$L348)</x:f>
       </x:c>
       <x:c r="N348" s="86" t="str">
-        <x:f>IF($M348="","",$C348+$M348)</x:f>
+        <x:f>IF($M348="","",ROUNDDOWN($C348+$M348,2))</x:f>
       </x:c>
       <x:c r="O348" s="74" t="str">
-        <x:f>IF($N348="","",ROUNDDOWN($N348*$E348,3))</x:f>
+        <x:f>IF($N348="","",ROUNDDOWN(ROUNDDOWN($N348,2)*$E348,3))</x:f>
       </x:c>
       <x:c r="P348" s="77" t="str">
         <x:f>IF($L348="","",$I348*$L348)</x:f>
@@ -19258,10 +19258,10 @@
         <x:f>IF($L349="","",$C349*$L349)</x:f>
       </x:c>
       <x:c r="N349" s="86" t="str">
-        <x:f>IF($M349="","",$C349+$M349)</x:f>
+        <x:f>IF($M349="","",ROUNDDOWN($C349+$M349,2))</x:f>
       </x:c>
       <x:c r="O349" s="74" t="str">
-        <x:f>IF($N349="","",ROUNDDOWN($N349*$E349,3))</x:f>
+        <x:f>IF($N349="","",ROUNDDOWN(ROUNDDOWN($N349,2)*$E349,3))</x:f>
       </x:c>
       <x:c r="P349" s="77" t="str">
         <x:f>IF($L349="","",$I349*$L349)</x:f>
@@ -19311,10 +19311,10 @@
         <x:f>IF($L350="","",$C350*$L350)</x:f>
       </x:c>
       <x:c r="N350" s="86" t="str">
-        <x:f>IF($M350="","",$C350+$M350)</x:f>
+        <x:f>IF($M350="","",ROUNDDOWN($C350+$M350,2))</x:f>
       </x:c>
       <x:c r="O350" s="74" t="str">
-        <x:f>IF($N350="","",ROUNDDOWN($N350*$E350,3))</x:f>
+        <x:f>IF($N350="","",ROUNDDOWN(ROUNDDOWN($N350,2)*$E350,3))</x:f>
       </x:c>
       <x:c r="P350" s="77" t="str">
         <x:f>IF($L350="","",$I350*$L350)</x:f>
@@ -19364,10 +19364,10 @@
         <x:f>IF($L351="","",$C351*$L351)</x:f>
       </x:c>
       <x:c r="N351" s="86" t="str">
-        <x:f>IF($M351="","",$C351+$M351)</x:f>
+        <x:f>IF($M351="","",ROUNDDOWN($C351+$M351,2))</x:f>
       </x:c>
       <x:c r="O351" s="74" t="str">
-        <x:f>IF($N351="","",ROUNDDOWN($N351*$E351,3))</x:f>
+        <x:f>IF($N351="","",ROUNDDOWN(ROUNDDOWN($N351,2)*$E351,3))</x:f>
       </x:c>
       <x:c r="P351" s="77" t="str">
         <x:f>IF($L351="","",$I351*$L351)</x:f>
@@ -19417,10 +19417,10 @@
         <x:f>IF($L352="","",$C352*$L352)</x:f>
       </x:c>
       <x:c r="N352" s="86" t="str">
-        <x:f>IF($M352="","",$C352+$M352)</x:f>
+        <x:f>IF($M352="","",ROUNDDOWN($C352+$M352,2))</x:f>
       </x:c>
       <x:c r="O352" s="74" t="str">
-        <x:f>IF($N352="","",ROUNDDOWN($N352*$E352,3))</x:f>
+        <x:f>IF($N352="","",ROUNDDOWN(ROUNDDOWN($N352,2)*$E352,3))</x:f>
       </x:c>
       <x:c r="P352" s="77" t="str">
         <x:f>IF($L352="","",$I352*$L352)</x:f>
@@ -19470,10 +19470,10 @@
         <x:f>IF($L353="","",$C353*$L353)</x:f>
       </x:c>
       <x:c r="N353" s="86" t="str">
-        <x:f>IF($M353="","",$C353+$M353)</x:f>
+        <x:f>IF($M353="","",ROUNDDOWN($C353+$M353,2))</x:f>
       </x:c>
       <x:c r="O353" s="74" t="str">
-        <x:f>IF($N353="","",ROUNDDOWN($N353*$E353,3))</x:f>
+        <x:f>IF($N353="","",ROUNDDOWN(ROUNDDOWN($N353,2)*$E353,3))</x:f>
       </x:c>
       <x:c r="P353" s="77" t="str">
         <x:f>IF($L353="","",$I353*$L353)</x:f>
@@ -19523,10 +19523,10 @@
         <x:f>IF($L354="","",$C354*$L354)</x:f>
       </x:c>
       <x:c r="N354" s="87" t="str">
-        <x:f>IF($M354="","",$C354+$M354)</x:f>
+        <x:f>IF($M354="","",ROUNDDOWN($C354+$M354,2))</x:f>
       </x:c>
       <x:c r="O354" s="75" t="str">
-        <x:f>IF($N354="","",ROUNDDOWN($N354*$E354,3))</x:f>
+        <x:f>IF($N354="","",ROUNDDOWN(ROUNDDOWN($N354,2)*$E354,3))</x:f>
       </x:c>
       <x:c r="P354" s="78" t="str">
         <x:f>IF($L354="","",$I354*$L354)</x:f>
@@ -19562,7 +19562,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdce4c67ffc194390"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7f3a85f6a7a424c"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>